<commit_message>
Update live MLB hitter fantasy scores 2026-07-12 08:54:25 AM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
@@ -657,7 +657,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -771,7 +771,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -885,7 +885,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -999,7 +999,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1227,7 +1227,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1341,7 +1341,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1455,7 +1455,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1569,7 +1569,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1683,7 +1683,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1797,7 +1797,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1911,7 +1911,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2025,7 +2025,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2139,7 +2139,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2253,7 +2253,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2367,7 +2367,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2481,7 +2481,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2709,7 +2709,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:21 AM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2823,7 +2823,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:21 AM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2937,7 +2937,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:21 AM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3051,7 +3051,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:21 AM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3165,7 +3165,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:21 AM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3279,7 +3279,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:21 AM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3393,7 +3393,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:21 AM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:21 AM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3621,7 +3621,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:21 AM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3735,7 +3735,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3849,7 +3849,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -3963,7 +3963,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4077,7 +4077,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4191,7 +4191,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4305,7 +4305,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4419,7 +4419,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4533,7 +4533,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4647,7 +4647,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4761,7 +4761,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4875,7 +4875,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -4989,7 +4989,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5103,7 +5103,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5217,7 +5217,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5331,7 +5331,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5445,7 +5445,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5559,7 +5559,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5673,7 +5673,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5787,7 +5787,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5901,7 +5901,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6015,7 +6015,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6129,7 +6129,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6243,7 +6243,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6357,7 +6357,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6471,7 +6471,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6585,7 +6585,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6699,7 +6699,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6813,7 +6813,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -6927,7 +6927,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7041,7 +7041,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7155,7 +7155,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7269,7 +7269,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7383,7 +7383,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7497,7 +7497,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7611,7 +7611,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7725,7 +7725,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7839,7 +7839,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -7953,7 +7953,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8067,7 +8067,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8181,7 +8181,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8295,7 +8295,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8409,7 +8409,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8523,7 +8523,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8637,7 +8637,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8751,7 +8751,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8865,7 +8865,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -8979,7 +8979,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9093,7 +9093,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9207,7 +9207,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9321,7 +9321,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9435,7 +9435,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9549,7 +9549,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9663,7 +9663,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9777,7 +9777,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -9891,7 +9891,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:21 AM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10005,7 +10005,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:21 AM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10119,7 +10119,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:21 AM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10233,7 +10233,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:21 AM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10347,7 +10347,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:21 AM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10461,7 +10461,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:21 AM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10575,7 +10575,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:21 AM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10689,7 +10689,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:21 AM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10803,7 +10803,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:21 AM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -10917,7 +10917,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11031,7 +11031,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11145,7 +11145,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11259,7 +11259,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11373,7 +11373,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11487,7 +11487,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11601,7 +11601,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11715,7 +11715,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11829,7 +11829,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -11943,7 +11943,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12057,7 +12057,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12171,7 +12171,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12285,7 +12285,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12399,7 +12399,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12513,7 +12513,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12627,7 +12627,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12741,7 +12741,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12855,7 +12855,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -12969,7 +12969,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:21 AM PT</t>
+          <t>2026-07-12 08:54:21 AM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13092,7 +13092,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:21 AM PT</t>
+          <t>2026-07-12 08:54:21 AM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13215,7 +13215,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:21 AM PT</t>
+          <t>2026-07-12 08:54:21 AM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13338,7 +13338,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:21 AM PT</t>
+          <t>2026-07-12 08:54:21 AM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13461,7 +13461,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:21 AM PT</t>
+          <t>2026-07-12 08:54:21 AM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13584,7 +13584,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:21 AM PT</t>
+          <t>2026-07-12 08:54:21 AM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13707,7 +13707,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:21 AM PT</t>
+          <t>2026-07-12 08:54:21 AM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13830,7 +13830,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:21 AM PT</t>
+          <t>2026-07-12 08:54:21 AM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -13953,7 +13953,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:21 AM PT</t>
+          <t>2026-07-12 08:54:21 AM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14076,7 +14076,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14190,7 +14190,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14304,7 +14304,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14418,7 +14418,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14532,7 +14532,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14646,7 +14646,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14760,7 +14760,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14874,7 +14874,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -14988,7 +14988,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15102,7 +15102,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15216,7 +15216,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15330,7 +15330,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15444,7 +15444,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15558,7 +15558,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15672,7 +15672,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15786,7 +15786,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -15900,7 +15900,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16014,7 +16014,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16128,7 +16128,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16242,7 +16242,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16356,7 +16356,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16470,7 +16470,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16584,7 +16584,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16698,7 +16698,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16812,7 +16812,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -16926,7 +16926,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17040,7 +17040,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17154,7 +17154,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17268,7 +17268,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17382,7 +17382,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17496,7 +17496,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17610,7 +17610,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17724,7 +17724,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17838,7 +17838,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -17952,7 +17952,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18066,7 +18066,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18180,7 +18180,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:21 AM PT</t>
+          <t>2026-07-12 08:54:21 AM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18303,7 +18303,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:21 AM PT</t>
+          <t>2026-07-12 08:54:21 AM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18426,7 +18426,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:21 AM PT</t>
+          <t>2026-07-12 08:54:21 AM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18549,7 +18549,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:21 AM PT</t>
+          <t>2026-07-12 08:54:21 AM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18672,7 +18672,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:21 AM PT</t>
+          <t>2026-07-12 08:54:21 AM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18795,7 +18795,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:21 AM PT</t>
+          <t>2026-07-12 08:54:21 AM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18918,7 +18918,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:21 AM PT</t>
+          <t>2026-07-12 08:54:21 AM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19041,7 +19041,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:21 AM PT</t>
+          <t>2026-07-12 08:54:21 AM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19164,7 +19164,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:21 AM PT</t>
+          <t>2026-07-12 08:54:21 AM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19287,7 +19287,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19401,7 +19401,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19515,7 +19515,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19629,7 +19629,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19743,7 +19743,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19857,7 +19857,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -19971,7 +19971,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -20085,7 +20085,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20199,7 +20199,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20313,7 +20313,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20427,7 +20427,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20541,7 +20541,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20655,7 +20655,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20769,7 +20769,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20883,7 +20883,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -20997,7 +20997,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21111,7 +21111,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21225,7 +21225,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21339,7 +21339,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21453,7 +21453,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21567,7 +21567,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21681,7 +21681,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21795,7 +21795,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21909,7 +21909,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -22023,7 +22023,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22137,7 +22137,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22251,7 +22251,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22365,7 +22365,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22471,7 +22471,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22577,7 +22577,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22683,7 +22683,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22789,7 +22789,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -22895,7 +22895,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -23001,7 +23001,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23107,7 +23107,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23213,7 +23213,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:23 AM PT</t>
+          <t>2026-07-12 08:54:23 AM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23319,7 +23319,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23433,7 +23433,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23547,7 +23547,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23661,7 +23661,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23775,7 +23775,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -23889,7 +23889,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -24003,7 +24003,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24117,7 +24117,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24231,7 +24231,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-12 08:52:22 AM PT</t>
+          <t>2026-07-12 08:54:22 AM PT</t>
         </is>
       </c>
       <c r="C208" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-12 08:56:24 AM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
@@ -657,7 +657,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -771,7 +771,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -885,7 +885,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -999,7 +999,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1227,7 +1227,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1341,7 +1341,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1455,7 +1455,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1569,7 +1569,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1683,7 +1683,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1797,7 +1797,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1911,7 +1911,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2025,7 +2025,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2139,7 +2139,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2253,7 +2253,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2367,7 +2367,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2481,7 +2481,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2709,7 +2709,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:21 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2823,7 +2823,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:21 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2937,7 +2937,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:21 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3051,7 +3051,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:21 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3165,7 +3165,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:21 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3279,7 +3279,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:21 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3393,7 +3393,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:21 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:21 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3621,7 +3621,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:21 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3735,7 +3735,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3849,7 +3849,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -3963,7 +3963,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4077,7 +4077,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4191,7 +4191,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4305,7 +4305,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4419,7 +4419,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4533,7 +4533,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4647,7 +4647,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4761,7 +4761,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4875,7 +4875,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -4989,7 +4989,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5103,7 +5103,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5217,7 +5217,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5331,7 +5331,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5445,7 +5445,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5559,7 +5559,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5673,7 +5673,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5787,7 +5787,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5901,7 +5901,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6015,7 +6015,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6129,7 +6129,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6243,7 +6243,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6357,7 +6357,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6471,7 +6471,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6585,7 +6585,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6699,7 +6699,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6813,7 +6813,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -6927,7 +6927,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7041,7 +7041,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7155,7 +7155,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7269,7 +7269,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7383,7 +7383,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7497,7 +7497,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7611,7 +7611,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7725,7 +7725,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7839,7 +7839,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -7953,7 +7953,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8067,7 +8067,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8181,7 +8181,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8295,7 +8295,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8409,7 +8409,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8523,7 +8523,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8637,7 +8637,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8751,7 +8751,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8865,7 +8865,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -8979,7 +8979,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9093,7 +9093,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9207,7 +9207,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9321,7 +9321,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9435,7 +9435,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9549,7 +9549,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9663,7 +9663,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9777,7 +9777,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -9891,7 +9891,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:21 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10005,7 +10005,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:21 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10119,7 +10119,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:21 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10233,7 +10233,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:21 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10347,7 +10347,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:21 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10461,7 +10461,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:21 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10575,7 +10575,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:21 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10689,7 +10689,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:21 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10803,7 +10803,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:21 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -10917,7 +10917,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11031,7 +11031,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11145,7 +11145,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11259,7 +11259,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11373,7 +11373,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11487,7 +11487,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11601,7 +11601,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11715,7 +11715,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11829,7 +11829,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -11943,7 +11943,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12057,7 +12057,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12171,7 +12171,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12285,7 +12285,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12399,7 +12399,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12513,7 +12513,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12627,7 +12627,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12741,7 +12741,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12855,7 +12855,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -12969,7 +12969,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:21 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13092,7 +13092,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:21 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13215,7 +13215,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:21 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13338,7 +13338,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:21 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13461,7 +13461,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:21 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13584,7 +13584,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:21 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13707,7 +13707,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:21 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13830,7 +13830,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:21 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -13953,7 +13953,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:21 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14076,7 +14076,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14190,7 +14190,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14304,7 +14304,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14418,7 +14418,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14532,7 +14532,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14646,7 +14646,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14760,7 +14760,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14874,7 +14874,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -14988,7 +14988,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15102,7 +15102,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15216,7 +15216,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15330,7 +15330,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15444,7 +15444,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15558,7 +15558,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15672,7 +15672,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15786,7 +15786,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -15900,7 +15900,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16014,7 +16014,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16128,7 +16128,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16242,7 +16242,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16356,7 +16356,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16470,7 +16470,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16584,7 +16584,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16698,7 +16698,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16812,7 +16812,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -16926,7 +16926,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17040,7 +17040,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17154,7 +17154,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17268,7 +17268,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17382,7 +17382,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17496,7 +17496,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17610,7 +17610,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17724,7 +17724,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17838,7 +17838,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -17952,7 +17952,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18066,7 +18066,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18180,7 +18180,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:21 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18303,7 +18303,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:21 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18426,7 +18426,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:21 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18549,7 +18549,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:21 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18672,7 +18672,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:21 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18795,7 +18795,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:21 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18918,7 +18918,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:21 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19041,7 +19041,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:21 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19164,7 +19164,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:21 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19287,7 +19287,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19401,7 +19401,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19515,7 +19515,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19629,7 +19629,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19743,7 +19743,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19857,7 +19857,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -19971,7 +19971,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -20085,7 +20085,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20199,7 +20199,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20313,7 +20313,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20427,7 +20427,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20541,7 +20541,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20655,7 +20655,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20769,7 +20769,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20883,7 +20883,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -20997,7 +20997,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21111,7 +21111,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21225,7 +21225,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21339,7 +21339,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21453,7 +21453,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21567,7 +21567,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21681,7 +21681,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21795,7 +21795,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21909,7 +21909,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -22023,7 +22023,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22137,7 +22137,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22251,7 +22251,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22365,7 +22365,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22471,7 +22471,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22577,7 +22577,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22683,7 +22683,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22789,7 +22789,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -22895,7 +22895,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -23001,7 +23001,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23107,7 +23107,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23213,7 +23213,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:23 AM PT</t>
+          <t>2026-07-12 08:56:22 AM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23319,7 +23319,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23433,7 +23433,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23547,7 +23547,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23661,7 +23661,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23775,7 +23775,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -23889,7 +23889,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -24003,7 +24003,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24117,7 +24117,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24231,7 +24231,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-12 08:54:22 AM PT</t>
+          <t>2026-07-12 08:56:21 AM PT</t>
         </is>
       </c>
       <c r="C208" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-12 08:58:23 AM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
@@ -657,7 +657,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -771,7 +771,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -885,7 +885,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -999,7 +999,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1227,7 +1227,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1341,7 +1341,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1455,7 +1455,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1569,7 +1569,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1683,7 +1683,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1797,7 +1797,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1911,7 +1911,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2025,7 +2025,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2139,7 +2139,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2253,7 +2253,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2367,7 +2367,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2481,7 +2481,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2709,7 +2709,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2823,7 +2823,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2937,7 +2937,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3051,7 +3051,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3165,7 +3165,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3279,7 +3279,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3393,7 +3393,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3621,7 +3621,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3735,7 +3735,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3849,7 +3849,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -3963,7 +3963,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4077,7 +4077,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4191,7 +4191,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4305,7 +4305,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4419,7 +4419,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4533,7 +4533,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4647,7 +4647,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4761,7 +4761,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4875,7 +4875,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -4989,7 +4989,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5103,7 +5103,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5217,7 +5217,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5331,7 +5331,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5445,7 +5445,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5559,7 +5559,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5673,7 +5673,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5787,7 +5787,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5901,7 +5901,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6015,7 +6015,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6129,7 +6129,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6243,7 +6243,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6357,7 +6357,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6471,7 +6471,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6585,7 +6585,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6699,7 +6699,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6813,7 +6813,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -6927,7 +6927,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7041,7 +7041,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7155,7 +7155,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7269,7 +7269,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7383,7 +7383,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7497,7 +7497,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7611,7 +7611,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7725,7 +7725,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7839,7 +7839,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -7953,7 +7953,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8067,7 +8067,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8181,7 +8181,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8295,7 +8295,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8409,7 +8409,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8523,7 +8523,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8637,7 +8637,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8751,7 +8751,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8865,7 +8865,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -8979,7 +8979,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9093,7 +9093,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9207,7 +9207,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9321,7 +9321,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9435,7 +9435,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9549,7 +9549,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9663,7 +9663,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9777,7 +9777,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -9891,7 +9891,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10005,7 +10005,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10119,7 +10119,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10233,7 +10233,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10347,7 +10347,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10461,7 +10461,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10575,7 +10575,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10689,7 +10689,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10803,7 +10803,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -10917,7 +10917,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11031,7 +11031,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11145,7 +11145,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11259,7 +11259,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11373,7 +11373,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11487,7 +11487,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11601,7 +11601,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11715,7 +11715,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11829,7 +11829,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -11943,7 +11943,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12057,7 +12057,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12171,7 +12171,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12285,7 +12285,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12399,7 +12399,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12513,7 +12513,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12627,7 +12627,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12741,7 +12741,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12855,7 +12855,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -12969,7 +12969,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13092,7 +13092,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13215,7 +13215,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13338,7 +13338,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13461,7 +13461,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13584,7 +13584,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13707,7 +13707,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13830,7 +13830,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -13953,7 +13953,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14076,7 +14076,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14190,7 +14190,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14304,7 +14304,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14418,7 +14418,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14532,7 +14532,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14646,7 +14646,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14760,7 +14760,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14874,7 +14874,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -14988,7 +14988,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15102,7 +15102,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15216,7 +15216,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15330,7 +15330,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15444,7 +15444,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15558,7 +15558,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15672,7 +15672,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15786,7 +15786,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -15900,7 +15900,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16014,7 +16014,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16128,7 +16128,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16242,7 +16242,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16356,7 +16356,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16470,7 +16470,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16584,7 +16584,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16698,7 +16698,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16812,7 +16812,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -16926,7 +16926,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17040,7 +17040,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17154,7 +17154,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17268,7 +17268,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17382,7 +17382,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17496,7 +17496,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17610,7 +17610,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17724,7 +17724,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17838,7 +17838,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -17952,7 +17952,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18066,7 +18066,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18180,7 +18180,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18303,7 +18303,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18426,7 +18426,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18549,7 +18549,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18672,7 +18672,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18795,7 +18795,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18918,7 +18918,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19041,7 +19041,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19164,7 +19164,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19287,7 +19287,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19401,7 +19401,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19515,7 +19515,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19629,7 +19629,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19743,7 +19743,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19857,7 +19857,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -19971,7 +19971,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -20085,7 +20085,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20199,7 +20199,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20313,7 +20313,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20427,7 +20427,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20541,7 +20541,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20655,7 +20655,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20769,7 +20769,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20883,7 +20883,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -20997,7 +20997,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21111,7 +21111,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21225,7 +21225,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21339,7 +21339,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21453,7 +21453,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21567,7 +21567,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21681,7 +21681,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21795,7 +21795,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21909,7 +21909,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -22023,7 +22023,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22137,7 +22137,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22251,7 +22251,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22365,7 +22365,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22471,7 +22471,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22577,7 +22577,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22683,7 +22683,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22789,7 +22789,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -22895,7 +22895,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -23001,7 +23001,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23107,7 +23107,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23213,7 +23213,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:22 AM PT</t>
+          <t>2026-07-12 08:58:22 AM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23319,7 +23319,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23433,7 +23433,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23547,7 +23547,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23661,7 +23661,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23775,7 +23775,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -23889,7 +23889,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -24003,7 +24003,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24117,7 +24117,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24231,7 +24231,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-12 08:56:21 AM PT</t>
+          <t>2026-07-12 08:58:21 AM PT</t>
         </is>
       </c>
       <c r="C208" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-12 09:00:23 AM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
@@ -657,7 +657,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -771,7 +771,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -885,7 +885,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -999,7 +999,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1227,7 +1227,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1341,7 +1341,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1455,7 +1455,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1569,7 +1569,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1683,7 +1683,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1797,7 +1797,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1911,7 +1911,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2025,7 +2025,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2139,7 +2139,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2253,7 +2253,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2367,7 +2367,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2481,7 +2481,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2709,7 +2709,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2823,7 +2823,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2937,7 +2937,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3051,7 +3051,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3165,7 +3165,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3279,7 +3279,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3393,7 +3393,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3621,7 +3621,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3735,7 +3735,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3849,7 +3849,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -3963,7 +3963,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4077,7 +4077,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4191,7 +4191,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4305,7 +4305,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4419,7 +4419,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4533,7 +4533,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4647,7 +4647,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4761,7 +4761,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4875,7 +4875,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -4989,7 +4989,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5103,7 +5103,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5217,7 +5217,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5331,7 +5331,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5445,7 +5445,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5559,7 +5559,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5673,7 +5673,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5787,7 +5787,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5901,7 +5901,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6015,7 +6015,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6129,7 +6129,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6243,7 +6243,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6357,7 +6357,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6471,7 +6471,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6585,7 +6585,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6699,7 +6699,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6813,7 +6813,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -6927,7 +6927,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7041,7 +7041,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7155,7 +7155,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7269,7 +7269,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7383,7 +7383,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7497,7 +7497,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7611,7 +7611,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7725,7 +7725,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7839,7 +7839,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -7953,7 +7953,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8067,7 +8067,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8181,7 +8181,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8295,7 +8295,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8409,7 +8409,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8523,7 +8523,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8637,7 +8637,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8751,7 +8751,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8865,7 +8865,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -8979,7 +8979,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9093,7 +9093,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9207,7 +9207,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9321,7 +9321,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9435,7 +9435,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9549,7 +9549,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9663,7 +9663,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9777,7 +9777,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -9891,7 +9891,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10005,7 +10005,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10119,7 +10119,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10233,7 +10233,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10347,7 +10347,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10461,7 +10461,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10575,7 +10575,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10689,7 +10689,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10803,7 +10803,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -10917,7 +10917,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11031,7 +11031,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11145,7 +11145,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11259,7 +11259,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11373,7 +11373,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11487,7 +11487,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11601,7 +11601,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11715,7 +11715,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11829,7 +11829,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -11943,7 +11943,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12057,7 +12057,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12171,7 +12171,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12285,7 +12285,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12399,7 +12399,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12513,7 +12513,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12627,7 +12627,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12741,7 +12741,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12855,7 +12855,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -12969,7 +12969,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13092,7 +13092,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13215,7 +13215,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13338,7 +13338,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13461,7 +13461,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13584,7 +13584,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13707,7 +13707,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13830,7 +13830,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -13953,7 +13953,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14076,7 +14076,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14190,7 +14190,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14304,7 +14304,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14418,7 +14418,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14532,7 +14532,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14646,7 +14646,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14760,7 +14760,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14874,7 +14874,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -14988,7 +14988,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15102,7 +15102,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15216,7 +15216,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15330,7 +15330,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15444,7 +15444,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15558,7 +15558,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15672,7 +15672,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15786,7 +15786,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -15900,7 +15900,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16014,7 +16014,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16128,7 +16128,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16242,7 +16242,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16356,7 +16356,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16470,7 +16470,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16584,7 +16584,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16698,7 +16698,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16812,7 +16812,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -16926,7 +16926,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17040,7 +17040,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17154,7 +17154,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17268,7 +17268,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17382,7 +17382,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17496,7 +17496,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17610,7 +17610,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17724,7 +17724,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17838,7 +17838,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -17952,7 +17952,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18066,7 +18066,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18180,7 +18180,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18303,7 +18303,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18426,7 +18426,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18549,7 +18549,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18672,7 +18672,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18795,7 +18795,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18918,7 +18918,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19041,7 +19041,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19164,7 +19164,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19287,7 +19287,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19401,7 +19401,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19515,7 +19515,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19629,7 +19629,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19743,7 +19743,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19857,7 +19857,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -19971,7 +19971,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -20085,7 +20085,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20199,7 +20199,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20313,7 +20313,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20427,7 +20427,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20541,7 +20541,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20655,7 +20655,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20769,7 +20769,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20883,7 +20883,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -20997,7 +20997,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21111,7 +21111,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21225,7 +21225,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21339,7 +21339,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21453,7 +21453,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21567,7 +21567,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21681,7 +21681,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21795,7 +21795,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21909,7 +21909,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -22023,7 +22023,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22137,7 +22137,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22251,7 +22251,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22365,7 +22365,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22471,7 +22471,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22577,7 +22577,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22683,7 +22683,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22789,7 +22789,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -22895,7 +22895,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -23001,7 +23001,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23107,7 +23107,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23213,7 +23213,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:22 AM PT</t>
+          <t>2026-07-12 09:00:22 AM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23319,7 +23319,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23433,7 +23433,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23547,7 +23547,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23661,7 +23661,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23775,7 +23775,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -23889,7 +23889,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -24003,7 +24003,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24117,7 +24117,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24231,7 +24231,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-12 08:58:21 AM PT</t>
+          <t>2026-07-12 09:00:21 AM PT</t>
         </is>
       </c>
       <c r="C208" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-12 09:02:23 AM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
@@ -657,7 +657,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -771,7 +771,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -885,7 +885,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -999,7 +999,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1227,7 +1227,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1341,7 +1341,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1455,7 +1455,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1569,7 +1569,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1683,7 +1683,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1797,7 +1797,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1911,7 +1911,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2025,7 +2025,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2139,7 +2139,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2253,7 +2253,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2367,7 +2367,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2481,7 +2481,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2709,7 +2709,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2823,7 +2823,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2937,7 +2937,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3051,7 +3051,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3165,7 +3165,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3279,7 +3279,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3393,7 +3393,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3621,7 +3621,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3735,7 +3735,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3849,7 +3849,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -3963,7 +3963,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4077,7 +4077,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4191,7 +4191,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4305,7 +4305,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4419,7 +4419,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4533,7 +4533,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4647,7 +4647,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4761,7 +4761,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4875,7 +4875,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -4989,7 +4989,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5103,7 +5103,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5217,7 +5217,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5331,7 +5331,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5445,7 +5445,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5559,7 +5559,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5673,7 +5673,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5787,7 +5787,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5901,7 +5901,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6015,7 +6015,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6129,7 +6129,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6243,7 +6243,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6357,7 +6357,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6471,7 +6471,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6585,7 +6585,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6699,7 +6699,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6813,7 +6813,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -6927,7 +6927,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7041,7 +7041,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7155,7 +7155,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7269,7 +7269,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7383,7 +7383,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7497,7 +7497,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7611,7 +7611,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7725,7 +7725,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7839,7 +7839,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -7953,7 +7953,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8067,7 +8067,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8181,7 +8181,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8295,7 +8295,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8409,7 +8409,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8523,7 +8523,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8637,7 +8637,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8751,7 +8751,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8865,7 +8865,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -8979,7 +8979,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9093,7 +9093,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9207,7 +9207,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9321,7 +9321,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9435,7 +9435,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9549,7 +9549,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9663,7 +9663,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9777,7 +9777,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -9891,7 +9891,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10005,7 +10005,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10119,7 +10119,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10233,7 +10233,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10347,7 +10347,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10461,7 +10461,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10575,7 +10575,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10689,7 +10689,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10803,7 +10803,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -10917,7 +10917,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11031,7 +11031,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11145,7 +11145,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11259,7 +11259,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11373,7 +11373,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11487,7 +11487,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11601,7 +11601,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11715,7 +11715,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11829,7 +11829,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -11943,7 +11943,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12057,7 +12057,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12171,7 +12171,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12285,7 +12285,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12399,7 +12399,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12513,7 +12513,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12627,7 +12627,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12741,7 +12741,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12855,7 +12855,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -12969,7 +12969,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13092,7 +13092,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13215,7 +13215,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13338,7 +13338,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13461,7 +13461,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13584,7 +13584,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13707,7 +13707,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13830,7 +13830,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -13953,7 +13953,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14076,7 +14076,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14190,7 +14190,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14304,7 +14304,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14418,7 +14418,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14532,7 +14532,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14646,7 +14646,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14760,7 +14760,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14874,7 +14874,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -14988,7 +14988,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15102,7 +15102,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15216,7 +15216,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15330,7 +15330,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15444,7 +15444,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15558,7 +15558,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15672,7 +15672,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15786,7 +15786,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -15900,7 +15900,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16014,7 +16014,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16128,7 +16128,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16242,7 +16242,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16356,7 +16356,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16470,7 +16470,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16584,7 +16584,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16698,7 +16698,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16812,7 +16812,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -16926,7 +16926,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17040,7 +17040,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17154,7 +17154,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17268,7 +17268,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17382,7 +17382,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17496,7 +17496,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17610,7 +17610,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17724,7 +17724,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17838,7 +17838,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -17952,7 +17952,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18066,7 +18066,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18180,7 +18180,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18303,7 +18303,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18426,7 +18426,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18549,7 +18549,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18672,7 +18672,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18795,7 +18795,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18918,7 +18918,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19041,7 +19041,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19164,7 +19164,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19287,7 +19287,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19401,7 +19401,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19515,7 +19515,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19629,7 +19629,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19743,7 +19743,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19857,7 +19857,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -19971,7 +19971,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -20085,7 +20085,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20199,7 +20199,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20313,7 +20313,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20427,7 +20427,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20541,7 +20541,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20655,7 +20655,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20769,7 +20769,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20883,7 +20883,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -20997,7 +20997,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21111,7 +21111,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21225,7 +21225,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21339,7 +21339,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21453,7 +21453,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21567,7 +21567,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21681,7 +21681,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21795,7 +21795,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21909,7 +21909,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -22023,7 +22023,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22137,7 +22137,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22251,7 +22251,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22365,7 +22365,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22471,7 +22471,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22577,7 +22577,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22683,7 +22683,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22789,7 +22789,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -22895,7 +22895,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -23001,7 +23001,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23107,7 +23107,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23213,7 +23213,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:22 AM PT</t>
+          <t>2026-07-12 09:02:22 AM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23319,7 +23319,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23433,7 +23433,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23547,7 +23547,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23661,7 +23661,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23775,7 +23775,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -23889,7 +23889,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -24003,7 +24003,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24117,7 +24117,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24231,7 +24231,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-12 09:00:21 AM PT</t>
+          <t>2026-07-12 09:02:21 AM PT</t>
         </is>
       </c>
       <c r="C208" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-12 09:45:36 AM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
@@ -669,7 +669,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -697,10 +697,10 @@
         <v>2</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -792,7 +792,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -820,10 +820,10 @@
         <v>2</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -915,7 +915,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -943,10 +943,10 @@
         <v>2</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -1038,7 +1038,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1066,10 +1066,10 @@
         <v>2</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1389,7 +1389,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1503,7 +1503,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1617,7 +1617,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1959,7 +1959,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2073,7 +2073,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2301,7 +2301,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2415,7 +2415,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2529,7 +2529,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2643,7 +2643,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2757,7 +2757,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2985,7 +2985,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3099,7 +3099,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3213,7 +3213,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3327,7 +3327,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3441,7 +3441,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3555,7 +3555,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3669,7 +3669,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3783,7 +3783,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3897,7 +3897,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -4011,7 +4011,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4125,7 +4125,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4239,7 +4239,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4353,7 +4353,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4467,7 +4467,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4581,7 +4581,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4695,7 +4695,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4809,7 +4809,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4923,7 +4923,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5037,7 +5037,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5151,7 +5151,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5265,7 +5265,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5379,7 +5379,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5493,7 +5493,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5607,7 +5607,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5721,7 +5721,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5835,7 +5835,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5949,7 +5949,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6063,7 +6063,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6177,7 +6177,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6291,7 +6291,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6405,7 +6405,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6519,7 +6519,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6633,7 +6633,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6747,7 +6747,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6861,7 +6861,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -6975,7 +6975,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7089,7 +7089,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7203,7 +7203,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7317,7 +7317,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7431,7 +7431,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7545,7 +7545,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7659,7 +7659,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7773,7 +7773,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7887,7 +7887,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -8001,7 +8001,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8115,7 +8115,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8229,7 +8229,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8343,7 +8343,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8457,7 +8457,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8571,7 +8571,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8685,7 +8685,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8799,7 +8799,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8913,7 +8913,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9027,7 +9027,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9141,7 +9141,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9255,7 +9255,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9369,7 +9369,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9483,7 +9483,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9597,7 +9597,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9711,7 +9711,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9825,7 +9825,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -9939,7 +9939,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10053,7 +10053,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10167,7 +10167,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10281,7 +10281,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10395,7 +10395,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10509,7 +10509,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10623,7 +10623,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10737,7 +10737,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10851,7 +10851,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -10965,7 +10965,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11079,7 +11079,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11193,7 +11193,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11307,7 +11307,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11421,7 +11421,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11535,7 +11535,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11649,7 +11649,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11763,7 +11763,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11877,7 +11877,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -11991,7 +11991,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12105,7 +12105,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12219,7 +12219,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12333,7 +12333,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12447,7 +12447,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12561,7 +12561,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12675,7 +12675,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12789,7 +12789,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12903,7 +12903,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13017,7 +13017,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13131,7 +13131,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13245,7 +13245,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13359,7 +13359,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13473,7 +13473,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13587,7 +13587,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13701,7 +13701,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13815,7 +13815,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -13929,7 +13929,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14043,7 +14043,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14157,7 +14157,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14271,7 +14271,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14385,7 +14385,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14499,7 +14499,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14527,10 +14527,10 @@
         <v>2</v>
       </c>
       <c r="I123" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J123" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K123" t="inlineStr">
         <is>
@@ -14622,7 +14622,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14650,10 +14650,10 @@
         <v>2</v>
       </c>
       <c r="I124" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J124" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K124" t="inlineStr">
         <is>
@@ -14745,7 +14745,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14773,10 +14773,10 @@
         <v>2</v>
       </c>
       <c r="I125" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J125" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K125" t="inlineStr">
         <is>
@@ -14868,7 +14868,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -14896,10 +14896,10 @@
         <v>2</v>
       </c>
       <c r="I126" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J126" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K126" t="inlineStr">
         <is>
@@ -14991,7 +14991,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15019,10 +15019,10 @@
         <v>2</v>
       </c>
       <c r="I127" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J127" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K127" t="inlineStr">
         <is>
@@ -15114,7 +15114,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15142,10 +15142,10 @@
         <v>2</v>
       </c>
       <c r="I128" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J128" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K128" t="inlineStr">
         <is>
@@ -15237,7 +15237,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15265,10 +15265,10 @@
         <v>2</v>
       </c>
       <c r="I129" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J129" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K129" t="inlineStr">
         <is>
@@ -15360,7 +15360,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15388,10 +15388,10 @@
         <v>2</v>
       </c>
       <c r="I130" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J130" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K130" t="inlineStr">
         <is>
@@ -15483,7 +15483,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15511,10 +15511,10 @@
         <v>2</v>
       </c>
       <c r="I131" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J131" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K131" t="inlineStr">
         <is>
@@ -15606,7 +15606,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15720,7 +15720,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15834,7 +15834,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -15948,7 +15948,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16062,7 +16062,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16176,7 +16176,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16290,7 +16290,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16404,7 +16404,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16518,7 +16518,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16632,7 +16632,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16746,7 +16746,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16860,7 +16860,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -16974,7 +16974,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17088,7 +17088,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17202,7 +17202,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17316,7 +17316,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17430,7 +17430,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17544,7 +17544,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17658,7 +17658,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17772,7 +17772,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17886,7 +17886,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -18000,7 +18000,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18114,7 +18114,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18228,7 +18228,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18342,7 +18342,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18456,7 +18456,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18570,7 +18570,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18684,7 +18684,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18798,7 +18798,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18912,7 +18912,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19026,7 +19026,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19140,7 +19140,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19254,7 +19254,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19368,7 +19368,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19482,7 +19482,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19596,7 +19596,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19710,7 +19710,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19738,10 +19738,10 @@
         <v>2</v>
       </c>
       <c r="I168" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J168" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K168" t="inlineStr">
         <is>
@@ -19833,7 +19833,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -19861,10 +19861,10 @@
         <v>2</v>
       </c>
       <c r="I169" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J169" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K169" t="inlineStr">
         <is>
@@ -19956,7 +19956,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -19984,10 +19984,10 @@
         <v>2</v>
       </c>
       <c r="I170" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J170" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K170" t="inlineStr">
         <is>
@@ -20079,7 +20079,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20107,10 +20107,10 @@
         <v>2</v>
       </c>
       <c r="I171" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J171" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K171" t="inlineStr">
         <is>
@@ -20202,7 +20202,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20230,10 +20230,10 @@
         <v>2</v>
       </c>
       <c r="I172" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J172" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K172" t="inlineStr">
         <is>
@@ -20325,7 +20325,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20439,7 +20439,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20553,7 +20553,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20667,7 +20667,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20781,7 +20781,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20895,7 +20895,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -21009,7 +21009,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21123,7 +21123,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21237,7 +21237,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21351,7 +21351,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21457,7 +21457,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21563,7 +21563,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21669,7 +21669,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21775,7 +21775,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21881,7 +21881,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -21987,7 +21987,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22093,7 +22093,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22199,7 +22199,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22305,7 +22305,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22419,7 +22419,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22533,7 +22533,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22647,7 +22647,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22761,7 +22761,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -22875,7 +22875,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -22989,7 +22989,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23103,7 +23103,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23217,7 +23217,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23331,7 +23331,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23445,7 +23445,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23559,7 +23559,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23673,7 +23673,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23787,7 +23787,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -23901,7 +23901,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -24015,7 +24015,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24129,7 +24129,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24243,7 +24243,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24357,7 +24357,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24471,7 +24471,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24585,7 +24585,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24699,7 +24699,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -24813,7 +24813,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -24927,7 +24927,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -25041,7 +25041,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25155,7 +25155,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25269,7 +25269,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:34 AM PT</t>
+          <t>2026-07-12 09:45:34 AM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25383,7 +25383,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25497,7 +25497,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25611,7 +25611,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25725,7 +25725,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -25839,7 +25839,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -25953,7 +25953,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26067,7 +26067,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26181,7 +26181,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26295,7 +26295,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-12 09:43:33 AM PT</t>
+          <t>2026-07-12 09:45:33 AM PT</t>
         </is>
       </c>
       <c r="C226" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-12 09:47:36 AM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
@@ -463,7 +463,7 @@
     <col width="27" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
@@ -669,7 +669,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -682,25 +682,25 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Bottom 2 | 2 out</t>
+          <t>Top 3 | 0 out</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -792,7 +792,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -805,25 +805,25 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Bottom 2 | 2 out</t>
+          <t>Top 3 | 0 out</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -915,7 +915,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -928,25 +928,25 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Bottom 2 | 2 out</t>
+          <t>Top 3 | 0 out</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -1038,7 +1038,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1051,25 +1051,25 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Bottom 2 | 2 out</t>
+          <t>Top 3 | 0 out</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1389,7 +1389,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1503,7 +1503,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1617,7 +1617,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1959,7 +1959,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2073,7 +2073,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2301,7 +2301,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2415,7 +2415,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2529,7 +2529,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2643,7 +2643,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2757,7 +2757,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2985,7 +2985,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3099,7 +3099,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3213,7 +3213,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3327,7 +3327,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3441,7 +3441,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3555,7 +3555,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3669,7 +3669,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3783,7 +3783,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3897,7 +3897,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -4011,7 +4011,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4125,7 +4125,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4239,7 +4239,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4353,7 +4353,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4467,7 +4467,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4581,7 +4581,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4695,7 +4695,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4809,7 +4809,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4923,7 +4923,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5037,7 +5037,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5151,7 +5151,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5265,7 +5265,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5379,7 +5379,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5493,7 +5493,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5607,7 +5607,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5721,7 +5721,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5835,7 +5835,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5949,7 +5949,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6063,7 +6063,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6177,7 +6177,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6291,7 +6291,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6405,7 +6405,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6519,7 +6519,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6633,7 +6633,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6747,7 +6747,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6861,7 +6861,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -6975,7 +6975,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7089,7 +7089,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7203,7 +7203,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7317,7 +7317,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7431,7 +7431,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7545,7 +7545,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7659,7 +7659,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7773,7 +7773,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7887,7 +7887,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -8001,7 +8001,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8115,7 +8115,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8229,7 +8229,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8343,7 +8343,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8457,7 +8457,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8571,7 +8571,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8685,7 +8685,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8799,7 +8799,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8913,7 +8913,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9027,7 +9027,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9141,7 +9141,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9255,7 +9255,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9369,7 +9369,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9483,7 +9483,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9597,7 +9597,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9711,7 +9711,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9825,7 +9825,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -9939,7 +9939,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10053,7 +10053,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10167,7 +10167,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10281,7 +10281,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10395,7 +10395,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10509,7 +10509,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10623,7 +10623,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10737,7 +10737,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10851,7 +10851,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -10965,7 +10965,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11079,7 +11079,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11193,7 +11193,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11307,7 +11307,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11421,7 +11421,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11535,7 +11535,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11649,7 +11649,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11763,7 +11763,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11877,7 +11877,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -11991,7 +11991,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12105,7 +12105,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12219,7 +12219,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12333,7 +12333,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12447,7 +12447,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12561,7 +12561,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12675,7 +12675,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12789,7 +12789,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12903,7 +12903,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13017,7 +13017,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13131,7 +13131,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13245,7 +13245,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13359,7 +13359,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13473,7 +13473,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13587,7 +13587,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13701,7 +13701,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13815,7 +13815,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -13929,7 +13929,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14043,7 +14043,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14157,7 +14157,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14271,7 +14271,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14385,7 +14385,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14499,7 +14499,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14512,25 +14512,25 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Bottom 2 | 2 out</t>
+          <t>Top 3 | 0 out</t>
         </is>
       </c>
       <c r="F123" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H123" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I123" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J123" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K123" t="inlineStr">
         <is>
@@ -14622,7 +14622,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14635,25 +14635,25 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Bottom 2 | 2 out</t>
+          <t>Top 3 | 0 out</t>
         </is>
       </c>
       <c r="F124" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H124" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I124" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J124" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K124" t="inlineStr">
         <is>
@@ -14745,7 +14745,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14758,25 +14758,25 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Bottom 2 | 2 out</t>
+          <t>Top 3 | 0 out</t>
         </is>
       </c>
       <c r="F125" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H125" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I125" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J125" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K125" t="inlineStr">
         <is>
@@ -14868,7 +14868,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -14881,25 +14881,25 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Bottom 2 | 2 out</t>
+          <t>Top 3 | 0 out</t>
         </is>
       </c>
       <c r="F126" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H126" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I126" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J126" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K126" t="inlineStr">
         <is>
@@ -14991,7 +14991,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15004,25 +15004,25 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Bottom 2 | 2 out</t>
+          <t>Top 3 | 0 out</t>
         </is>
       </c>
       <c r="F127" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H127" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I127" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J127" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K127" t="inlineStr">
         <is>
@@ -15114,7 +15114,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15127,25 +15127,25 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Bottom 2 | 2 out</t>
+          <t>Top 3 | 0 out</t>
         </is>
       </c>
       <c r="F128" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H128" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I128" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J128" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K128" t="inlineStr">
         <is>
@@ -15237,7 +15237,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15250,25 +15250,25 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Bottom 2 | 2 out</t>
+          <t>Top 3 | 0 out</t>
         </is>
       </c>
       <c r="F129" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H129" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I129" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J129" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K129" t="inlineStr">
         <is>
@@ -15360,7 +15360,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15373,25 +15373,25 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Bottom 2 | 2 out</t>
+          <t>Top 3 | 0 out</t>
         </is>
       </c>
       <c r="F130" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H130" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I130" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J130" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K130" t="inlineStr">
         <is>
@@ -15483,7 +15483,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15496,25 +15496,25 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Bottom 2 | 2 out</t>
+          <t>Top 3 | 0 out</t>
         </is>
       </c>
       <c r="F131" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H131" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I131" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J131" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K131" t="inlineStr">
         <is>
@@ -15606,7 +15606,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15720,7 +15720,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15834,7 +15834,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -15948,7 +15948,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16062,7 +16062,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16176,7 +16176,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16290,7 +16290,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16404,7 +16404,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16518,7 +16518,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16632,7 +16632,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16746,7 +16746,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16860,7 +16860,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -16974,7 +16974,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17088,7 +17088,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17202,7 +17202,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17316,7 +17316,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17430,7 +17430,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17544,7 +17544,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17658,7 +17658,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17772,7 +17772,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17886,7 +17886,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -18000,7 +18000,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18114,7 +18114,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18228,7 +18228,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18342,7 +18342,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18456,7 +18456,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18570,7 +18570,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18684,7 +18684,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18798,7 +18798,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18912,7 +18912,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19026,7 +19026,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19140,7 +19140,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19254,7 +19254,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19368,7 +19368,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19482,7 +19482,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19596,7 +19596,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19710,7 +19710,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19723,25 +19723,25 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>Bottom 2 | 2 out</t>
+          <t>Top 3 | 0 out</t>
         </is>
       </c>
       <c r="F168" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H168" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I168" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J168" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K168" t="inlineStr">
         <is>
@@ -19777,10 +19777,10 @@
         </is>
       </c>
       <c r="R168" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S168" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T168" t="n">
         <v>0</v>
@@ -19833,7 +19833,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -19846,25 +19846,25 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>Bottom 2 | 2 out</t>
+          <t>Top 3 | 0 out</t>
         </is>
       </c>
       <c r="F169" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H169" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I169" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J169" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K169" t="inlineStr">
         <is>
@@ -19956,7 +19956,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -19969,25 +19969,25 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>Bottom 2 | 2 out</t>
+          <t>Top 3 | 0 out</t>
         </is>
       </c>
       <c r="F170" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H170" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I170" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J170" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K170" t="inlineStr">
         <is>
@@ -20079,7 +20079,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20092,25 +20092,25 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>Bottom 2 | 2 out</t>
+          <t>Top 3 | 0 out</t>
         </is>
       </c>
       <c r="F171" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H171" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I171" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J171" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K171" t="inlineStr">
         <is>
@@ -20202,7 +20202,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20215,25 +20215,25 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>Bottom 2 | 2 out</t>
+          <t>Top 3 | 0 out</t>
         </is>
       </c>
       <c r="F172" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H172" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I172" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J172" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K172" t="inlineStr">
         <is>
@@ -20325,7 +20325,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20439,7 +20439,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20553,7 +20553,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20667,7 +20667,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20781,7 +20781,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20895,7 +20895,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -21009,7 +21009,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21123,7 +21123,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21237,7 +21237,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21351,7 +21351,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21457,7 +21457,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21563,7 +21563,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21669,7 +21669,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21775,7 +21775,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21881,7 +21881,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -21987,7 +21987,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22093,7 +22093,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22199,7 +22199,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22305,7 +22305,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22419,7 +22419,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22533,7 +22533,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22647,7 +22647,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22761,7 +22761,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -22875,7 +22875,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -22989,7 +22989,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23103,7 +23103,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23217,7 +23217,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23331,7 +23331,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23445,7 +23445,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23559,7 +23559,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23673,7 +23673,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23787,7 +23787,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -23901,7 +23901,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -24015,7 +24015,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24129,7 +24129,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24243,7 +24243,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24357,7 +24357,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24471,7 +24471,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24585,7 +24585,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24699,7 +24699,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -24813,7 +24813,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -24927,7 +24927,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -25041,7 +25041,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25155,7 +25155,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25269,7 +25269,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:34 AM PT</t>
+          <t>2026-07-12 09:47:34 AM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25383,7 +25383,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25497,7 +25497,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25611,7 +25611,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25725,7 +25725,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -25839,7 +25839,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -25953,7 +25953,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26067,7 +26067,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26181,7 +26181,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26295,7 +26295,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-12 09:45:33 AM PT</t>
+          <t>2026-07-12 09:47:33 AM PT</t>
         </is>
       </c>
       <c r="C226" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-12 09:49:36 AM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
@@ -669,7 +669,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -697,10 +697,10 @@
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -792,7 +792,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -820,10 +820,10 @@
         <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -915,7 +915,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -943,10 +943,10 @@
         <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -1038,7 +1038,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1066,10 +1066,10 @@
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1389,7 +1389,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1503,7 +1503,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1617,7 +1617,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1959,7 +1959,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2073,7 +2073,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2301,7 +2301,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2415,7 +2415,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2529,7 +2529,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2643,7 +2643,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2757,7 +2757,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2985,7 +2985,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3099,7 +3099,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3213,7 +3213,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3327,7 +3327,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3441,7 +3441,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3555,7 +3555,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3669,7 +3669,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3783,7 +3783,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3897,7 +3897,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -4011,7 +4011,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4125,7 +4125,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4239,7 +4239,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4353,7 +4353,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4467,7 +4467,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4581,7 +4581,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4695,7 +4695,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4809,7 +4809,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4923,7 +4923,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5037,7 +5037,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5151,7 +5151,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5265,7 +5265,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5379,7 +5379,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5493,7 +5493,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5607,7 +5607,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5721,7 +5721,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5835,7 +5835,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5949,7 +5949,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6063,7 +6063,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6177,7 +6177,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6291,7 +6291,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6405,7 +6405,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6519,7 +6519,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6633,7 +6633,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6747,7 +6747,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6861,7 +6861,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -6975,7 +6975,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7089,7 +7089,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7203,7 +7203,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7317,7 +7317,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7431,7 +7431,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7545,7 +7545,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7659,7 +7659,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7773,7 +7773,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7887,7 +7887,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -8001,7 +8001,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8115,7 +8115,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8229,7 +8229,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8343,7 +8343,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8457,7 +8457,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8571,7 +8571,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8685,7 +8685,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8799,7 +8799,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8913,7 +8913,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9027,7 +9027,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9141,7 +9141,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9255,7 +9255,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9369,7 +9369,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9483,7 +9483,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9597,7 +9597,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9711,7 +9711,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9825,7 +9825,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -9939,7 +9939,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10053,7 +10053,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10167,7 +10167,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10281,7 +10281,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10395,7 +10395,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10509,7 +10509,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10623,7 +10623,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10737,7 +10737,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10851,7 +10851,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -10965,7 +10965,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11079,7 +11079,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11193,7 +11193,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11307,7 +11307,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11421,7 +11421,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11535,7 +11535,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11649,7 +11649,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11763,7 +11763,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11877,7 +11877,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -11991,7 +11991,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12105,7 +12105,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12219,7 +12219,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12333,7 +12333,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12447,7 +12447,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12561,7 +12561,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12675,7 +12675,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12789,7 +12789,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12903,7 +12903,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13017,7 +13017,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13131,7 +13131,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13245,7 +13245,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13359,7 +13359,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13473,7 +13473,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13587,7 +13587,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13701,7 +13701,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13815,7 +13815,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -13929,7 +13929,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14043,7 +14043,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14157,7 +14157,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14271,7 +14271,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14385,7 +14385,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14499,7 +14499,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14527,10 +14527,10 @@
         <v>0</v>
       </c>
       <c r="I123" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J123" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K123" t="inlineStr">
         <is>
@@ -14622,7 +14622,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14650,10 +14650,10 @@
         <v>0</v>
       </c>
       <c r="I124" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J124" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K124" t="inlineStr">
         <is>
@@ -14745,7 +14745,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14773,10 +14773,10 @@
         <v>0</v>
       </c>
       <c r="I125" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J125" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K125" t="inlineStr">
         <is>
@@ -14868,7 +14868,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -14896,10 +14896,10 @@
         <v>0</v>
       </c>
       <c r="I126" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J126" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K126" t="inlineStr">
         <is>
@@ -14991,7 +14991,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15019,10 +15019,10 @@
         <v>0</v>
       </c>
       <c r="I127" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J127" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K127" t="inlineStr">
         <is>
@@ -15114,7 +15114,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15142,10 +15142,10 @@
         <v>0</v>
       </c>
       <c r="I128" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J128" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K128" t="inlineStr">
         <is>
@@ -15237,7 +15237,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15265,10 +15265,10 @@
         <v>0</v>
       </c>
       <c r="I129" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J129" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K129" t="inlineStr">
         <is>
@@ -15360,7 +15360,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15388,10 +15388,10 @@
         <v>0</v>
       </c>
       <c r="I130" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J130" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K130" t="inlineStr">
         <is>
@@ -15483,7 +15483,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15511,10 +15511,10 @@
         <v>0</v>
       </c>
       <c r="I131" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J131" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K131" t="inlineStr">
         <is>
@@ -15606,7 +15606,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15720,7 +15720,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15834,7 +15834,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -15948,7 +15948,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16062,7 +16062,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16176,7 +16176,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16290,7 +16290,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16404,7 +16404,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16518,7 +16518,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16632,7 +16632,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16746,7 +16746,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16860,7 +16860,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -16974,7 +16974,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17088,7 +17088,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17202,7 +17202,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17316,7 +17316,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17430,7 +17430,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17544,7 +17544,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17658,7 +17658,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17772,7 +17772,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17886,7 +17886,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -18000,7 +18000,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18114,7 +18114,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18228,7 +18228,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18342,7 +18342,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18456,7 +18456,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18570,7 +18570,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18684,7 +18684,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18798,7 +18798,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18912,7 +18912,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19026,7 +19026,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19140,7 +19140,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19254,7 +19254,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19368,7 +19368,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19482,7 +19482,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19596,7 +19596,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19710,7 +19710,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19738,10 +19738,10 @@
         <v>0</v>
       </c>
       <c r="I168" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J168" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K168" t="inlineStr">
         <is>
@@ -19833,7 +19833,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -19861,10 +19861,10 @@
         <v>0</v>
       </c>
       <c r="I169" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J169" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K169" t="inlineStr">
         <is>
@@ -19956,7 +19956,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -19984,10 +19984,10 @@
         <v>0</v>
       </c>
       <c r="I170" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J170" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K170" t="inlineStr">
         <is>
@@ -20079,7 +20079,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20107,10 +20107,10 @@
         <v>0</v>
       </c>
       <c r="I171" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J171" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K171" t="inlineStr">
         <is>
@@ -20202,7 +20202,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20230,10 +20230,10 @@
         <v>0</v>
       </c>
       <c r="I172" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J172" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K172" t="inlineStr">
         <is>
@@ -20325,7 +20325,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20439,7 +20439,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20553,7 +20553,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20667,7 +20667,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20781,7 +20781,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20895,7 +20895,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -21009,7 +21009,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21123,7 +21123,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21237,7 +21237,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21351,7 +21351,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21457,7 +21457,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21563,7 +21563,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21669,7 +21669,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21775,7 +21775,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21881,7 +21881,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -21987,7 +21987,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22093,7 +22093,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22199,7 +22199,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22305,7 +22305,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22419,7 +22419,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22533,7 +22533,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22647,7 +22647,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22761,7 +22761,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -22875,7 +22875,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -22989,7 +22989,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23103,7 +23103,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23217,7 +23217,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23331,7 +23331,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23445,7 +23445,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23559,7 +23559,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23673,7 +23673,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23787,7 +23787,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -23901,7 +23901,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -24015,7 +24015,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24129,7 +24129,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24243,7 +24243,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24357,7 +24357,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24471,7 +24471,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24585,7 +24585,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24699,7 +24699,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -24813,7 +24813,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -24927,7 +24927,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -25041,7 +25041,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25155,7 +25155,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25269,7 +25269,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:34 AM PT</t>
+          <t>2026-07-12 09:49:34 AM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25383,7 +25383,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25497,7 +25497,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25611,7 +25611,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25725,7 +25725,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -25839,7 +25839,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -25953,7 +25953,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26067,7 +26067,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26181,7 +26181,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26295,7 +26295,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-12 09:47:33 AM PT</t>
+          <t>2026-07-12 09:49:33 AM PT</t>
         </is>
       </c>
       <c r="C226" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-12 09:53:36 AM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
@@ -669,7 +669,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -682,7 +682,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Top 3 | 1 out</t>
+          <t>Top 3 | 2 out</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -694,10 +694,10 @@
         </is>
       </c>
       <c r="H2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I2" t="n">
         <v>1</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
       </c>
       <c r="J2" t="n">
         <v>2</v>
@@ -792,7 +792,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -805,7 +805,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Top 3 | 1 out</t>
+          <t>Top 3 | 2 out</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -817,10 +817,10 @@
         </is>
       </c>
       <c r="H3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I3" t="n">
         <v>1</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0</v>
       </c>
       <c r="J3" t="n">
         <v>2</v>
@@ -915,7 +915,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -928,7 +928,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Top 3 | 1 out</t>
+          <t>Top 3 | 2 out</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -940,10 +940,10 @@
         </is>
       </c>
       <c r="H4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I4" t="n">
         <v>1</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0</v>
       </c>
       <c r="J4" t="n">
         <v>2</v>
@@ -1038,7 +1038,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1051,7 +1051,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Top 3 | 1 out</t>
+          <t>Top 3 | 2 out</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -1063,10 +1063,10 @@
         </is>
       </c>
       <c r="H5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I5" t="n">
         <v>1</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0</v>
       </c>
       <c r="J5" t="n">
         <v>2</v>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1389,7 +1389,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1503,7 +1503,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1617,7 +1617,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1959,7 +1959,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2073,7 +2073,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2301,7 +2301,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2415,7 +2415,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2529,7 +2529,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2643,7 +2643,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2757,7 +2757,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2985,7 +2985,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3099,7 +3099,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3213,7 +3213,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3327,7 +3327,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3441,7 +3441,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3555,7 +3555,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3669,7 +3669,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3783,7 +3783,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3897,7 +3897,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -4011,7 +4011,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4125,7 +4125,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4239,7 +4239,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4353,7 +4353,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4467,7 +4467,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4581,7 +4581,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4695,7 +4695,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4809,7 +4809,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4923,7 +4923,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5037,7 +5037,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5151,7 +5151,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5265,7 +5265,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5379,7 +5379,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5493,7 +5493,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5607,7 +5607,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5721,7 +5721,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5835,7 +5835,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5949,7 +5949,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6063,7 +6063,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6177,7 +6177,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6291,7 +6291,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6405,7 +6405,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6519,7 +6519,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6633,7 +6633,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6747,7 +6747,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6861,7 +6861,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -6975,7 +6975,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7089,7 +7089,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7203,7 +7203,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7317,7 +7317,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7431,7 +7431,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7545,7 +7545,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7659,7 +7659,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7773,7 +7773,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7887,7 +7887,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -8001,7 +8001,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8115,7 +8115,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8229,7 +8229,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8343,7 +8343,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8457,7 +8457,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8571,7 +8571,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8685,7 +8685,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8799,7 +8799,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8913,7 +8913,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9027,7 +9027,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9141,7 +9141,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9255,7 +9255,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9369,7 +9369,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9483,7 +9483,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9597,7 +9597,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9711,7 +9711,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9825,7 +9825,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -9939,7 +9939,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10053,7 +10053,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10167,7 +10167,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10281,7 +10281,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10395,7 +10395,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10509,7 +10509,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10623,7 +10623,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10737,7 +10737,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10851,7 +10851,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -10965,7 +10965,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11079,7 +11079,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11193,7 +11193,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11307,7 +11307,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11421,7 +11421,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11535,7 +11535,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11649,7 +11649,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11763,7 +11763,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11877,7 +11877,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -11991,7 +11991,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12105,7 +12105,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12219,7 +12219,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12333,7 +12333,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12447,7 +12447,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12561,7 +12561,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12675,7 +12675,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12789,7 +12789,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12903,7 +12903,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13017,7 +13017,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13131,7 +13131,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13245,7 +13245,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13359,7 +13359,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13473,7 +13473,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13587,7 +13587,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13701,7 +13701,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13815,7 +13815,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -13929,7 +13929,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14043,7 +14043,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14157,7 +14157,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14271,7 +14271,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14385,7 +14385,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14499,7 +14499,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14512,7 +14512,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Top 3 | 1 out</t>
+          <t>Top 3 | 2 out</t>
         </is>
       </c>
       <c r="F123" t="n">
@@ -14524,10 +14524,10 @@
         </is>
       </c>
       <c r="H123" t="n">
+        <v>2</v>
+      </c>
+      <c r="I123" t="n">
         <v>1</v>
-      </c>
-      <c r="I123" t="n">
-        <v>0</v>
       </c>
       <c r="J123" t="n">
         <v>2</v>
@@ -14622,7 +14622,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14635,7 +14635,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Top 3 | 1 out</t>
+          <t>Top 3 | 2 out</t>
         </is>
       </c>
       <c r="F124" t="n">
@@ -14647,10 +14647,10 @@
         </is>
       </c>
       <c r="H124" t="n">
+        <v>2</v>
+      </c>
+      <c r="I124" t="n">
         <v>1</v>
-      </c>
-      <c r="I124" t="n">
-        <v>0</v>
       </c>
       <c r="J124" t="n">
         <v>2</v>
@@ -14745,7 +14745,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14758,7 +14758,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Top 3 | 1 out</t>
+          <t>Top 3 | 2 out</t>
         </is>
       </c>
       <c r="F125" t="n">
@@ -14770,10 +14770,10 @@
         </is>
       </c>
       <c r="H125" t="n">
+        <v>2</v>
+      </c>
+      <c r="I125" t="n">
         <v>1</v>
-      </c>
-      <c r="I125" t="n">
-        <v>0</v>
       </c>
       <c r="J125" t="n">
         <v>2</v>
@@ -14868,7 +14868,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -14881,7 +14881,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Top 3 | 1 out</t>
+          <t>Top 3 | 2 out</t>
         </is>
       </c>
       <c r="F126" t="n">
@@ -14893,10 +14893,10 @@
         </is>
       </c>
       <c r="H126" t="n">
+        <v>2</v>
+      </c>
+      <c r="I126" t="n">
         <v>1</v>
-      </c>
-      <c r="I126" t="n">
-        <v>0</v>
       </c>
       <c r="J126" t="n">
         <v>2</v>
@@ -14991,7 +14991,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15004,7 +15004,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Top 3 | 1 out</t>
+          <t>Top 3 | 2 out</t>
         </is>
       </c>
       <c r="F127" t="n">
@@ -15016,10 +15016,10 @@
         </is>
       </c>
       <c r="H127" t="n">
+        <v>2</v>
+      </c>
+      <c r="I127" t="n">
         <v>1</v>
-      </c>
-      <c r="I127" t="n">
-        <v>0</v>
       </c>
       <c r="J127" t="n">
         <v>2</v>
@@ -15114,7 +15114,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15127,7 +15127,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Top 3 | 1 out</t>
+          <t>Top 3 | 2 out</t>
         </is>
       </c>
       <c r="F128" t="n">
@@ -15139,10 +15139,10 @@
         </is>
       </c>
       <c r="H128" t="n">
+        <v>2</v>
+      </c>
+      <c r="I128" t="n">
         <v>1</v>
-      </c>
-      <c r="I128" t="n">
-        <v>0</v>
       </c>
       <c r="J128" t="n">
         <v>2</v>
@@ -15237,7 +15237,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15250,7 +15250,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Top 3 | 1 out</t>
+          <t>Top 3 | 2 out</t>
         </is>
       </c>
       <c r="F129" t="n">
@@ -15262,10 +15262,10 @@
         </is>
       </c>
       <c r="H129" t="n">
+        <v>2</v>
+      </c>
+      <c r="I129" t="n">
         <v>1</v>
-      </c>
-      <c r="I129" t="n">
-        <v>0</v>
       </c>
       <c r="J129" t="n">
         <v>2</v>
@@ -15360,7 +15360,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15373,7 +15373,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Top 3 | 1 out</t>
+          <t>Top 3 | 2 out</t>
         </is>
       </c>
       <c r="F130" t="n">
@@ -15385,10 +15385,10 @@
         </is>
       </c>
       <c r="H130" t="n">
+        <v>2</v>
+      </c>
+      <c r="I130" t="n">
         <v>1</v>
-      </c>
-      <c r="I130" t="n">
-        <v>0</v>
       </c>
       <c r="J130" t="n">
         <v>2</v>
@@ -15427,10 +15427,10 @@
         </is>
       </c>
       <c r="R130" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S130" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T130" t="n">
         <v>0</v>
@@ -15463,7 +15463,7 @@
         <v>0</v>
       </c>
       <c r="AD130" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE130" s="4" t="n">
         <v>0</v>
@@ -15483,7 +15483,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15496,7 +15496,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Top 3 | 1 out</t>
+          <t>Top 3 | 2 out</t>
         </is>
       </c>
       <c r="F131" t="n">
@@ -15508,10 +15508,10 @@
         </is>
       </c>
       <c r="H131" t="n">
+        <v>2</v>
+      </c>
+      <c r="I131" t="n">
         <v>1</v>
-      </c>
-      <c r="I131" t="n">
-        <v>0</v>
       </c>
       <c r="J131" t="n">
         <v>2</v>
@@ -15606,7 +15606,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15720,7 +15720,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15834,7 +15834,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -15948,7 +15948,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16062,7 +16062,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16176,7 +16176,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16290,7 +16290,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16404,7 +16404,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16518,7 +16518,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16632,7 +16632,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16746,7 +16746,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16860,7 +16860,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -16974,7 +16974,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17088,7 +17088,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17202,7 +17202,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17316,7 +17316,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17430,7 +17430,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17544,7 +17544,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17658,7 +17658,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17772,7 +17772,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17886,7 +17886,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -18000,7 +18000,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18114,7 +18114,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18228,7 +18228,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18342,7 +18342,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18456,7 +18456,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18570,7 +18570,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18684,7 +18684,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18798,7 +18798,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18912,7 +18912,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19026,7 +19026,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19140,7 +19140,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19254,7 +19254,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19368,7 +19368,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19482,7 +19482,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19596,7 +19596,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19710,7 +19710,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19723,7 +19723,7 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>Top 3 | 1 out</t>
+          <t>Top 3 | 2 out</t>
         </is>
       </c>
       <c r="F168" t="n">
@@ -19735,10 +19735,10 @@
         </is>
       </c>
       <c r="H168" t="n">
+        <v>2</v>
+      </c>
+      <c r="I168" t="n">
         <v>1</v>
-      </c>
-      <c r="I168" t="n">
-        <v>0</v>
       </c>
       <c r="J168" t="n">
         <v>2</v>
@@ -19833,7 +19833,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -19846,7 +19846,7 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>Top 3 | 1 out</t>
+          <t>Top 3 | 2 out</t>
         </is>
       </c>
       <c r="F169" t="n">
@@ -19858,10 +19858,10 @@
         </is>
       </c>
       <c r="H169" t="n">
+        <v>2</v>
+      </c>
+      <c r="I169" t="n">
         <v>1</v>
-      </c>
-      <c r="I169" t="n">
-        <v>0</v>
       </c>
       <c r="J169" t="n">
         <v>2</v>
@@ -19956,7 +19956,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -19969,7 +19969,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>Top 3 | 1 out</t>
+          <t>Top 3 | 2 out</t>
         </is>
       </c>
       <c r="F170" t="n">
@@ -19981,10 +19981,10 @@
         </is>
       </c>
       <c r="H170" t="n">
+        <v>2</v>
+      </c>
+      <c r="I170" t="n">
         <v>1</v>
-      </c>
-      <c r="I170" t="n">
-        <v>0</v>
       </c>
       <c r="J170" t="n">
         <v>2</v>
@@ -20079,7 +20079,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20092,7 +20092,7 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>Top 3 | 1 out</t>
+          <t>Top 3 | 2 out</t>
         </is>
       </c>
       <c r="F171" t="n">
@@ -20104,10 +20104,10 @@
         </is>
       </c>
       <c r="H171" t="n">
+        <v>2</v>
+      </c>
+      <c r="I171" t="n">
         <v>1</v>
-      </c>
-      <c r="I171" t="n">
-        <v>0</v>
       </c>
       <c r="J171" t="n">
         <v>2</v>
@@ -20202,7 +20202,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20215,7 +20215,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>Top 3 | 1 out</t>
+          <t>Top 3 | 2 out</t>
         </is>
       </c>
       <c r="F172" t="n">
@@ -20227,10 +20227,10 @@
         </is>
       </c>
       <c r="H172" t="n">
+        <v>2</v>
+      </c>
+      <c r="I172" t="n">
         <v>1</v>
-      </c>
-      <c r="I172" t="n">
-        <v>0</v>
       </c>
       <c r="J172" t="n">
         <v>2</v>
@@ -20325,7 +20325,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:35 AM PT</t>
+          <t>2026-07-12 09:53:35 AM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20431,7 +20431,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:35 AM PT</t>
+          <t>2026-07-12 09:53:35 AM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20537,7 +20537,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:35 AM PT</t>
+          <t>2026-07-12 09:53:35 AM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20643,7 +20643,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:35 AM PT</t>
+          <t>2026-07-12 09:53:35 AM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20749,7 +20749,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:35 AM PT</t>
+          <t>2026-07-12 09:53:35 AM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20855,7 +20855,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:35 AM PT</t>
+          <t>2026-07-12 09:53:35 AM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -20961,7 +20961,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:35 AM PT</t>
+          <t>2026-07-12 09:53:35 AM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21067,7 +21067,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:35 AM PT</t>
+          <t>2026-07-12 09:53:35 AM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21173,7 +21173,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:35 AM PT</t>
+          <t>2026-07-12 09:53:35 AM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21279,7 +21279,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21393,7 +21393,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21507,7 +21507,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21621,7 +21621,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21735,7 +21735,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21849,7 +21849,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -21963,7 +21963,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22077,7 +22077,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22191,7 +22191,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22305,7 +22305,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22411,7 +22411,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22517,7 +22517,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22623,7 +22623,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22729,7 +22729,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -22835,7 +22835,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -22941,7 +22941,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23047,7 +23047,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23153,7 +23153,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23259,7 +23259,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23373,7 +23373,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23487,7 +23487,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23601,7 +23601,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23715,7 +23715,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -23829,7 +23829,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -23943,7 +23943,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24057,7 +24057,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24171,7 +24171,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24285,7 +24285,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24399,7 +24399,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24513,7 +24513,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24627,7 +24627,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -24741,7 +24741,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -24855,7 +24855,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -24969,7 +24969,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25083,7 +25083,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25197,7 +25197,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25311,7 +25311,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25425,7 +25425,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25539,7 +25539,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25653,7 +25653,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -25767,7 +25767,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -25881,7 +25881,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -25995,7 +25995,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26109,7 +26109,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26223,7 +26223,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:34 AM PT</t>
+          <t>2026-07-12 09:53:34 AM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26337,7 +26337,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26451,7 +26451,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26565,7 +26565,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26679,7 +26679,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -26793,7 +26793,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -26907,7 +26907,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27021,7 +27021,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27135,7 +27135,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27249,7 +27249,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-12 09:51:33 AM PT</t>
+          <t>2026-07-12 09:53:33 AM PT</t>
         </is>
       </c>
       <c r="C235" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-12 09:55:36 AM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
@@ -463,7 +463,7 @@
     <col width="27" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
@@ -669,7 +669,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -682,7 +682,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Top 3 | 2 out</t>
+          <t>Bottom 3 | 0 out</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -690,17 +690,17 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -792,7 +792,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -805,7 +805,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Top 3 | 2 out</t>
+          <t>Bottom 3 | 0 out</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -813,17 +813,17 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -915,7 +915,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -928,7 +928,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Top 3 | 2 out</t>
+          <t>Bottom 3 | 0 out</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -936,17 +936,17 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -1038,7 +1038,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1051,7 +1051,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Top 3 | 2 out</t>
+          <t>Bottom 3 | 0 out</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -1059,17 +1059,17 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1389,7 +1389,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1503,7 +1503,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1617,7 +1617,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1959,7 +1959,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2073,7 +2073,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2301,7 +2301,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2415,7 +2415,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2529,7 +2529,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2643,7 +2643,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2757,7 +2757,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2985,7 +2985,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3099,7 +3099,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3213,7 +3213,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3327,7 +3327,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3441,7 +3441,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3555,7 +3555,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3669,7 +3669,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3783,7 +3783,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3897,7 +3897,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -4011,7 +4011,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4125,7 +4125,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4239,7 +4239,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4353,7 +4353,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4467,7 +4467,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4581,7 +4581,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4695,7 +4695,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4809,7 +4809,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4923,7 +4923,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5037,7 +5037,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5151,7 +5151,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5265,7 +5265,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5379,7 +5379,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5493,7 +5493,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5607,7 +5607,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5721,7 +5721,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5835,7 +5835,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5949,7 +5949,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6063,7 +6063,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6177,7 +6177,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6291,7 +6291,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6405,7 +6405,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6519,7 +6519,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6633,7 +6633,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6747,7 +6747,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6861,7 +6861,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -6975,7 +6975,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7089,7 +7089,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7203,7 +7203,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7317,7 +7317,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7431,7 +7431,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7545,7 +7545,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7659,7 +7659,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7773,7 +7773,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7887,7 +7887,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -8001,7 +8001,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8115,7 +8115,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8229,7 +8229,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8343,7 +8343,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8457,7 +8457,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8571,7 +8571,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8685,7 +8685,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8799,7 +8799,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8913,7 +8913,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9027,7 +9027,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9141,7 +9141,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9255,7 +9255,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9369,7 +9369,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9483,7 +9483,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9597,7 +9597,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9711,7 +9711,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9825,7 +9825,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -9939,7 +9939,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10053,7 +10053,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10167,7 +10167,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10281,7 +10281,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10395,7 +10395,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10509,7 +10509,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10623,7 +10623,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10737,7 +10737,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10851,7 +10851,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -10965,7 +10965,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11079,7 +11079,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11193,7 +11193,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11307,7 +11307,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11421,7 +11421,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11535,7 +11535,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11649,7 +11649,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11763,7 +11763,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11877,7 +11877,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -11991,7 +11991,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12105,7 +12105,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12219,7 +12219,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12333,7 +12333,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12447,7 +12447,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12561,7 +12561,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12675,7 +12675,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12789,7 +12789,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12903,7 +12903,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13017,7 +13017,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13131,7 +13131,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13245,7 +13245,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13359,7 +13359,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13473,7 +13473,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13587,7 +13587,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13701,7 +13701,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13815,7 +13815,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -13929,7 +13929,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14043,7 +14043,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14157,7 +14157,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14271,7 +14271,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14385,7 +14385,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14499,7 +14499,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14512,7 +14512,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Top 3 | 2 out</t>
+          <t>Bottom 3 | 0 out</t>
         </is>
       </c>
       <c r="F123" t="n">
@@ -14520,17 +14520,17 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H123" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I123" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J123" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K123" t="inlineStr">
         <is>
@@ -14622,7 +14622,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14635,7 +14635,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Top 3 | 2 out</t>
+          <t>Bottom 3 | 0 out</t>
         </is>
       </c>
       <c r="F124" t="n">
@@ -14643,17 +14643,17 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H124" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I124" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J124" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K124" t="inlineStr">
         <is>
@@ -14745,7 +14745,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14758,7 +14758,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Top 3 | 2 out</t>
+          <t>Bottom 3 | 0 out</t>
         </is>
       </c>
       <c r="F125" t="n">
@@ -14766,17 +14766,17 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H125" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I125" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J125" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K125" t="inlineStr">
         <is>
@@ -14868,7 +14868,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -14881,7 +14881,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Top 3 | 2 out</t>
+          <t>Bottom 3 | 0 out</t>
         </is>
       </c>
       <c r="F126" t="n">
@@ -14889,17 +14889,17 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H126" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I126" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J126" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K126" t="inlineStr">
         <is>
@@ -14991,7 +14991,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15004,7 +15004,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Top 3 | 2 out</t>
+          <t>Bottom 3 | 0 out</t>
         </is>
       </c>
       <c r="F127" t="n">
@@ -15012,17 +15012,17 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H127" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I127" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J127" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K127" t="inlineStr">
         <is>
@@ -15114,7 +15114,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15127,7 +15127,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Top 3 | 2 out</t>
+          <t>Bottom 3 | 0 out</t>
         </is>
       </c>
       <c r="F128" t="n">
@@ -15135,17 +15135,17 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H128" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I128" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J128" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K128" t="inlineStr">
         <is>
@@ -15237,7 +15237,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15250,7 +15250,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Top 3 | 2 out</t>
+          <t>Bottom 3 | 0 out</t>
         </is>
       </c>
       <c r="F129" t="n">
@@ -15258,17 +15258,17 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H129" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I129" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J129" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K129" t="inlineStr">
         <is>
@@ -15360,7 +15360,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15373,7 +15373,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Top 3 | 2 out</t>
+          <t>Bottom 3 | 0 out</t>
         </is>
       </c>
       <c r="F130" t="n">
@@ -15381,17 +15381,17 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H130" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I130" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J130" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K130" t="inlineStr">
         <is>
@@ -15483,7 +15483,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15496,7 +15496,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Top 3 | 2 out</t>
+          <t>Bottom 3 | 0 out</t>
         </is>
       </c>
       <c r="F131" t="n">
@@ -15504,17 +15504,17 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H131" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I131" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J131" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K131" t="inlineStr">
         <is>
@@ -15550,10 +15550,10 @@
         </is>
       </c>
       <c r="R131" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S131" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T131" t="n">
         <v>0</v>
@@ -15586,7 +15586,7 @@
         <v>0</v>
       </c>
       <c r="AD131" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE131" s="4" t="n">
         <v>0</v>
@@ -15606,7 +15606,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15720,7 +15720,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15834,7 +15834,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -15948,7 +15948,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16062,7 +16062,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16176,7 +16176,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16290,7 +16290,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16404,7 +16404,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16518,7 +16518,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16632,7 +16632,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16746,7 +16746,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16860,7 +16860,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -16974,7 +16974,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17088,7 +17088,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17202,7 +17202,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17316,7 +17316,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17430,7 +17430,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17544,7 +17544,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17658,7 +17658,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17772,7 +17772,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17886,7 +17886,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -18000,7 +18000,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18114,7 +18114,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18228,7 +18228,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18342,7 +18342,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18456,7 +18456,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18570,7 +18570,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18684,7 +18684,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18798,7 +18798,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18912,7 +18912,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19026,7 +19026,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19140,7 +19140,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19254,7 +19254,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19368,7 +19368,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19482,7 +19482,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19596,7 +19596,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19710,7 +19710,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19723,7 +19723,7 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>Top 3 | 2 out</t>
+          <t>Bottom 3 | 0 out</t>
         </is>
       </c>
       <c r="F168" t="n">
@@ -19731,17 +19731,17 @@
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H168" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I168" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J168" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K168" t="inlineStr">
         <is>
@@ -19833,7 +19833,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -19846,7 +19846,7 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>Top 3 | 2 out</t>
+          <t>Bottom 3 | 0 out</t>
         </is>
       </c>
       <c r="F169" t="n">
@@ -19854,17 +19854,17 @@
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H169" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I169" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J169" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K169" t="inlineStr">
         <is>
@@ -19956,7 +19956,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -19969,7 +19969,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>Top 3 | 2 out</t>
+          <t>Bottom 3 | 0 out</t>
         </is>
       </c>
       <c r="F170" t="n">
@@ -19977,17 +19977,17 @@
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H170" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I170" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J170" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K170" t="inlineStr">
         <is>
@@ -20079,7 +20079,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20092,7 +20092,7 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>Top 3 | 2 out</t>
+          <t>Bottom 3 | 0 out</t>
         </is>
       </c>
       <c r="F171" t="n">
@@ -20100,17 +20100,17 @@
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H171" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I171" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J171" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K171" t="inlineStr">
         <is>
@@ -20202,7 +20202,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20215,7 +20215,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>Top 3 | 2 out</t>
+          <t>Bottom 3 | 0 out</t>
         </is>
       </c>
       <c r="F172" t="n">
@@ -20223,17 +20223,17 @@
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H172" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I172" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J172" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K172" t="inlineStr">
         <is>
@@ -20325,7 +20325,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:35 AM PT</t>
+          <t>2026-07-12 09:55:35 AM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20431,7 +20431,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:35 AM PT</t>
+          <t>2026-07-12 09:55:35 AM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20537,7 +20537,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:35 AM PT</t>
+          <t>2026-07-12 09:55:35 AM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20643,7 +20643,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:35 AM PT</t>
+          <t>2026-07-12 09:55:35 AM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20749,7 +20749,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:35 AM PT</t>
+          <t>2026-07-12 09:55:35 AM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20855,7 +20855,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:35 AM PT</t>
+          <t>2026-07-12 09:55:35 AM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -20961,7 +20961,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:35 AM PT</t>
+          <t>2026-07-12 09:55:35 AM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21067,7 +21067,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:35 AM PT</t>
+          <t>2026-07-12 09:55:35 AM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21173,7 +21173,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:35 AM PT</t>
+          <t>2026-07-12 09:55:35 AM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21279,7 +21279,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21393,7 +21393,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21507,7 +21507,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21621,7 +21621,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21735,7 +21735,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21849,7 +21849,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -21963,7 +21963,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22077,7 +22077,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22191,7 +22191,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22305,7 +22305,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22411,7 +22411,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22517,7 +22517,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22623,7 +22623,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22729,7 +22729,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -22835,7 +22835,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -22941,7 +22941,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23047,7 +23047,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23153,7 +23153,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23259,7 +23259,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23373,7 +23373,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23487,7 +23487,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23601,7 +23601,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23715,7 +23715,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -23829,7 +23829,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -23943,7 +23943,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24057,7 +24057,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24171,7 +24171,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24285,7 +24285,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24399,7 +24399,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24513,7 +24513,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24627,7 +24627,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -24741,7 +24741,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -24855,7 +24855,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -24969,7 +24969,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25083,7 +25083,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25197,7 +25197,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25311,7 +25311,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25425,7 +25425,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25539,7 +25539,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25653,7 +25653,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -25767,7 +25767,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -25881,7 +25881,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -25995,7 +25995,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26109,7 +26109,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26223,7 +26223,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:34 AM PT</t>
+          <t>2026-07-12 09:55:34 AM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26337,7 +26337,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26451,7 +26451,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26565,7 +26565,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26679,7 +26679,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -26793,7 +26793,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -26907,7 +26907,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27021,7 +27021,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27135,7 +27135,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27249,7 +27249,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-12 09:53:33 AM PT</t>
+          <t>2026-07-12 09:55:33 AM PT</t>
         </is>
       </c>
       <c r="C235" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-12 09:57:36 AM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
@@ -669,7 +669,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -682,7 +682,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Bottom 3 | 0 out</t>
+          <t>Bottom 3 | 1 out</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
@@ -792,7 +792,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -805,7 +805,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Bottom 3 | 0 out</t>
+          <t>Bottom 3 | 1 out</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -817,7 +817,7 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -915,7 +915,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -928,7 +928,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Bottom 3 | 0 out</t>
+          <t>Bottom 3 | 1 out</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -940,7 +940,7 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
@@ -1038,7 +1038,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1051,7 +1051,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Bottom 3 | 0 out</t>
+          <t>Bottom 3 | 1 out</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -1063,7 +1063,7 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1389,7 +1389,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1503,7 +1503,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1617,7 +1617,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1959,7 +1959,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2073,7 +2073,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2301,7 +2301,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2415,7 +2415,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2529,7 +2529,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2643,7 +2643,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2757,7 +2757,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2985,7 +2985,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3099,7 +3099,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3213,7 +3213,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3327,7 +3327,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3441,7 +3441,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3555,7 +3555,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3669,7 +3669,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3783,7 +3783,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3897,7 +3897,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -4011,7 +4011,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4125,7 +4125,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4239,7 +4239,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4353,7 +4353,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4467,7 +4467,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4581,7 +4581,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4695,7 +4695,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4809,7 +4809,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4923,7 +4923,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5037,7 +5037,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5151,7 +5151,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5265,7 +5265,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5379,7 +5379,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5493,7 +5493,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5607,7 +5607,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5721,7 +5721,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5835,7 +5835,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5949,7 +5949,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6063,7 +6063,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6177,7 +6177,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6291,7 +6291,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6405,7 +6405,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6519,7 +6519,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6633,7 +6633,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6747,7 +6747,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6861,7 +6861,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -6975,7 +6975,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7089,7 +7089,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7203,7 +7203,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7317,7 +7317,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7431,7 +7431,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7545,7 +7545,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7659,7 +7659,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7773,7 +7773,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7887,7 +7887,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -8001,7 +8001,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8115,7 +8115,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8229,7 +8229,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8343,7 +8343,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8457,7 +8457,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8571,7 +8571,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8685,7 +8685,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8799,7 +8799,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8913,7 +8913,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9027,7 +9027,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9141,7 +9141,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9255,7 +9255,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9369,7 +9369,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9483,7 +9483,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9597,7 +9597,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9711,7 +9711,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9825,7 +9825,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -9939,7 +9939,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10053,7 +10053,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10167,7 +10167,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10281,7 +10281,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10395,7 +10395,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10509,7 +10509,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10623,7 +10623,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10737,7 +10737,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10851,7 +10851,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -10965,7 +10965,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11079,7 +11079,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11193,7 +11193,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11307,7 +11307,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11421,7 +11421,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11535,7 +11535,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11649,7 +11649,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11763,7 +11763,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11877,7 +11877,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -11991,7 +11991,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12105,7 +12105,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12219,7 +12219,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12333,7 +12333,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12447,7 +12447,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12561,7 +12561,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12675,7 +12675,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12789,7 +12789,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12903,7 +12903,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13017,7 +13017,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13131,7 +13131,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13245,7 +13245,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13359,7 +13359,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13473,7 +13473,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13587,7 +13587,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13701,7 +13701,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13815,7 +13815,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -13929,7 +13929,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14043,7 +14043,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14157,7 +14157,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14271,7 +14271,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14385,7 +14385,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14499,7 +14499,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14512,7 +14512,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Bottom 3 | 0 out</t>
+          <t>Bottom 3 | 1 out</t>
         </is>
       </c>
       <c r="F123" t="n">
@@ -14524,7 +14524,7 @@
         </is>
       </c>
       <c r="H123" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I123" t="n">
         <v>0</v>
@@ -14622,7 +14622,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14635,7 +14635,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Bottom 3 | 0 out</t>
+          <t>Bottom 3 | 1 out</t>
         </is>
       </c>
       <c r="F124" t="n">
@@ -14647,7 +14647,7 @@
         </is>
       </c>
       <c r="H124" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I124" t="n">
         <v>0</v>
@@ -14745,7 +14745,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14758,7 +14758,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Bottom 3 | 0 out</t>
+          <t>Bottom 3 | 1 out</t>
         </is>
       </c>
       <c r="F125" t="n">
@@ -14770,7 +14770,7 @@
         </is>
       </c>
       <c r="H125" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I125" t="n">
         <v>0</v>
@@ -14868,7 +14868,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -14881,7 +14881,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Bottom 3 | 0 out</t>
+          <t>Bottom 3 | 1 out</t>
         </is>
       </c>
       <c r="F126" t="n">
@@ -14893,7 +14893,7 @@
         </is>
       </c>
       <c r="H126" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I126" t="n">
         <v>0</v>
@@ -14991,7 +14991,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15004,7 +15004,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Bottom 3 | 0 out</t>
+          <t>Bottom 3 | 1 out</t>
         </is>
       </c>
       <c r="F127" t="n">
@@ -15016,7 +15016,7 @@
         </is>
       </c>
       <c r="H127" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I127" t="n">
         <v>0</v>
@@ -15114,7 +15114,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15127,7 +15127,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Bottom 3 | 0 out</t>
+          <t>Bottom 3 | 1 out</t>
         </is>
       </c>
       <c r="F128" t="n">
@@ -15139,7 +15139,7 @@
         </is>
       </c>
       <c r="H128" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I128" t="n">
         <v>0</v>
@@ -15237,7 +15237,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15250,7 +15250,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Bottom 3 | 0 out</t>
+          <t>Bottom 3 | 1 out</t>
         </is>
       </c>
       <c r="F129" t="n">
@@ -15262,7 +15262,7 @@
         </is>
       </c>
       <c r="H129" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I129" t="n">
         <v>0</v>
@@ -15360,7 +15360,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15373,7 +15373,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Bottom 3 | 0 out</t>
+          <t>Bottom 3 | 1 out</t>
         </is>
       </c>
       <c r="F130" t="n">
@@ -15385,7 +15385,7 @@
         </is>
       </c>
       <c r="H130" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I130" t="n">
         <v>0</v>
@@ -15483,7 +15483,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15496,7 +15496,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Bottom 3 | 0 out</t>
+          <t>Bottom 3 | 1 out</t>
         </is>
       </c>
       <c r="F131" t="n">
@@ -15508,7 +15508,7 @@
         </is>
       </c>
       <c r="H131" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I131" t="n">
         <v>0</v>
@@ -15606,7 +15606,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15720,7 +15720,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15834,7 +15834,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -15948,7 +15948,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16062,7 +16062,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16176,7 +16176,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16290,7 +16290,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16404,7 +16404,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16518,7 +16518,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16632,7 +16632,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16746,7 +16746,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16860,7 +16860,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -16974,7 +16974,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17088,7 +17088,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17202,7 +17202,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17316,7 +17316,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17430,7 +17430,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17544,7 +17544,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17658,7 +17658,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17772,7 +17772,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17886,7 +17886,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -18000,7 +18000,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18114,7 +18114,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18228,7 +18228,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18342,7 +18342,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18456,7 +18456,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18570,7 +18570,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18684,7 +18684,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18798,7 +18798,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18912,7 +18912,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19026,7 +19026,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19140,7 +19140,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19254,7 +19254,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19368,7 +19368,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19482,7 +19482,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19596,7 +19596,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19710,7 +19710,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19723,7 +19723,7 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>Bottom 3 | 0 out</t>
+          <t>Bottom 3 | 1 out</t>
         </is>
       </c>
       <c r="F168" t="n">
@@ -19735,7 +19735,7 @@
         </is>
       </c>
       <c r="H168" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I168" t="n">
         <v>0</v>
@@ -19833,7 +19833,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -19846,7 +19846,7 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>Bottom 3 | 0 out</t>
+          <t>Bottom 3 | 1 out</t>
         </is>
       </c>
       <c r="F169" t="n">
@@ -19858,7 +19858,7 @@
         </is>
       </c>
       <c r="H169" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I169" t="n">
         <v>0</v>
@@ -19900,10 +19900,10 @@
         </is>
       </c>
       <c r="R169" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S169" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T169" t="n">
         <v>0</v>
@@ -19936,7 +19936,7 @@
         <v>0</v>
       </c>
       <c r="AD169" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AE169" s="4" t="n">
         <v>0</v>
@@ -19956,7 +19956,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -19969,7 +19969,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>Bottom 3 | 0 out</t>
+          <t>Bottom 3 | 1 out</t>
         </is>
       </c>
       <c r="F170" t="n">
@@ -19981,7 +19981,7 @@
         </is>
       </c>
       <c r="H170" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I170" t="n">
         <v>0</v>
@@ -20079,7 +20079,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20092,7 +20092,7 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>Bottom 3 | 0 out</t>
+          <t>Bottom 3 | 1 out</t>
         </is>
       </c>
       <c r="F171" t="n">
@@ -20104,7 +20104,7 @@
         </is>
       </c>
       <c r="H171" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I171" t="n">
         <v>0</v>
@@ -20202,7 +20202,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20215,7 +20215,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>Bottom 3 | 0 out</t>
+          <t>Bottom 3 | 1 out</t>
         </is>
       </c>
       <c r="F172" t="n">
@@ -20227,7 +20227,7 @@
         </is>
       </c>
       <c r="H172" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I172" t="n">
         <v>0</v>
@@ -20325,7 +20325,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:35 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20431,7 +20431,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:35 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20537,7 +20537,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:35 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20643,7 +20643,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:35 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20749,7 +20749,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:35 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20855,7 +20855,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:35 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -20961,7 +20961,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:35 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21067,7 +21067,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:35 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21173,7 +21173,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:35 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21279,7 +21279,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21393,7 +21393,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21507,7 +21507,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21621,7 +21621,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21735,7 +21735,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21849,7 +21849,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -21963,7 +21963,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22077,7 +22077,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22191,7 +22191,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22305,7 +22305,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22411,7 +22411,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22517,7 +22517,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22623,7 +22623,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22729,7 +22729,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -22835,7 +22835,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -22941,7 +22941,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23047,7 +23047,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23153,7 +23153,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23259,7 +23259,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23373,7 +23373,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23487,7 +23487,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23601,7 +23601,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23715,7 +23715,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -23829,7 +23829,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -23943,7 +23943,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24057,7 +24057,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24171,7 +24171,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24285,7 +24285,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24399,7 +24399,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24513,7 +24513,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24627,7 +24627,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -24741,7 +24741,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -24855,7 +24855,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -24969,7 +24969,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25083,7 +25083,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25197,7 +25197,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:34 AM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25311,7 +25311,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25425,7 +25425,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25539,7 +25539,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25653,7 +25653,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -25767,7 +25767,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -25881,7 +25881,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -25995,7 +25995,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26109,7 +26109,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26223,7 +26223,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:34 AM PT</t>
+          <t>2026-07-12 09:57:35 AM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26337,7 +26337,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26451,7 +26451,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26565,7 +26565,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26679,7 +26679,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -26793,7 +26793,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -26907,7 +26907,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27021,7 +27021,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27135,7 +27135,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27249,7 +27249,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-12 09:55:33 AM PT</t>
+          <t>2026-07-12 09:57:33 AM PT</t>
         </is>
       </c>
       <c r="C235" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-12 10:01:36 AM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
@@ -669,7 +669,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -700,7 +700,7 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -792,7 +792,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -823,7 +823,7 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -915,7 +915,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -946,7 +946,7 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -1038,7 +1038,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1069,7 +1069,7 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1192,7 +1192,7 @@
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -1284,7 +1284,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1398,7 +1398,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1512,7 +1512,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1626,7 +1626,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1740,7 +1740,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1968,7 +1968,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2082,7 +2082,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2196,7 +2196,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2310,7 +2310,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2424,7 +2424,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2538,7 +2538,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2652,7 +2652,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2766,7 +2766,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2880,7 +2880,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2994,7 +2994,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3108,7 +3108,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3222,7 +3222,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3336,7 +3336,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3450,7 +3450,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3564,7 +3564,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3678,7 +3678,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3906,7 +3906,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -4020,7 +4020,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4134,7 +4134,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4248,7 +4248,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4362,7 +4362,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4476,7 +4476,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4590,7 +4590,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4704,7 +4704,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4818,7 +4818,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4932,7 +4932,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5046,7 +5046,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5160,7 +5160,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5274,7 +5274,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5388,7 +5388,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5502,7 +5502,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5616,7 +5616,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5730,7 +5730,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5844,7 +5844,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5958,7 +5958,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6072,7 +6072,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6186,7 +6186,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6300,7 +6300,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6414,7 +6414,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6528,7 +6528,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6642,7 +6642,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6756,7 +6756,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6870,7 +6870,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -6984,7 +6984,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7098,7 +7098,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7212,7 +7212,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7326,7 +7326,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7440,7 +7440,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7554,7 +7554,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7668,7 +7668,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7782,7 +7782,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7896,7 +7896,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -8010,7 +8010,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8124,7 +8124,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8238,7 +8238,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8352,7 +8352,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8466,7 +8466,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8580,7 +8580,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8694,7 +8694,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8808,7 +8808,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8922,7 +8922,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9036,7 +9036,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9150,7 +9150,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9378,7 +9378,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9492,7 +9492,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9606,7 +9606,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9720,7 +9720,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9834,7 +9834,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -9948,7 +9948,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10062,7 +10062,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10176,7 +10176,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10290,7 +10290,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10404,7 +10404,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10518,7 +10518,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10632,7 +10632,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10746,7 +10746,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10860,7 +10860,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -10974,7 +10974,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11088,7 +11088,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11202,7 +11202,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11316,7 +11316,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11430,7 +11430,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11544,7 +11544,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11658,7 +11658,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11772,7 +11772,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11886,7 +11886,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -12000,7 +12000,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12114,7 +12114,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12228,7 +12228,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12342,7 +12342,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12456,7 +12456,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12570,7 +12570,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12684,7 +12684,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12798,7 +12798,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12912,7 +12912,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13026,7 +13026,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13140,7 +13140,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13254,7 +13254,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13368,7 +13368,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13482,7 +13482,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13596,7 +13596,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13710,7 +13710,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13824,7 +13824,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -13938,7 +13938,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14052,7 +14052,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14166,7 +14166,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14280,7 +14280,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14394,7 +14394,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14508,7 +14508,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14622,7 +14622,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14653,7 +14653,7 @@
         <v>0</v>
       </c>
       <c r="J124" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K124" t="inlineStr">
         <is>
@@ -14745,7 +14745,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14776,7 +14776,7 @@
         <v>0</v>
       </c>
       <c r="J125" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K125" t="inlineStr">
         <is>
@@ -14868,7 +14868,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -14899,7 +14899,7 @@
         <v>0</v>
       </c>
       <c r="J126" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K126" t="inlineStr">
         <is>
@@ -14991,7 +14991,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15022,7 +15022,7 @@
         <v>0</v>
       </c>
       <c r="J127" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K127" t="inlineStr">
         <is>
@@ -15114,7 +15114,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15145,7 +15145,7 @@
         <v>0</v>
       </c>
       <c r="J128" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K128" t="inlineStr">
         <is>
@@ -15237,7 +15237,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15268,7 +15268,7 @@
         <v>0</v>
       </c>
       <c r="J129" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K129" t="inlineStr">
         <is>
@@ -15360,7 +15360,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15391,7 +15391,7 @@
         <v>0</v>
       </c>
       <c r="J130" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K130" t="inlineStr">
         <is>
@@ -15483,7 +15483,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15514,7 +15514,7 @@
         <v>0</v>
       </c>
       <c r="J131" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K131" t="inlineStr">
         <is>
@@ -15606,7 +15606,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15637,7 +15637,7 @@
         <v>0</v>
       </c>
       <c r="J132" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K132" t="inlineStr">
         <is>
@@ -15729,7 +15729,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15843,7 +15843,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -15957,7 +15957,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16071,7 +16071,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16185,7 +16185,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16299,7 +16299,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16413,7 +16413,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16527,7 +16527,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16641,7 +16641,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16755,7 +16755,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16869,7 +16869,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -16983,7 +16983,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17097,7 +17097,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17211,7 +17211,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17325,7 +17325,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17439,7 +17439,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17553,7 +17553,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17667,7 +17667,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17781,7 +17781,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17895,7 +17895,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -18009,7 +18009,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18123,7 +18123,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18237,7 +18237,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18351,7 +18351,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18465,7 +18465,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18579,7 +18579,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18693,7 +18693,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18807,7 +18807,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18921,7 +18921,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19035,7 +19035,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19149,7 +19149,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19263,7 +19263,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19377,7 +19377,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19491,7 +19491,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19605,7 +19605,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19719,7 +19719,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19833,7 +19833,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -19864,7 +19864,7 @@
         <v>0</v>
       </c>
       <c r="J169" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K169" t="inlineStr">
         <is>
@@ -19956,7 +19956,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -19987,7 +19987,7 @@
         <v>0</v>
       </c>
       <c r="J170" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K170" t="inlineStr">
         <is>
@@ -20079,7 +20079,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20110,7 +20110,7 @@
         <v>0</v>
       </c>
       <c r="J171" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K171" t="inlineStr">
         <is>
@@ -20202,7 +20202,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20233,7 +20233,7 @@
         <v>0</v>
       </c>
       <c r="J172" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K172" t="inlineStr">
         <is>
@@ -20325,7 +20325,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:35 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20431,7 +20431,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:35 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20537,7 +20537,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:35 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20643,7 +20643,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:35 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20749,7 +20749,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:35 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20855,7 +20855,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:35 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -20961,7 +20961,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:35 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21067,7 +21067,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:35 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21173,7 +21173,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:35 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21279,7 +21279,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21393,7 +21393,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21507,7 +21507,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21621,7 +21621,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21735,7 +21735,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21849,7 +21849,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -21963,7 +21963,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22077,7 +22077,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22191,7 +22191,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22305,7 +22305,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22411,7 +22411,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22517,7 +22517,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22623,7 +22623,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22729,7 +22729,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -22835,7 +22835,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -22941,7 +22941,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23047,7 +23047,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23153,7 +23153,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23259,7 +23259,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23373,7 +23373,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23487,7 +23487,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23601,7 +23601,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23715,7 +23715,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -23829,7 +23829,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -23943,7 +23943,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24057,7 +24057,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24171,7 +24171,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24285,7 +24285,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24399,7 +24399,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24513,7 +24513,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24627,7 +24627,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -24741,7 +24741,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -24855,7 +24855,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -24969,7 +24969,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25083,7 +25083,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25197,7 +25197,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25311,7 +25311,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25425,7 +25425,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25539,7 +25539,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25653,7 +25653,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -25767,7 +25767,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -25881,7 +25881,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -25995,7 +25995,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26109,7 +26109,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26223,7 +26223,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:34 AM PT</t>
+          <t>2026-07-12 10:01:34 AM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26337,7 +26337,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26451,7 +26451,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26565,7 +26565,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26679,7 +26679,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -26793,7 +26793,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -26907,7 +26907,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27021,7 +27021,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27135,7 +27135,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27249,7 +27249,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-12 09:59:33 AM PT</t>
+          <t>2026-07-12 10:01:33 AM PT</t>
         </is>
       </c>
       <c r="C235" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-12 10:03:36 AM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
@@ -36,7 +36,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -58,6 +58,11 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE5CD"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -77,7 +82,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -88,6 +93,7 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -669,7 +675,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -697,10 +703,10 @@
         <v>2</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -792,7 +798,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -820,10 +826,10 @@
         <v>2</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -859,7 +865,7 @@
         </is>
       </c>
       <c r="R3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S3" t="n">
         <v>1</v>
@@ -888,8 +894,8 @@
       <c r="AA3" t="n">
         <v>0</v>
       </c>
-      <c r="AB3" t="n">
-        <v>0</v>
+      <c r="AB3" s="6" t="n">
+        <v>1</v>
       </c>
       <c r="AC3" t="n">
         <v>0</v>
@@ -898,7 +904,7 @@
         <v>0</v>
       </c>
       <c r="AE3" s="4" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="AF3" t="n">
         <v>4</v>
@@ -915,7 +921,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -943,10 +949,10 @@
         <v>2</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -1038,7 +1044,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1066,10 +1072,10 @@
         <v>2</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -1161,7 +1167,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1189,10 +1195,10 @@
         <v>2</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -1284,7 +1290,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1398,7 +1404,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1512,7 +1518,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1626,7 +1632,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1740,7 +1746,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1854,7 +1860,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1968,7 +1974,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2082,7 +2088,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2196,7 +2202,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2310,7 +2316,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2424,7 +2430,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2538,7 +2544,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2652,7 +2658,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2766,7 +2772,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2880,7 +2886,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2994,7 +3000,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3108,7 +3114,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3222,7 +3228,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3336,7 +3342,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3450,7 +3456,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3564,7 +3570,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3678,7 +3684,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3792,7 +3798,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3906,7 +3912,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -4020,7 +4026,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4134,7 +4140,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4248,7 +4254,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4362,7 +4368,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4476,7 +4482,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4590,7 +4596,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4704,7 +4710,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4818,7 +4824,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4932,7 +4938,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5046,7 +5052,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5160,7 +5166,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5274,7 +5280,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5388,7 +5394,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5502,7 +5508,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5616,7 +5622,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5730,7 +5736,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5844,7 +5850,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5958,7 +5964,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6072,7 +6078,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6186,7 +6192,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6300,7 +6306,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6414,7 +6420,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6528,7 +6534,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6642,7 +6648,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6756,7 +6762,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6870,7 +6876,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -6984,7 +6990,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7098,7 +7104,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7212,7 +7218,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7326,7 +7332,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7440,7 +7446,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7554,7 +7560,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7668,7 +7674,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7782,7 +7788,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7896,7 +7902,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -8010,7 +8016,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8124,7 +8130,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8238,7 +8244,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8352,7 +8358,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8466,7 +8472,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8580,7 +8586,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8694,7 +8700,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8808,7 +8814,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8922,7 +8928,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9036,7 +9042,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9150,7 +9156,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9264,7 +9270,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9378,7 +9384,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9492,7 +9498,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9606,7 +9612,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9720,7 +9726,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9834,7 +9840,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -9948,7 +9954,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10062,7 +10068,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10176,7 +10182,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10290,7 +10296,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10404,7 +10410,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10518,7 +10524,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10632,7 +10638,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10746,7 +10752,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10860,7 +10866,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -10974,7 +10980,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11088,7 +11094,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11202,7 +11208,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11316,7 +11322,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11430,7 +11436,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11544,7 +11550,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11658,7 +11664,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11772,7 +11778,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11886,7 +11892,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -12000,7 +12006,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12114,7 +12120,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12228,7 +12234,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12342,7 +12348,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12456,7 +12462,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12570,7 +12576,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12684,7 +12690,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12798,7 +12804,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12912,7 +12918,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13026,7 +13032,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13140,7 +13146,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13254,7 +13260,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13368,7 +13374,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13482,7 +13488,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13596,7 +13602,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13710,7 +13716,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13824,7 +13830,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -13938,7 +13944,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14052,7 +14058,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14166,7 +14172,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14280,7 +14286,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14394,7 +14400,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14508,7 +14514,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14622,7 +14628,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14650,10 +14656,10 @@
         <v>2</v>
       </c>
       <c r="I124" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J124" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K124" t="inlineStr">
         <is>
@@ -14745,7 +14751,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14773,10 +14779,10 @@
         <v>2</v>
       </c>
       <c r="I125" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J125" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K125" t="inlineStr">
         <is>
@@ -14868,7 +14874,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -14896,10 +14902,10 @@
         <v>2</v>
       </c>
       <c r="I126" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J126" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K126" t="inlineStr">
         <is>
@@ -14991,7 +14997,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15019,10 +15025,10 @@
         <v>2</v>
       </c>
       <c r="I127" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J127" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K127" t="inlineStr">
         <is>
@@ -15114,7 +15120,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15142,10 +15148,10 @@
         <v>2</v>
       </c>
       <c r="I128" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J128" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K128" t="inlineStr">
         <is>
@@ -15237,7 +15243,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15265,10 +15271,10 @@
         <v>2</v>
       </c>
       <c r="I129" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J129" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K129" t="inlineStr">
         <is>
@@ -15360,7 +15366,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15388,10 +15394,10 @@
         <v>2</v>
       </c>
       <c r="I130" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J130" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K130" t="inlineStr">
         <is>
@@ -15483,7 +15489,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15511,10 +15517,10 @@
         <v>2</v>
       </c>
       <c r="I131" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J131" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K131" t="inlineStr">
         <is>
@@ -15606,7 +15612,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15634,10 +15640,10 @@
         <v>2</v>
       </c>
       <c r="I132" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J132" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K132" t="inlineStr">
         <is>
@@ -15729,7 +15735,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15843,7 +15849,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -15957,7 +15963,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16071,7 +16077,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16185,7 +16191,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16299,7 +16305,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16413,7 +16419,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16527,7 +16533,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16641,7 +16647,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16755,7 +16761,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16869,7 +16875,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -16983,7 +16989,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17097,7 +17103,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17211,7 +17217,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17325,7 +17331,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17439,7 +17445,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17553,7 +17559,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17667,7 +17673,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17781,7 +17787,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17895,7 +17901,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -18009,7 +18015,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18123,7 +18129,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18237,7 +18243,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18351,7 +18357,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18465,7 +18471,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18579,7 +18585,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18693,7 +18699,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18807,7 +18813,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18921,7 +18927,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19035,7 +19041,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19149,7 +19155,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19263,7 +19269,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19377,7 +19383,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19491,7 +19497,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19605,7 +19611,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19719,7 +19725,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19833,7 +19839,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -19861,10 +19867,10 @@
         <v>2</v>
       </c>
       <c r="I169" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J169" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K169" t="inlineStr">
         <is>
@@ -19956,7 +19962,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -19984,10 +19990,10 @@
         <v>2</v>
       </c>
       <c r="I170" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J170" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K170" t="inlineStr">
         <is>
@@ -20079,7 +20085,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20107,10 +20113,10 @@
         <v>2</v>
       </c>
       <c r="I171" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J171" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K171" t="inlineStr">
         <is>
@@ -20202,7 +20208,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20230,10 +20236,10 @@
         <v>2</v>
       </c>
       <c r="I172" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J172" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K172" t="inlineStr">
         <is>
@@ -20325,7 +20331,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:35 AM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20431,7 +20437,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:35 AM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20537,7 +20543,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:35 AM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20643,7 +20649,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:35 AM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20749,7 +20755,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:35 AM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20855,7 +20861,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:35 AM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -20961,7 +20967,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:35 AM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21067,7 +21073,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:35 AM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21173,7 +21179,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:35 AM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21279,7 +21285,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21393,7 +21399,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21507,7 +21513,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21621,7 +21627,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21735,7 +21741,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21849,7 +21855,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -21963,7 +21969,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22077,7 +22083,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22191,7 +22197,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22305,7 +22311,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22411,7 +22417,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22517,7 +22523,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22623,7 +22629,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22729,7 +22735,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -22835,7 +22841,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -22941,7 +22947,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23047,7 +23053,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23153,7 +23159,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23259,7 +23265,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23373,7 +23379,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23487,7 +23493,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23601,7 +23607,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23715,7 +23721,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -23829,7 +23835,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -23943,7 +23949,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24057,7 +24063,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24171,7 +24177,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24285,7 +24291,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24399,7 +24405,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24513,7 +24519,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24627,7 +24633,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -24741,7 +24747,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -24855,7 +24861,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -24969,7 +24975,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25083,7 +25089,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25197,7 +25203,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25311,7 +25317,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25425,7 +25431,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25539,7 +25545,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25653,7 +25659,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -25767,7 +25773,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -25881,7 +25887,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -25995,7 +26001,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26109,7 +26115,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26223,7 +26229,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:34 AM PT</t>
+          <t>2026-07-12 10:03:34 AM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26337,7 +26343,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26451,7 +26457,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26565,7 +26571,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26679,7 +26685,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -26793,7 +26799,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -26907,7 +26913,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27021,7 +27027,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27135,7 +27141,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27249,7 +27255,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-12 10:01:33 AM PT</t>
+          <t>2026-07-12 10:03:33 AM PT</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -27387,12 +27393,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Stat Type</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>Points</t>
         </is>

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-12 10:05:36 AM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
@@ -675,7 +675,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -688,7 +688,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Bottom 3 | 2 out</t>
+          <t>Bottom 3 | 3 out</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -700,7 +700,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I2" t="n">
         <v>2</v>
@@ -798,7 +798,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -811,7 +811,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Bottom 3 | 2 out</t>
+          <t>Bottom 3 | 3 out</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -823,7 +823,7 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I3" t="n">
         <v>2</v>
@@ -921,7 +921,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -934,7 +934,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Bottom 3 | 2 out</t>
+          <t>Bottom 3 | 3 out</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -946,7 +946,7 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I4" t="n">
         <v>2</v>
@@ -1044,7 +1044,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Bottom 3 | 2 out</t>
+          <t>Bottom 3 | 3 out</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -1069,7 +1069,7 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I5" t="n">
         <v>2</v>
@@ -1167,7 +1167,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1180,7 +1180,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Bottom 3 | 2 out</t>
+          <t>Bottom 3 | 3 out</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -1192,7 +1192,7 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I6" t="n">
         <v>2</v>
@@ -1290,7 +1290,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1404,7 +1404,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1518,7 +1518,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1632,7 +1632,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1746,7 +1746,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1860,7 +1860,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1974,7 +1974,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2088,7 +2088,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2202,7 +2202,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2316,7 +2316,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2430,7 +2430,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2658,7 +2658,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2772,7 +2772,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2886,7 +2886,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -3000,7 +3000,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3114,7 +3114,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3228,7 +3228,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3342,7 +3342,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3456,7 +3456,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3570,7 +3570,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3684,7 +3684,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3798,7 +3798,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3912,7 +3912,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -4026,7 +4026,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4140,7 +4140,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4254,7 +4254,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4368,7 +4368,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4482,7 +4482,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4596,7 +4596,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4710,7 +4710,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4824,7 +4824,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4938,7 +4938,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5052,7 +5052,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5166,7 +5166,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5280,7 +5280,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5394,7 +5394,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5508,7 +5508,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5622,7 +5622,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5736,7 +5736,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5850,7 +5850,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5964,7 +5964,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6078,7 +6078,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6192,7 +6192,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6306,7 +6306,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6420,7 +6420,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6534,7 +6534,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6648,7 +6648,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6762,7 +6762,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6876,7 +6876,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -6990,7 +6990,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7104,7 +7104,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7218,7 +7218,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7332,7 +7332,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7446,7 +7446,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7560,7 +7560,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7674,7 +7674,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7788,7 +7788,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7902,7 +7902,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -8016,7 +8016,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8130,7 +8130,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8244,7 +8244,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8358,7 +8358,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8472,7 +8472,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8586,7 +8586,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8700,7 +8700,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8928,7 +8928,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9042,7 +9042,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9156,7 +9156,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9270,7 +9270,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9384,7 +9384,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9498,7 +9498,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9612,7 +9612,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9726,7 +9726,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9840,7 +9840,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -9954,7 +9954,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10068,7 +10068,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10182,7 +10182,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10296,7 +10296,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10410,7 +10410,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10524,7 +10524,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10638,7 +10638,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10752,7 +10752,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10866,7 +10866,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -10980,7 +10980,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11094,7 +11094,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11208,7 +11208,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11322,7 +11322,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11436,7 +11436,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11550,7 +11550,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11664,7 +11664,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11778,7 +11778,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11892,7 +11892,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -12006,7 +12006,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12120,7 +12120,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12234,7 +12234,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12348,7 +12348,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12462,7 +12462,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12576,7 +12576,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12690,7 +12690,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12804,7 +12804,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12918,7 +12918,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13032,7 +13032,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13146,7 +13146,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13260,7 +13260,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13374,7 +13374,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13488,7 +13488,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13602,7 +13602,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13716,7 +13716,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13830,7 +13830,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -13944,7 +13944,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14058,7 +14058,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14172,7 +14172,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14286,7 +14286,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14400,7 +14400,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14514,7 +14514,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14628,7 +14628,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14641,7 +14641,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Bottom 3 | 2 out</t>
+          <t>Bottom 3 | 3 out</t>
         </is>
       </c>
       <c r="F124" t="n">
@@ -14653,7 +14653,7 @@
         </is>
       </c>
       <c r="H124" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I124" t="n">
         <v>2</v>
@@ -14751,7 +14751,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14764,7 +14764,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Bottom 3 | 2 out</t>
+          <t>Bottom 3 | 3 out</t>
         </is>
       </c>
       <c r="F125" t="n">
@@ -14776,7 +14776,7 @@
         </is>
       </c>
       <c r="H125" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I125" t="n">
         <v>2</v>
@@ -14874,7 +14874,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -14887,7 +14887,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Bottom 3 | 2 out</t>
+          <t>Bottom 3 | 3 out</t>
         </is>
       </c>
       <c r="F126" t="n">
@@ -14899,7 +14899,7 @@
         </is>
       </c>
       <c r="H126" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I126" t="n">
         <v>2</v>
@@ -14997,7 +14997,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15010,7 +15010,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Bottom 3 | 2 out</t>
+          <t>Bottom 3 | 3 out</t>
         </is>
       </c>
       <c r="F127" t="n">
@@ -15022,7 +15022,7 @@
         </is>
       </c>
       <c r="H127" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I127" t="n">
         <v>2</v>
@@ -15120,7 +15120,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15133,7 +15133,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Bottom 3 | 2 out</t>
+          <t>Bottom 3 | 3 out</t>
         </is>
       </c>
       <c r="F128" t="n">
@@ -15145,7 +15145,7 @@
         </is>
       </c>
       <c r="H128" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I128" t="n">
         <v>2</v>
@@ -15243,7 +15243,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15256,7 +15256,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Bottom 3 | 2 out</t>
+          <t>Bottom 3 | 3 out</t>
         </is>
       </c>
       <c r="F129" t="n">
@@ -15268,7 +15268,7 @@
         </is>
       </c>
       <c r="H129" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I129" t="n">
         <v>2</v>
@@ -15366,7 +15366,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15379,7 +15379,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Bottom 3 | 2 out</t>
+          <t>Bottom 3 | 3 out</t>
         </is>
       </c>
       <c r="F130" t="n">
@@ -15391,7 +15391,7 @@
         </is>
       </c>
       <c r="H130" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I130" t="n">
         <v>2</v>
@@ -15489,7 +15489,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15502,7 +15502,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Bottom 3 | 2 out</t>
+          <t>Bottom 3 | 3 out</t>
         </is>
       </c>
       <c r="F131" t="n">
@@ -15514,7 +15514,7 @@
         </is>
       </c>
       <c r="H131" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I131" t="n">
         <v>2</v>
@@ -15612,7 +15612,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15625,7 +15625,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Bottom 3 | 2 out</t>
+          <t>Bottom 3 | 3 out</t>
         </is>
       </c>
       <c r="F132" t="n">
@@ -15637,7 +15637,7 @@
         </is>
       </c>
       <c r="H132" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I132" t="n">
         <v>2</v>
@@ -15735,7 +15735,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15849,7 +15849,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -15963,7 +15963,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16077,7 +16077,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16191,7 +16191,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16305,7 +16305,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16419,7 +16419,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16533,7 +16533,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16647,7 +16647,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16761,7 +16761,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16875,7 +16875,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -16989,7 +16989,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17103,7 +17103,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17217,7 +17217,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17331,7 +17331,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17445,7 +17445,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17559,7 +17559,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17673,7 +17673,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17787,7 +17787,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17901,7 +17901,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -18015,7 +18015,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18129,7 +18129,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18243,7 +18243,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18357,7 +18357,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18471,7 +18471,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18585,7 +18585,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18699,7 +18699,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18813,7 +18813,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18927,7 +18927,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19041,7 +19041,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19155,7 +19155,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19269,7 +19269,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19383,7 +19383,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19497,7 +19497,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19611,7 +19611,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19725,7 +19725,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19839,7 +19839,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -19852,7 +19852,7 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>Bottom 3 | 2 out</t>
+          <t>Bottom 3 | 3 out</t>
         </is>
       </c>
       <c r="F169" t="n">
@@ -19864,7 +19864,7 @@
         </is>
       </c>
       <c r="H169" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I169" t="n">
         <v>2</v>
@@ -19962,7 +19962,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -19975,7 +19975,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>Bottom 3 | 2 out</t>
+          <t>Bottom 3 | 3 out</t>
         </is>
       </c>
       <c r="F170" t="n">
@@ -19987,7 +19987,7 @@
         </is>
       </c>
       <c r="H170" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I170" t="n">
         <v>2</v>
@@ -20085,7 +20085,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20098,7 +20098,7 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>Bottom 3 | 2 out</t>
+          <t>Bottom 3 | 3 out</t>
         </is>
       </c>
       <c r="F171" t="n">
@@ -20110,7 +20110,7 @@
         </is>
       </c>
       <c r="H171" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I171" t="n">
         <v>2</v>
@@ -20152,10 +20152,10 @@
         </is>
       </c>
       <c r="R171" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S171" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T171" t="n">
         <v>0</v>
@@ -20208,7 +20208,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20221,7 +20221,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>Bottom 3 | 2 out</t>
+          <t>Bottom 3 | 3 out</t>
         </is>
       </c>
       <c r="F172" t="n">
@@ -20233,7 +20233,7 @@
         </is>
       </c>
       <c r="H172" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I172" t="n">
         <v>2</v>
@@ -20331,7 +20331,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:35 AM PT</t>
+          <t>2026-07-12 10:05:35 AM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20437,7 +20437,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:35 AM PT</t>
+          <t>2026-07-12 10:05:35 AM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20543,7 +20543,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:35 AM PT</t>
+          <t>2026-07-12 10:05:35 AM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20649,7 +20649,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:35 AM PT</t>
+          <t>2026-07-12 10:05:35 AM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20755,7 +20755,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:35 AM PT</t>
+          <t>2026-07-12 10:05:35 AM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20861,7 +20861,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:35 AM PT</t>
+          <t>2026-07-12 10:05:35 AM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -20967,7 +20967,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:35 AM PT</t>
+          <t>2026-07-12 10:05:35 AM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21073,7 +21073,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:35 AM PT</t>
+          <t>2026-07-12 10:05:35 AM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21179,7 +21179,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:35 AM PT</t>
+          <t>2026-07-12 10:05:35 AM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21285,7 +21285,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21399,7 +21399,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21513,7 +21513,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21627,7 +21627,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21741,7 +21741,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21855,7 +21855,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -21969,7 +21969,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22083,7 +22083,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22197,7 +22197,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22311,7 +22311,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22417,7 +22417,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22523,7 +22523,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22629,7 +22629,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22735,7 +22735,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -22841,7 +22841,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -22947,7 +22947,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23053,7 +23053,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23159,7 +23159,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23265,7 +23265,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23379,7 +23379,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23493,7 +23493,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23607,7 +23607,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23721,7 +23721,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -23835,7 +23835,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -23949,7 +23949,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24063,7 +24063,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24177,7 +24177,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24291,7 +24291,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24405,7 +24405,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24519,7 +24519,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24633,7 +24633,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -24747,7 +24747,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -24861,7 +24861,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -24975,7 +24975,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25089,7 +25089,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25203,7 +25203,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25317,7 +25317,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25431,7 +25431,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25545,7 +25545,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25659,7 +25659,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -25773,7 +25773,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -25887,7 +25887,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26001,7 +26001,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26115,7 +26115,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26229,7 +26229,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:34 AM PT</t>
+          <t>2026-07-12 10:05:34 AM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26343,7 +26343,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26457,7 +26457,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26571,7 +26571,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26685,7 +26685,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -26799,7 +26799,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -26913,7 +26913,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27027,7 +27027,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27141,7 +27141,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27255,7 +27255,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-12 10:03:33 AM PT</t>
+          <t>2026-07-12 10:05:33 AM PT</t>
         </is>
       </c>
       <c r="C235" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-12 10:17:09 AM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
@@ -475,7 +475,7 @@
     <col width="27" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
@@ -681,7 +681,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -694,7 +694,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Top 4 | 2 out</t>
+          <t>Bottom 4 | 0 out</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -702,11 +702,11 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
@@ -804,7 +804,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -817,7 +817,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Top 4 | 2 out</t>
+          <t>Bottom 4 | 0 out</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -825,11 +825,11 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -927,7 +927,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -940,7 +940,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Top 4 | 2 out</t>
+          <t>Bottom 4 | 0 out</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -948,11 +948,11 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
@@ -1050,7 +1050,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1063,7 +1063,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Top 4 | 2 out</t>
+          <t>Bottom 4 | 0 out</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -1071,11 +1071,11 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -1173,7 +1173,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1186,7 +1186,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Top 4 | 2 out</t>
+          <t>Bottom 4 | 0 out</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -1194,11 +1194,11 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
@@ -1296,7 +1296,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1309,7 +1309,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Top 4 | 2 out</t>
+          <t>Bottom 4 | 0 out</t>
         </is>
       </c>
       <c r="F7" t="n">
@@ -1317,11 +1317,11 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
@@ -1419,7 +1419,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1432,7 +1432,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Top 4 | 2 out</t>
+          <t>Bottom 4 | 0 out</t>
         </is>
       </c>
       <c r="F8" t="n">
@@ -1440,11 +1440,11 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
@@ -1542,7 +1542,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1555,7 +1555,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Top 4 | 2 out</t>
+          <t>Bottom 4 | 0 out</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -1563,11 +1563,11 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
@@ -1665,7 +1665,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1678,7 +1678,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Top 4 | 2 out</t>
+          <t>Bottom 4 | 0 out</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -1686,11 +1686,11 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
@@ -1788,7 +1788,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1902,7 +1902,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -2016,7 +2016,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2130,7 +2130,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2244,7 +2244,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2472,7 +2472,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2586,7 +2586,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2700,7 +2700,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2814,7 +2814,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -3042,7 +3042,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3156,7 +3156,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3270,7 +3270,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3384,7 +3384,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3498,7 +3498,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3612,7 +3612,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3726,7 +3726,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3840,7 +3840,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3963,7 +3963,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -4086,7 +4086,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4209,7 +4209,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4332,7 +4332,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4455,7 +4455,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4578,7 +4578,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4701,7 +4701,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4824,7 +4824,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4947,7 +4947,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -5070,7 +5070,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5193,7 +5193,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5316,7 +5316,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5439,7 +5439,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5562,7 +5562,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5685,7 +5685,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5808,7 +5808,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5931,7 +5931,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -6054,7 +6054,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -6168,7 +6168,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6282,7 +6282,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6396,7 +6396,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6510,7 +6510,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6624,7 +6624,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6738,7 +6738,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6852,7 +6852,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6966,7 +6966,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -7080,7 +7080,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -7194,7 +7194,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7308,7 +7308,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7422,7 +7422,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7536,7 +7536,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7650,7 +7650,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7764,7 +7764,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7878,7 +7878,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7992,7 +7992,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -8106,7 +8106,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -8119,7 +8119,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Top 1 | 0 out</t>
         </is>
       </c>
       <c r="F65" t="n">
@@ -8129,6 +8129,15 @@
         <is>
           <t>Top</t>
         </is>
+      </c>
+      <c r="H65" t="n">
+        <v>0</v>
+      </c>
+      <c r="I65" t="n">
+        <v>0</v>
+      </c>
+      <c r="J65" t="n">
+        <v>0</v>
       </c>
       <c r="K65" t="inlineStr">
         <is>
@@ -8220,7 +8229,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8233,7 +8242,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Top 1 | 0 out</t>
         </is>
       </c>
       <c r="F66" t="n">
@@ -8243,6 +8252,15 @@
         <is>
           <t>Top</t>
         </is>
+      </c>
+      <c r="H66" t="n">
+        <v>0</v>
+      </c>
+      <c r="I66" t="n">
+        <v>0</v>
+      </c>
+      <c r="J66" t="n">
+        <v>0</v>
       </c>
       <c r="K66" t="inlineStr">
         <is>
@@ -8334,7 +8352,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8347,7 +8365,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Top 1 | 0 out</t>
         </is>
       </c>
       <c r="F67" t="n">
@@ -8357,6 +8375,15 @@
         <is>
           <t>Top</t>
         </is>
+      </c>
+      <c r="H67" t="n">
+        <v>0</v>
+      </c>
+      <c r="I67" t="n">
+        <v>0</v>
+      </c>
+      <c r="J67" t="n">
+        <v>0</v>
       </c>
       <c r="K67" t="inlineStr">
         <is>
@@ -8448,7 +8475,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8461,7 +8488,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Top 1 | 0 out</t>
         </is>
       </c>
       <c r="F68" t="n">
@@ -8471,6 +8498,15 @@
         <is>
           <t>Top</t>
         </is>
+      </c>
+      <c r="H68" t="n">
+        <v>0</v>
+      </c>
+      <c r="I68" t="n">
+        <v>0</v>
+      </c>
+      <c r="J68" t="n">
+        <v>0</v>
       </c>
       <c r="K68" t="inlineStr">
         <is>
@@ -8562,7 +8598,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8575,7 +8611,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Top 1 | 0 out</t>
         </is>
       </c>
       <c r="F69" t="n">
@@ -8585,6 +8621,15 @@
         <is>
           <t>Top</t>
         </is>
+      </c>
+      <c r="H69" t="n">
+        <v>0</v>
+      </c>
+      <c r="I69" t="n">
+        <v>0</v>
+      </c>
+      <c r="J69" t="n">
+        <v>0</v>
       </c>
       <c r="K69" t="inlineStr">
         <is>
@@ -8676,7 +8721,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8689,7 +8734,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Top 1 | 0 out</t>
         </is>
       </c>
       <c r="F70" t="n">
@@ -8699,6 +8744,15 @@
         <is>
           <t>Top</t>
         </is>
+      </c>
+      <c r="H70" t="n">
+        <v>0</v>
+      </c>
+      <c r="I70" t="n">
+        <v>0</v>
+      </c>
+      <c r="J70" t="n">
+        <v>0</v>
       </c>
       <c r="K70" t="inlineStr">
         <is>
@@ -8790,7 +8844,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8803,7 +8857,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Top 1 | 0 out</t>
         </is>
       </c>
       <c r="F71" t="n">
@@ -8813,6 +8867,15 @@
         <is>
           <t>Top</t>
         </is>
+      </c>
+      <c r="H71" t="n">
+        <v>0</v>
+      </c>
+      <c r="I71" t="n">
+        <v>0</v>
+      </c>
+      <c r="J71" t="n">
+        <v>0</v>
       </c>
       <c r="K71" t="inlineStr">
         <is>
@@ -8904,7 +8967,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8917,7 +8980,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Top 1 | 0 out</t>
         </is>
       </c>
       <c r="F72" t="n">
@@ -8927,6 +8990,15 @@
         <is>
           <t>Top</t>
         </is>
+      </c>
+      <c r="H72" t="n">
+        <v>0</v>
+      </c>
+      <c r="I72" t="n">
+        <v>0</v>
+      </c>
+      <c r="J72" t="n">
+        <v>0</v>
       </c>
       <c r="K72" t="inlineStr">
         <is>
@@ -9018,7 +9090,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -9031,7 +9103,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Top 1 | 0 out</t>
         </is>
       </c>
       <c r="F73" t="n">
@@ -9041,6 +9113,15 @@
         <is>
           <t>Top</t>
         </is>
+      </c>
+      <c r="H73" t="n">
+        <v>0</v>
+      </c>
+      <c r="I73" t="n">
+        <v>0</v>
+      </c>
+      <c r="J73" t="n">
+        <v>0</v>
       </c>
       <c r="K73" t="inlineStr">
         <is>
@@ -9132,7 +9213,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9246,7 +9327,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9360,7 +9441,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9474,7 +9555,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9588,7 +9669,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9702,7 +9783,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9816,7 +9897,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9930,7 +10011,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -10044,7 +10125,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -10158,7 +10239,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10272,7 +10353,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10386,7 +10467,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10500,7 +10581,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10614,7 +10695,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10728,7 +10809,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10842,7 +10923,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10956,7 +11037,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -11070,7 +11151,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -11184,7 +11265,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11298,7 +11379,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11412,7 +11493,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11526,7 +11607,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11640,7 +11721,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11754,7 +11835,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11868,7 +11949,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11982,7 +12063,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -12096,7 +12177,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -12210,7 +12291,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12324,7 +12405,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12438,7 +12519,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12552,7 +12633,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12666,7 +12747,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12780,7 +12861,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12894,7 +12975,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -13008,7 +13089,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -13122,7 +13203,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13236,7 +13317,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13359,7 +13440,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13482,7 +13563,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13605,7 +13686,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13728,7 +13809,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13851,7 +13932,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13974,7 +14055,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -14097,7 +14178,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -14220,7 +14301,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14343,7 +14424,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14457,7 +14538,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14571,7 +14652,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14685,7 +14766,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14799,7 +14880,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14913,7 +14994,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -15027,7 +15108,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -15141,7 +15222,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -15255,7 +15336,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15369,7 +15450,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:08 AM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15475,7 +15556,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:08 AM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15581,7 +15662,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:08 AM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15687,7 +15768,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:08 AM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15793,7 +15874,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:08 AM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15899,7 +15980,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:08 AM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -16005,7 +16086,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:08 AM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -16111,7 +16192,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:08 AM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16217,7 +16298,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:08 AM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16323,7 +16404,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16336,7 +16417,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Top 1 | 0 out</t>
         </is>
       </c>
       <c r="F137" t="n">
@@ -16346,6 +16427,15 @@
         <is>
           <t>Top</t>
         </is>
+      </c>
+      <c r="H137" t="n">
+        <v>0</v>
+      </c>
+      <c r="I137" t="n">
+        <v>0</v>
+      </c>
+      <c r="J137" t="n">
+        <v>0</v>
       </c>
       <c r="K137" t="inlineStr">
         <is>
@@ -16437,7 +16527,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16450,7 +16540,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Top 1 | 0 out</t>
         </is>
       </c>
       <c r="F138" t="n">
@@ -16460,6 +16550,15 @@
         <is>
           <t>Top</t>
         </is>
+      </c>
+      <c r="H138" t="n">
+        <v>0</v>
+      </c>
+      <c r="I138" t="n">
+        <v>0</v>
+      </c>
+      <c r="J138" t="n">
+        <v>0</v>
       </c>
       <c r="K138" t="inlineStr">
         <is>
@@ -16551,7 +16650,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16564,7 +16663,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Top 1 | 0 out</t>
         </is>
       </c>
       <c r="F139" t="n">
@@ -16574,6 +16673,15 @@
         <is>
           <t>Top</t>
         </is>
+      </c>
+      <c r="H139" t="n">
+        <v>0</v>
+      </c>
+      <c r="I139" t="n">
+        <v>0</v>
+      </c>
+      <c r="J139" t="n">
+        <v>0</v>
       </c>
       <c r="K139" t="inlineStr">
         <is>
@@ -16665,7 +16773,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16678,7 +16786,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Top 1 | 0 out</t>
         </is>
       </c>
       <c r="F140" t="n">
@@ -16688,6 +16796,15 @@
         <is>
           <t>Top</t>
         </is>
+      </c>
+      <c r="H140" t="n">
+        <v>0</v>
+      </c>
+      <c r="I140" t="n">
+        <v>0</v>
+      </c>
+      <c r="J140" t="n">
+        <v>0</v>
       </c>
       <c r="K140" t="inlineStr">
         <is>
@@ -16779,7 +16896,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16792,7 +16909,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Top 1 | 0 out</t>
         </is>
       </c>
       <c r="F141" t="n">
@@ -16802,6 +16919,15 @@
         <is>
           <t>Top</t>
         </is>
+      </c>
+      <c r="H141" t="n">
+        <v>0</v>
+      </c>
+      <c r="I141" t="n">
+        <v>0</v>
+      </c>
+      <c r="J141" t="n">
+        <v>0</v>
       </c>
       <c r="K141" t="inlineStr">
         <is>
@@ -16893,7 +17019,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16906,7 +17032,7 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Top 1 | 0 out</t>
         </is>
       </c>
       <c r="F142" t="n">
@@ -16916,6 +17042,15 @@
         <is>
           <t>Top</t>
         </is>
+      </c>
+      <c r="H142" t="n">
+        <v>0</v>
+      </c>
+      <c r="I142" t="n">
+        <v>0</v>
+      </c>
+      <c r="J142" t="n">
+        <v>0</v>
       </c>
       <c r="K142" t="inlineStr">
         <is>
@@ -17007,7 +17142,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -17020,7 +17155,7 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Top 1 | 0 out</t>
         </is>
       </c>
       <c r="F143" t="n">
@@ -17030,6 +17165,15 @@
         <is>
           <t>Top</t>
         </is>
+      </c>
+      <c r="H143" t="n">
+        <v>0</v>
+      </c>
+      <c r="I143" t="n">
+        <v>0</v>
+      </c>
+      <c r="J143" t="n">
+        <v>0</v>
       </c>
       <c r="K143" t="inlineStr">
         <is>
@@ -17121,7 +17265,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17134,7 +17278,7 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Top 1 | 0 out</t>
         </is>
       </c>
       <c r="F144" t="n">
@@ -17144,6 +17288,15 @@
         <is>
           <t>Top</t>
         </is>
+      </c>
+      <c r="H144" t="n">
+        <v>0</v>
+      </c>
+      <c r="I144" t="n">
+        <v>0</v>
+      </c>
+      <c r="J144" t="n">
+        <v>0</v>
       </c>
       <c r="K144" t="inlineStr">
         <is>
@@ -17235,7 +17388,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17248,7 +17401,7 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Top 1 | 0 out</t>
         </is>
       </c>
       <c r="F145" t="n">
@@ -17258,6 +17411,15 @@
         <is>
           <t>Top</t>
         </is>
+      </c>
+      <c r="H145" t="n">
+        <v>0</v>
+      </c>
+      <c r="I145" t="n">
+        <v>0</v>
+      </c>
+      <c r="J145" t="n">
+        <v>0</v>
       </c>
       <c r="K145" t="inlineStr">
         <is>
@@ -17349,7 +17511,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17362,7 +17524,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>Top 4 | 2 out</t>
+          <t>Bottom 4 | 0 out</t>
         </is>
       </c>
       <c r="F146" t="n">
@@ -17370,11 +17532,11 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H146" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I146" t="n">
         <v>0</v>
@@ -17472,7 +17634,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17485,7 +17647,7 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>Top 4 | 2 out</t>
+          <t>Bottom 4 | 0 out</t>
         </is>
       </c>
       <c r="F147" t="n">
@@ -17493,11 +17655,11 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H147" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I147" t="n">
         <v>0</v>
@@ -17539,10 +17701,10 @@
         </is>
       </c>
       <c r="R147" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S147" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T147" t="n">
         <v>0</v>
@@ -17595,7 +17757,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17608,7 +17770,7 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>Top 4 | 2 out</t>
+          <t>Bottom 4 | 0 out</t>
         </is>
       </c>
       <c r="F148" t="n">
@@ -17616,11 +17778,11 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H148" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I148" t="n">
         <v>0</v>
@@ -17718,7 +17880,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17731,7 +17893,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>Top 4 | 2 out</t>
+          <t>Bottom 4 | 0 out</t>
         </is>
       </c>
       <c r="F149" t="n">
@@ -17739,11 +17901,11 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H149" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I149" t="n">
         <v>0</v>
@@ -17841,7 +18003,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17854,7 +18016,7 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>Top 4 | 2 out</t>
+          <t>Bottom 4 | 0 out</t>
         </is>
       </c>
       <c r="F150" t="n">
@@ -17862,11 +18024,11 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H150" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I150" t="n">
         <v>0</v>
@@ -17964,7 +18126,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -18078,7 +18240,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -18192,7 +18354,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18306,7 +18468,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18420,7 +18582,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18534,7 +18696,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18648,7 +18810,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18762,7 +18924,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18876,7 +19038,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18990,7 +19152,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -19113,7 +19275,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19236,7 +19398,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19359,7 +19521,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19482,7 +19644,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19605,7 +19767,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19728,7 +19890,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19851,7 +20013,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19974,7 +20136,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -20097,7 +20259,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -20220,7 +20382,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -20343,7 +20505,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20466,7 +20628,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20589,7 +20751,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20712,7 +20874,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20835,7 +20997,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20958,7 +21120,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -21081,7 +21243,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -21204,7 +21366,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -21318,7 +21480,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21432,7 +21594,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21546,7 +21708,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21660,7 +21822,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21774,7 +21936,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21888,7 +22050,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -22002,7 +22164,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -22116,7 +22278,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -22230,7 +22392,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -22243,7 +22405,7 @@
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>Top 4 | 2 out</t>
+          <t>Bottom 4 | 0 out</t>
         </is>
       </c>
       <c r="F187" t="n">
@@ -22251,11 +22413,11 @@
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H187" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I187" t="n">
         <v>0</v>
@@ -22353,7 +22515,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22366,7 +22528,7 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>Top 4 | 2 out</t>
+          <t>Bottom 4 | 0 out</t>
         </is>
       </c>
       <c r="F188" t="n">
@@ -22374,11 +22536,11 @@
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H188" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I188" t="n">
         <v>0</v>
@@ -22476,7 +22638,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22489,7 +22651,7 @@
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>Top 4 | 2 out</t>
+          <t>Bottom 4 | 0 out</t>
         </is>
       </c>
       <c r="F189" t="n">
@@ -22497,11 +22659,11 @@
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H189" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I189" t="n">
         <v>0</v>
@@ -22599,7 +22761,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22612,7 +22774,7 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>Top 4 | 2 out</t>
+          <t>Bottom 4 | 0 out</t>
         </is>
       </c>
       <c r="F190" t="n">
@@ -22620,11 +22782,11 @@
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H190" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I190" t="n">
         <v>0</v>
@@ -22722,7 +22884,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:08 AM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22828,7 +22990,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:08 AM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22934,7 +23096,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:08 AM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -23040,7 +23202,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:08 AM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -23146,7 +23308,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:08 AM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -23252,7 +23414,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:08 AM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -23358,7 +23520,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:08 AM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23464,7 +23626,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:08 AM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23570,7 +23732,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:08 AM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23676,7 +23838,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23790,7 +23952,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23904,7 +24066,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -24018,7 +24180,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -24132,7 +24294,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -24246,7 +24408,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -24360,7 +24522,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24474,7 +24636,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24588,7 +24750,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24702,7 +24864,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24816,7 +24978,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24930,7 +25092,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -25044,7 +25206,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -25158,7 +25320,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -25272,7 +25434,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -25386,7 +25548,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25500,7 +25662,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25614,7 +25776,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25728,7 +25890,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25842,7 +26004,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25956,7 +26118,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -26070,7 +26232,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -26184,7 +26346,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -26298,7 +26460,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26412,7 +26574,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26526,7 +26688,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26640,7 +26802,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26754,7 +26916,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26868,7 +27030,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26982,7 +27144,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -27096,7 +27258,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -27210,7 +27372,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -27324,7 +27486,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27438,7 +27600,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27552,7 +27714,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27666,7 +27828,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -27780,7 +27942,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -27894,7 +28056,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -28008,7 +28170,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -28122,7 +28284,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -28236,7 +28398,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -28350,7 +28512,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -28464,7 +28626,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -28578,7 +28740,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -28692,7 +28854,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:08 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -28806,7 +28968,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -28929,7 +29091,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -29052,7 +29214,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -29175,7 +29337,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -29298,7 +29460,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -29421,7 +29583,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -29544,7 +29706,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -29667,7 +29829,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -29790,7 +29952,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-07-12 10:15:07 AM PT</t>
+          <t>2026-07-12 10:17:07 AM PT</t>
         </is>
       </c>
       <c r="C253" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-12 10:19:09 AM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
@@ -681,7 +681,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -712,7 +712,7 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -731,33 +731,33 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Henry Davis</t>
+          <t>Marcell Ozuna</t>
         </is>
       </c>
       <c r="O2" t="n">
-        <v>680779</v>
+        <v>542303</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>DH</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="R2" t="n">
+        <v>2</v>
+      </c>
+      <c r="S2" t="n">
+        <v>2</v>
+      </c>
+      <c r="T2" t="n">
+        <v>2</v>
+      </c>
+      <c r="U2" t="n">
         <v>1</v>
-      </c>
-      <c r="S2" t="n">
-        <v>1</v>
-      </c>
-      <c r="T2" t="n">
-        <v>1</v>
-      </c>
-      <c r="U2" t="n">
-        <v>0</v>
       </c>
       <c r="V2" t="n">
         <v>0</v>
@@ -769,7 +769,7 @@
         <v>1</v>
       </c>
       <c r="Y2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Z2" t="n">
         <v>2</v>
@@ -787,13 +787,13 @@
         <v>0</v>
       </c>
       <c r="AE2" s="4" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="AF2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AG2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
@@ -804,7 +804,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -835,7 +835,7 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -854,24 +854,24 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Ryan O'Hearn</t>
+          <t>Henry Davis</t>
         </is>
       </c>
       <c r="O3" t="n">
-        <v>656811</v>
+        <v>680779</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>1B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="R3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S3" t="n">
         <v>1</v>
@@ -882,26 +882,26 @@
       <c r="U3" t="n">
         <v>0</v>
       </c>
-      <c r="V3" s="5" t="n">
+      <c r="V3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W3" t="n">
+        <v>0</v>
+      </c>
+      <c r="X3" s="3" t="n">
         <v>1</v>
-      </c>
-      <c r="W3" t="n">
-        <v>0</v>
-      </c>
-      <c r="X3" t="n">
-        <v>0</v>
       </c>
       <c r="Y3" t="n">
         <v>1</v>
       </c>
       <c r="Z3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AA3" t="n">
         <v>0</v>
       </c>
-      <c r="AB3" s="6" t="n">
-        <v>1</v>
+      <c r="AB3" t="n">
+        <v>0</v>
       </c>
       <c r="AC3" t="n">
         <v>0</v>
@@ -910,13 +910,13 @@
         <v>0</v>
       </c>
       <c r="AE3" s="4" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="AF3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AG3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
@@ -927,7 +927,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -958,46 +958,46 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Away</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
+          <t>PIT</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
           <t>MIL</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>PIT</t>
-        </is>
-      </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Jackson Chourio</t>
+          <t>Ryan O'Hearn</t>
         </is>
       </c>
       <c r="O4" t="n">
-        <v>694192</v>
+        <v>656811</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>LF</t>
+          <t>1B</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="R4" t="n">
         <v>2</v>
       </c>
       <c r="S4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T4" t="n">
         <v>1</v>
@@ -1023,23 +1023,23 @@
       <c r="AA4" t="n">
         <v>0</v>
       </c>
-      <c r="AB4" t="n">
-        <v>0</v>
+      <c r="AB4" s="6" t="n">
+        <v>1</v>
       </c>
       <c r="AC4" t="n">
         <v>0</v>
       </c>
       <c r="AD4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AE4" s="4" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="AF4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AG4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5">
@@ -1050,7 +1050,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1081,7 +1081,7 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -1100,20 +1100,20 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Christian Yelich</t>
+          <t>Jackson Chourio</t>
         </is>
       </c>
       <c r="O5" t="n">
-        <v>592885</v>
+        <v>694192</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>DH</t>
+          <t>LF</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R5" t="n">
@@ -1141,7 +1141,7 @@
         <v>1</v>
       </c>
       <c r="Z5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA5" t="n">
         <v>0</v>
@@ -1153,10 +1153,10 @@
         <v>0</v>
       </c>
       <c r="AD5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE5" s="4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="AF5" t="n">
         <v>2</v>
@@ -1173,7 +1173,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1204,39 +1204,39 @@
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Home</t>
+          <t>Away</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
+          <t>MIL</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
           <t>PIT</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>MIL</t>
-        </is>
-      </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Esmerlyn Valdez</t>
+          <t>Christian Yelich</t>
         </is>
       </c>
       <c r="O6" t="n">
-        <v>699013</v>
+        <v>592885</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>RF</t>
+          <t>DH</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="R6" t="n">
@@ -1282,10 +1282,10 @@
         <v>7</v>
       </c>
       <c r="AF6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AG6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -1296,7 +1296,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1327,7 +1327,7 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -1346,36 +1346,36 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Marcell Ozuna</t>
+          <t>Esmerlyn Valdez</t>
         </is>
       </c>
       <c r="O7" t="n">
-        <v>542303</v>
+        <v>699013</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>DH</t>
+          <t>RF</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>4</t>
         </is>
       </c>
       <c r="R7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T7" t="n">
         <v>1</v>
       </c>
       <c r="U7" t="n">
+        <v>0</v>
+      </c>
+      <c r="V7" s="5" t="n">
         <v>1</v>
-      </c>
-      <c r="V7" t="n">
-        <v>0</v>
       </c>
       <c r="W7" t="n">
         <v>0</v>
@@ -1387,7 +1387,7 @@
         <v>1</v>
       </c>
       <c r="Z7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA7" t="n">
         <v>0</v>
@@ -1405,10 +1405,10 @@
         <v>7</v>
       </c>
       <c r="AF7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AG7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1450,7 +1450,7 @@
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -1528,10 +1528,10 @@
         <v>3</v>
       </c>
       <c r="AF8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AG8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
@@ -1542,7 +1542,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1573,7 +1573,7 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -1665,7 +1665,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1696,7 +1696,7 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -1788,7 +1788,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1902,7 +1902,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -2016,7 +2016,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2130,7 +2130,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2244,7 +2244,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2472,7 +2472,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2586,7 +2586,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2700,7 +2700,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2814,7 +2814,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -3042,7 +3042,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3156,7 +3156,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3270,7 +3270,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3384,7 +3384,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3498,7 +3498,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3612,7 +3612,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3726,7 +3726,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3840,7 +3840,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3963,7 +3963,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -4086,7 +4086,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4209,7 +4209,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4332,7 +4332,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4455,7 +4455,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4578,7 +4578,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4701,7 +4701,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4824,7 +4824,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4947,7 +4947,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -5070,7 +5070,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5193,7 +5193,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5316,7 +5316,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5439,7 +5439,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5562,7 +5562,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5685,7 +5685,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5808,7 +5808,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5931,7 +5931,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -6054,7 +6054,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -6168,7 +6168,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6282,7 +6282,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6396,7 +6396,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6510,7 +6510,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6624,7 +6624,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6738,7 +6738,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6852,7 +6852,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6966,7 +6966,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -7080,7 +7080,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -7194,7 +7194,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7308,7 +7308,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7422,7 +7422,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7536,7 +7536,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7650,7 +7650,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7764,7 +7764,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7878,7 +7878,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7992,7 +7992,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -8106,7 +8106,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -8229,7 +8229,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8352,7 +8352,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8475,7 +8475,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8598,7 +8598,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8721,7 +8721,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8844,7 +8844,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8967,7 +8967,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -9090,7 +9090,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -9213,7 +9213,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9327,7 +9327,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9441,7 +9441,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9555,7 +9555,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9669,7 +9669,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9783,7 +9783,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9897,7 +9897,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -10011,7 +10011,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -10125,7 +10125,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -10239,7 +10239,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10353,7 +10353,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10467,7 +10467,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10581,7 +10581,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10695,7 +10695,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10809,7 +10809,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10923,7 +10923,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -11037,7 +11037,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -11151,7 +11151,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -11265,7 +11265,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11278,7 +11278,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Top 1 | 0 out</t>
         </is>
       </c>
       <c r="F92" t="n">
@@ -11288,6 +11288,15 @@
         <is>
           <t>Top</t>
         </is>
+      </c>
+      <c r="H92" t="n">
+        <v>0</v>
+      </c>
+      <c r="I92" t="n">
+        <v>0</v>
+      </c>
+      <c r="J92" t="n">
+        <v>0</v>
       </c>
       <c r="K92" t="inlineStr">
         <is>
@@ -11379,7 +11388,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11392,7 +11401,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Top 1 | 0 out</t>
         </is>
       </c>
       <c r="F93" t="n">
@@ -11402,6 +11411,15 @@
         <is>
           <t>Top</t>
         </is>
+      </c>
+      <c r="H93" t="n">
+        <v>0</v>
+      </c>
+      <c r="I93" t="n">
+        <v>0</v>
+      </c>
+      <c r="J93" t="n">
+        <v>0</v>
       </c>
       <c r="K93" t="inlineStr">
         <is>
@@ -11493,7 +11511,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11506,7 +11524,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Top 1 | 0 out</t>
         </is>
       </c>
       <c r="F94" t="n">
@@ -11516,6 +11534,15 @@
         <is>
           <t>Top</t>
         </is>
+      </c>
+      <c r="H94" t="n">
+        <v>0</v>
+      </c>
+      <c r="I94" t="n">
+        <v>0</v>
+      </c>
+      <c r="J94" t="n">
+        <v>0</v>
       </c>
       <c r="K94" t="inlineStr">
         <is>
@@ -11607,7 +11634,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11620,7 +11647,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Top 1 | 0 out</t>
         </is>
       </c>
       <c r="F95" t="n">
@@ -11630,6 +11657,15 @@
         <is>
           <t>Top</t>
         </is>
+      </c>
+      <c r="H95" t="n">
+        <v>0</v>
+      </c>
+      <c r="I95" t="n">
+        <v>0</v>
+      </c>
+      <c r="J95" t="n">
+        <v>0</v>
       </c>
       <c r="K95" t="inlineStr">
         <is>
@@ -11721,7 +11757,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11734,7 +11770,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Top 1 | 0 out</t>
         </is>
       </c>
       <c r="F96" t="n">
@@ -11744,6 +11780,15 @@
         <is>
           <t>Top</t>
         </is>
+      </c>
+      <c r="H96" t="n">
+        <v>0</v>
+      </c>
+      <c r="I96" t="n">
+        <v>0</v>
+      </c>
+      <c r="J96" t="n">
+        <v>0</v>
       </c>
       <c r="K96" t="inlineStr">
         <is>
@@ -11835,7 +11880,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11848,7 +11893,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Top 1 | 0 out</t>
         </is>
       </c>
       <c r="F97" t="n">
@@ -11858,6 +11903,15 @@
         <is>
           <t>Top</t>
         </is>
+      </c>
+      <c r="H97" t="n">
+        <v>0</v>
+      </c>
+      <c r="I97" t="n">
+        <v>0</v>
+      </c>
+      <c r="J97" t="n">
+        <v>0</v>
       </c>
       <c r="K97" t="inlineStr">
         <is>
@@ -11949,7 +12003,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11962,7 +12016,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Top 1 | 0 out</t>
         </is>
       </c>
       <c r="F98" t="n">
@@ -11972,6 +12026,15 @@
         <is>
           <t>Top</t>
         </is>
+      </c>
+      <c r="H98" t="n">
+        <v>0</v>
+      </c>
+      <c r="I98" t="n">
+        <v>0</v>
+      </c>
+      <c r="J98" t="n">
+        <v>0</v>
       </c>
       <c r="K98" t="inlineStr">
         <is>
@@ -12063,7 +12126,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -12076,7 +12139,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Top 1 | 0 out</t>
         </is>
       </c>
       <c r="F99" t="n">
@@ -12086,6 +12149,15 @@
         <is>
           <t>Top</t>
         </is>
+      </c>
+      <c r="H99" t="n">
+        <v>0</v>
+      </c>
+      <c r="I99" t="n">
+        <v>0</v>
+      </c>
+      <c r="J99" t="n">
+        <v>0</v>
       </c>
       <c r="K99" t="inlineStr">
         <is>
@@ -12177,7 +12249,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -12190,7 +12262,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Top 1 | 0 out</t>
         </is>
       </c>
       <c r="F100" t="n">
@@ -12200,6 +12272,15 @@
         <is>
           <t>Top</t>
         </is>
+      </c>
+      <c r="H100" t="n">
+        <v>0</v>
+      </c>
+      <c r="I100" t="n">
+        <v>0</v>
+      </c>
+      <c r="J100" t="n">
+        <v>0</v>
       </c>
       <c r="K100" t="inlineStr">
         <is>
@@ -12291,7 +12372,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12405,7 +12486,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12519,7 +12600,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12633,7 +12714,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12747,7 +12828,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12861,7 +12942,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12975,7 +13056,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -13089,7 +13170,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -13203,7 +13284,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13317,7 +13398,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13440,7 +13521,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13563,7 +13644,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13686,7 +13767,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13809,7 +13890,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13932,7 +14013,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -14055,7 +14136,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -14178,7 +14259,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -14301,7 +14382,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14424,7 +14505,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14538,7 +14619,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14652,7 +14733,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14766,7 +14847,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14880,7 +14961,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14994,7 +15075,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -15108,7 +15189,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -15222,7 +15303,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -15336,7 +15417,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15450,7 +15531,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:08 AM PT</t>
+          <t>2026-07-12 10:19:08 AM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15556,7 +15637,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:08 AM PT</t>
+          <t>2026-07-12 10:19:08 AM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15662,7 +15743,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:08 AM PT</t>
+          <t>2026-07-12 10:19:08 AM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15768,7 +15849,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:08 AM PT</t>
+          <t>2026-07-12 10:19:08 AM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15874,7 +15955,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:08 AM PT</t>
+          <t>2026-07-12 10:19:08 AM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15980,7 +16061,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:08 AM PT</t>
+          <t>2026-07-12 10:19:08 AM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -16086,7 +16167,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:08 AM PT</t>
+          <t>2026-07-12 10:19:08 AM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -16192,7 +16273,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:08 AM PT</t>
+          <t>2026-07-12 10:19:08 AM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16298,7 +16379,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:08 AM PT</t>
+          <t>2026-07-12 10:19:08 AM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16404,7 +16485,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16527,7 +16608,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16650,7 +16731,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16773,7 +16854,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16896,7 +16977,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -17019,7 +17100,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -17142,7 +17223,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -17265,7 +17346,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17388,7 +17469,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17511,7 +17592,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17542,7 +17623,7 @@
         <v>0</v>
       </c>
       <c r="J146" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K146" t="inlineStr">
         <is>
@@ -17634,7 +17715,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17665,7 +17746,7 @@
         <v>0</v>
       </c>
       <c r="J147" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K147" t="inlineStr">
         <is>
@@ -17757,7 +17838,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17788,7 +17869,7 @@
         <v>0</v>
       </c>
       <c r="J148" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K148" t="inlineStr">
         <is>
@@ -17880,7 +17961,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17911,7 +17992,7 @@
         <v>0</v>
       </c>
       <c r="J149" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K149" t="inlineStr">
         <is>
@@ -18003,7 +18084,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -18034,7 +18115,7 @@
         <v>0</v>
       </c>
       <c r="J150" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K150" t="inlineStr">
         <is>
@@ -18126,7 +18207,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -18240,7 +18321,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -18354,7 +18435,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18468,7 +18549,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18582,7 +18663,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18696,7 +18777,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18810,7 +18891,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18924,7 +19005,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -19038,7 +19119,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -19152,7 +19233,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -19275,7 +19356,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19398,7 +19479,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19521,7 +19602,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19644,7 +19725,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19767,7 +19848,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19890,7 +19971,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -20013,7 +20094,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -20136,7 +20217,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -20259,7 +20340,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -20382,7 +20463,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -20505,7 +20586,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20628,7 +20709,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20751,7 +20832,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20874,7 +20955,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20997,7 +21078,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -21120,7 +21201,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -21243,7 +21324,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -21366,7 +21447,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -21379,7 +21460,7 @@
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Top 1 | 0 out</t>
         </is>
       </c>
       <c r="F178" t="n">
@@ -21389,6 +21470,15 @@
         <is>
           <t>Top</t>
         </is>
+      </c>
+      <c r="H178" t="n">
+        <v>0</v>
+      </c>
+      <c r="I178" t="n">
+        <v>0</v>
+      </c>
+      <c r="J178" t="n">
+        <v>0</v>
       </c>
       <c r="K178" t="inlineStr">
         <is>
@@ -21480,7 +21570,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21493,7 +21583,7 @@
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Top 1 | 0 out</t>
         </is>
       </c>
       <c r="F179" t="n">
@@ -21503,6 +21593,15 @@
         <is>
           <t>Top</t>
         </is>
+      </c>
+      <c r="H179" t="n">
+        <v>0</v>
+      </c>
+      <c r="I179" t="n">
+        <v>0</v>
+      </c>
+      <c r="J179" t="n">
+        <v>0</v>
       </c>
       <c r="K179" t="inlineStr">
         <is>
@@ -21594,7 +21693,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21607,7 +21706,7 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Top 1 | 0 out</t>
         </is>
       </c>
       <c r="F180" t="n">
@@ -21617,6 +21716,15 @@
         <is>
           <t>Top</t>
         </is>
+      </c>
+      <c r="H180" t="n">
+        <v>0</v>
+      </c>
+      <c r="I180" t="n">
+        <v>0</v>
+      </c>
+      <c r="J180" t="n">
+        <v>0</v>
       </c>
       <c r="K180" t="inlineStr">
         <is>
@@ -21708,7 +21816,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21721,7 +21829,7 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Top 1 | 0 out</t>
         </is>
       </c>
       <c r="F181" t="n">
@@ -21731,6 +21839,15 @@
         <is>
           <t>Top</t>
         </is>
+      </c>
+      <c r="H181" t="n">
+        <v>0</v>
+      </c>
+      <c r="I181" t="n">
+        <v>0</v>
+      </c>
+      <c r="J181" t="n">
+        <v>0</v>
       </c>
       <c r="K181" t="inlineStr">
         <is>
@@ -21822,7 +21939,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21835,7 +21952,7 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Top 1 | 0 out</t>
         </is>
       </c>
       <c r="F182" t="n">
@@ -21845,6 +21962,15 @@
         <is>
           <t>Top</t>
         </is>
+      </c>
+      <c r="H182" t="n">
+        <v>0</v>
+      </c>
+      <c r="I182" t="n">
+        <v>0</v>
+      </c>
+      <c r="J182" t="n">
+        <v>0</v>
       </c>
       <c r="K182" t="inlineStr">
         <is>
@@ -21936,7 +22062,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21949,7 +22075,7 @@
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Top 1 | 0 out</t>
         </is>
       </c>
       <c r="F183" t="n">
@@ -21959,6 +22085,15 @@
         <is>
           <t>Top</t>
         </is>
+      </c>
+      <c r="H183" t="n">
+        <v>0</v>
+      </c>
+      <c r="I183" t="n">
+        <v>0</v>
+      </c>
+      <c r="J183" t="n">
+        <v>0</v>
       </c>
       <c r="K183" t="inlineStr">
         <is>
@@ -22050,7 +22185,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -22063,7 +22198,7 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Top 1 | 0 out</t>
         </is>
       </c>
       <c r="F184" t="n">
@@ -22073,6 +22208,15 @@
         <is>
           <t>Top</t>
         </is>
+      </c>
+      <c r="H184" t="n">
+        <v>0</v>
+      </c>
+      <c r="I184" t="n">
+        <v>0</v>
+      </c>
+      <c r="J184" t="n">
+        <v>0</v>
       </c>
       <c r="K184" t="inlineStr">
         <is>
@@ -22164,7 +22308,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -22177,7 +22321,7 @@
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Top 1 | 0 out</t>
         </is>
       </c>
       <c r="F185" t="n">
@@ -22187,6 +22331,15 @@
         <is>
           <t>Top</t>
         </is>
+      </c>
+      <c r="H185" t="n">
+        <v>0</v>
+      </c>
+      <c r="I185" t="n">
+        <v>0</v>
+      </c>
+      <c r="J185" t="n">
+        <v>0</v>
       </c>
       <c r="K185" t="inlineStr">
         <is>
@@ -22278,7 +22431,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -22291,7 +22444,7 @@
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Top 1 | 0 out</t>
         </is>
       </c>
       <c r="F186" t="n">
@@ -22301,6 +22454,15 @@
         <is>
           <t>Top</t>
         </is>
+      </c>
+      <c r="H186" t="n">
+        <v>0</v>
+      </c>
+      <c r="I186" t="n">
+        <v>0</v>
+      </c>
+      <c r="J186" t="n">
+        <v>0</v>
       </c>
       <c r="K186" t="inlineStr">
         <is>
@@ -22392,7 +22554,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -22423,7 +22585,7 @@
         <v>0</v>
       </c>
       <c r="J187" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K187" t="inlineStr">
         <is>
@@ -22501,10 +22663,10 @@
         <v>0</v>
       </c>
       <c r="AF187" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AG187" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="188">
@@ -22515,7 +22677,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22546,7 +22708,7 @@
         <v>0</v>
       </c>
       <c r="J188" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K188" t="inlineStr">
         <is>
@@ -22624,10 +22786,10 @@
         <v>0</v>
       </c>
       <c r="AF188" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AG188" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="189">
@@ -22638,7 +22800,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22669,7 +22831,7 @@
         <v>0</v>
       </c>
       <c r="J189" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K189" t="inlineStr">
         <is>
@@ -22747,10 +22909,10 @@
         <v>0</v>
       </c>
       <c r="AF189" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AG189" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="190">
@@ -22761,7 +22923,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22792,7 +22954,7 @@
         <v>0</v>
       </c>
       <c r="J190" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K190" t="inlineStr">
         <is>
@@ -22870,10 +23032,10 @@
         <v>0</v>
       </c>
       <c r="AF190" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AG190" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="191">
@@ -22884,7 +23046,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:08 AM PT</t>
+          <t>2026-07-12 10:19:08 AM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22990,7 +23152,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:08 AM PT</t>
+          <t>2026-07-12 10:19:08 AM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -23096,7 +23258,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:08 AM PT</t>
+          <t>2026-07-12 10:19:08 AM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -23202,7 +23364,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:08 AM PT</t>
+          <t>2026-07-12 10:19:08 AM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -23308,7 +23470,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:08 AM PT</t>
+          <t>2026-07-12 10:19:08 AM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -23414,7 +23576,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:08 AM PT</t>
+          <t>2026-07-12 10:19:08 AM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -23520,7 +23682,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:08 AM PT</t>
+          <t>2026-07-12 10:19:08 AM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23626,7 +23788,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:08 AM PT</t>
+          <t>2026-07-12 10:19:08 AM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23732,7 +23894,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:08 AM PT</t>
+          <t>2026-07-12 10:19:08 AM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23838,7 +24000,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23952,7 +24114,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -24066,7 +24228,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -24180,7 +24342,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -24294,7 +24456,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -24408,7 +24570,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -24522,7 +24684,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24636,7 +24798,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24750,7 +24912,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24864,7 +25026,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24978,7 +25140,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -25092,7 +25254,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -25206,7 +25368,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -25320,7 +25482,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -25434,7 +25596,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -25548,7 +25710,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25662,7 +25824,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25776,7 +25938,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25890,7 +26052,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -26004,7 +26166,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -26118,7 +26280,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -26232,7 +26394,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -26346,7 +26508,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -26460,7 +26622,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26574,7 +26736,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26688,7 +26850,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26802,7 +26964,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26916,7 +27078,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -27030,7 +27192,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -27144,7 +27306,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -27258,7 +27420,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -27372,7 +27534,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -27486,7 +27648,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27600,7 +27762,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27714,7 +27876,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27828,7 +27990,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -27942,7 +28104,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -28056,7 +28218,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -28170,7 +28332,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -28284,7 +28446,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -28398,7 +28560,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -28512,7 +28674,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -28626,7 +28788,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -28740,7 +28902,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -28854,7 +29016,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -28968,7 +29130,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -29091,7 +29253,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -29214,7 +29376,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -29337,7 +29499,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -29460,7 +29622,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -29583,7 +29745,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -29706,7 +29868,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -29829,7 +29991,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -29952,7 +30114,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-07-12 10:17:07 AM PT</t>
+          <t>2026-07-12 10:19:07 AM PT</t>
         </is>
       </c>
       <c r="C253" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-12 03:19:34 PM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -807,7 +807,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:15 PM PT</t>
+          <t>2026-07-12 03:19:30 PM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -921,7 +921,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1405,10 +1405,10 @@
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -1500,7 +1500,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:18 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1528,10 +1528,10 @@
         <v>1</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -1623,7 +1623,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1737,7 +1737,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1851,7 +1851,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:15 PM PT</t>
+          <t>2026-07-12 03:19:30 PM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1965,7 +1965,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2079,7 +2079,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:15 PM PT</t>
+          <t>2026-07-12 03:19:30 PM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2193,7 +2193,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2307,7 +2307,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:15 PM PT</t>
+          <t>2026-07-12 03:19:30 PM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2421,7 +2421,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2535,7 +2535,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2649,7 +2649,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2763,7 +2763,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2877,7 +2877,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2991,7 +2991,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:15 PM PT</t>
+          <t>2026-07-12 03:19:30 PM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3105,7 +3105,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3219,7 +3219,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3333,7 +3333,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3447,7 +3447,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:18 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3460,7 +3460,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 1 out</t>
         </is>
       </c>
       <c r="F26" t="n">
@@ -3472,13 +3472,13 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I26" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J26" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
@@ -3570,7 +3570,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3684,7 +3684,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3798,7 +3798,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3912,7 +3912,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -4026,7 +4026,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4140,7 +4140,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4254,7 +4254,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4368,7 +4368,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4482,7 +4482,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4596,7 +4596,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4710,7 +4710,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:15 PM PT</t>
+          <t>2026-07-12 03:19:30 PM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4824,7 +4824,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4938,7 +4938,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:15 PM PT</t>
+          <t>2026-07-12 03:19:30 PM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5052,7 +5052,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:15 PM PT</t>
+          <t>2026-07-12 03:19:30 PM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5166,7 +5166,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5280,7 +5280,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5394,7 +5394,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5508,7 +5508,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:18 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5521,7 +5521,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 1 out</t>
         </is>
       </c>
       <c r="F44" t="n">
@@ -5533,13 +5533,13 @@
         </is>
       </c>
       <c r="H44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I44" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J44" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K44" t="inlineStr">
         <is>
@@ -5631,7 +5631,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5745,7 +5745,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5859,7 +5859,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5973,7 +5973,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6087,7 +6087,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6201,7 +6201,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:15 PM PT</t>
+          <t>2026-07-12 03:19:30 PM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6315,7 +6315,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:18 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6343,10 +6343,10 @@
         <v>1</v>
       </c>
       <c r="I51" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J51" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K51" t="inlineStr">
         <is>
@@ -6438,7 +6438,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6552,7 +6552,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6666,7 +6666,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6780,7 +6780,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6894,7 +6894,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:15 PM PT</t>
+          <t>2026-07-12 03:19:30 PM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -7008,7 +7008,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7122,7 +7122,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7150,10 +7150,10 @@
         <v>0</v>
       </c>
       <c r="I58" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J58" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K58" t="inlineStr">
         <is>
@@ -7245,7 +7245,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7359,7 +7359,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7473,7 +7473,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7587,7 +7587,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7701,7 +7701,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7815,7 +7815,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7929,7 +7929,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -8043,7 +8043,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8157,7 +8157,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:18 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8170,7 +8170,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 1 out</t>
         </is>
       </c>
       <c r="F67" t="n">
@@ -8182,13 +8182,13 @@
         </is>
       </c>
       <c r="H67" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I67" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J67" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K67" t="inlineStr">
         <is>
@@ -8280,7 +8280,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8394,7 +8394,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:18 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8422,10 +8422,10 @@
         <v>1</v>
       </c>
       <c r="I69" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J69" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K69" t="inlineStr">
         <is>
@@ -8517,7 +8517,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8631,7 +8631,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8745,7 +8745,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8859,7 +8859,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8973,7 +8973,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9087,7 +9087,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9201,7 +9201,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9315,7 +9315,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9429,7 +9429,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9543,7 +9543,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9657,7 +9657,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9771,7 +9771,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9885,7 +9885,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -9999,7 +9999,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10113,7 +10113,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10227,7 +10227,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:18 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10240,7 +10240,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 1 out</t>
         </is>
       </c>
       <c r="F85" t="n">
@@ -10252,13 +10252,13 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I85" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J85" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K85" t="inlineStr">
         <is>
@@ -10350,7 +10350,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10464,7 +10464,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:18 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10477,7 +10477,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 1 out</t>
         </is>
       </c>
       <c r="F87" t="n">
@@ -10489,13 +10489,13 @@
         </is>
       </c>
       <c r="H87" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I87" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J87" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K87" t="inlineStr">
         <is>
@@ -10531,10 +10531,10 @@
         </is>
       </c>
       <c r="R87" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S87" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T87" t="n">
         <v>1</v>
@@ -10587,7 +10587,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:18 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10615,10 +10615,10 @@
         <v>1</v>
       </c>
       <c r="I88" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J88" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K88" t="inlineStr">
         <is>
@@ -10710,7 +10710,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10824,7 +10824,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10938,7 +10938,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -11052,7 +11052,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11166,7 +11166,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11280,7 +11280,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:18 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11308,10 +11308,10 @@
         <v>1</v>
       </c>
       <c r="I94" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J94" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K94" t="inlineStr">
         <is>
@@ -11403,7 +11403,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11517,7 +11517,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:15 PM PT</t>
+          <t>2026-07-12 03:19:30 PM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11631,7 +11631,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:15 PM PT</t>
+          <t>2026-07-12 03:19:30 PM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11745,7 +11745,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:15 PM PT</t>
+          <t>2026-07-12 03:19:30 PM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11859,7 +11859,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:15 PM PT</t>
+          <t>2026-07-12 03:19:30 PM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11973,7 +11973,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -12087,7 +12087,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12201,7 +12201,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12315,7 +12315,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:18 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12328,7 +12328,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 1 out</t>
         </is>
       </c>
       <c r="F103" t="n">
@@ -12340,13 +12340,13 @@
         </is>
       </c>
       <c r="H103" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I103" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J103" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K103" t="inlineStr">
         <is>
@@ -12438,7 +12438,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12466,10 +12466,10 @@
         <v>0</v>
       </c>
       <c r="I104" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J104" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K104" t="inlineStr">
         <is>
@@ -12561,7 +12561,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12589,10 +12589,10 @@
         <v>0</v>
       </c>
       <c r="I105" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J105" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K105" t="inlineStr">
         <is>
@@ -12684,7 +12684,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12798,7 +12798,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12912,7 +12912,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -13026,7 +13026,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:18 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13039,7 +13039,7 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 1 out</t>
         </is>
       </c>
       <c r="F109" t="n">
@@ -13051,13 +13051,13 @@
         </is>
       </c>
       <c r="H109" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I109" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J109" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K109" t="inlineStr">
         <is>
@@ -13149,7 +13149,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13263,7 +13263,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13377,7 +13377,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13491,7 +13491,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13519,10 +13519,10 @@
         <v>0</v>
       </c>
       <c r="I113" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J113" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K113" t="inlineStr">
         <is>
@@ -13614,7 +13614,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13728,7 +13728,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13842,7 +13842,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13956,7 +13956,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -13984,10 +13984,10 @@
         <v>0</v>
       </c>
       <c r="I117" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J117" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K117" t="inlineStr">
         <is>
@@ -14079,7 +14079,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14193,7 +14193,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14307,7 +14307,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14421,7 +14421,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14535,7 +14535,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14649,7 +14649,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14763,7 +14763,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14877,7 +14877,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14991,7 +14991,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -15105,7 +15105,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15219,7 +15219,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15333,7 +15333,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15447,7 +15447,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15561,7 +15561,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15675,7 +15675,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15789,7 +15789,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15903,7 +15903,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -16017,7 +16017,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16131,7 +16131,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16245,7 +16245,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16359,7 +16359,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16473,7 +16473,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16587,7 +16587,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16701,7 +16701,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16815,7 +16815,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16929,7 +16929,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -17043,7 +17043,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17157,7 +17157,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17271,7 +17271,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:15 PM PT</t>
+          <t>2026-07-12 03:19:30 PM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17385,7 +17385,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:18 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17398,7 +17398,7 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 1 out</t>
         </is>
       </c>
       <c r="F147" t="n">
@@ -17410,13 +17410,13 @@
         </is>
       </c>
       <c r="H147" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I147" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J147" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K147" t="inlineStr">
         <is>
@@ -17508,7 +17508,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17622,7 +17622,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17650,10 +17650,10 @@
         <v>0</v>
       </c>
       <c r="I149" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J149" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K149" t="inlineStr">
         <is>
@@ -17745,7 +17745,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17859,7 +17859,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17973,7 +17973,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:18 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -18001,10 +18001,10 @@
         <v>1</v>
       </c>
       <c r="I152" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J152" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K152" t="inlineStr">
         <is>
@@ -18096,7 +18096,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18210,7 +18210,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18324,7 +18324,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18438,7 +18438,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:18 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18466,10 +18466,10 @@
         <v>1</v>
       </c>
       <c r="I156" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J156" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K156" t="inlineStr">
         <is>
@@ -18561,7 +18561,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18675,7 +18675,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18789,7 +18789,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:18 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18802,7 +18802,7 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 1 out</t>
         </is>
       </c>
       <c r="F159" t="n">
@@ -18814,13 +18814,13 @@
         </is>
       </c>
       <c r="H159" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I159" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J159" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K159" t="inlineStr">
         <is>
@@ -18912,7 +18912,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:18 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18925,7 +18925,7 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 1 out</t>
         </is>
       </c>
       <c r="F160" t="n">
@@ -18937,13 +18937,13 @@
         </is>
       </c>
       <c r="H160" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I160" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J160" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K160" t="inlineStr">
         <is>
@@ -19035,7 +19035,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19149,7 +19149,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19177,10 +19177,10 @@
         <v>0</v>
       </c>
       <c r="I162" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J162" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K162" t="inlineStr">
         <is>
@@ -19272,7 +19272,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19300,10 +19300,10 @@
         <v>0</v>
       </c>
       <c r="I163" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J163" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K163" t="inlineStr">
         <is>
@@ -19395,7 +19395,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19509,7 +19509,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19623,7 +19623,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19737,7 +19737,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19851,7 +19851,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19965,7 +19965,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -20079,7 +20079,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -20193,7 +20193,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20307,7 +20307,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20421,7 +20421,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20535,7 +20535,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20563,10 +20563,10 @@
         <v>0</v>
       </c>
       <c r="I174" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J174" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K174" t="inlineStr">
         <is>
@@ -20658,7 +20658,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20772,7 +20772,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20886,7 +20886,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -21000,7 +21000,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -21114,7 +21114,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:15 PM PT</t>
+          <t>2026-07-12 03:19:30 PM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21228,7 +21228,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21342,7 +21342,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21456,7 +21456,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21484,10 +21484,10 @@
         <v>0</v>
       </c>
       <c r="I182" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J182" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K182" t="inlineStr">
         <is>
@@ -21579,7 +21579,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21693,7 +21693,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21807,7 +21807,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21921,7 +21921,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:18 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21934,7 +21934,7 @@
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 1 out</t>
         </is>
       </c>
       <c r="F186" t="n">
@@ -21946,13 +21946,13 @@
         </is>
       </c>
       <c r="H186" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I186" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J186" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K186" t="inlineStr">
         <is>
@@ -22044,7 +22044,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:18 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -22057,7 +22057,7 @@
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 1 out</t>
         </is>
       </c>
       <c r="F187" t="n">
@@ -22069,13 +22069,13 @@
         </is>
       </c>
       <c r="H187" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I187" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J187" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K187" t="inlineStr">
         <is>
@@ -22167,7 +22167,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22281,7 +22281,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:18 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22309,10 +22309,10 @@
         <v>1</v>
       </c>
       <c r="I189" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J189" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K189" t="inlineStr">
         <is>
@@ -22404,7 +22404,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22518,7 +22518,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22632,7 +22632,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22746,7 +22746,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22860,7 +22860,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22974,7 +22974,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -23088,7 +23088,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -23202,7 +23202,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23316,7 +23316,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23430,7 +23430,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23458,10 +23458,10 @@
         <v>0</v>
       </c>
       <c r="I199" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J199" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K199" t="inlineStr">
         <is>
@@ -23553,7 +23553,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23581,10 +23581,10 @@
         <v>0</v>
       </c>
       <c r="I200" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J200" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K200" t="inlineStr">
         <is>
@@ -23676,7 +23676,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23790,7 +23790,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23904,7 +23904,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -24018,7 +24018,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -24132,7 +24132,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -24246,7 +24246,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24360,7 +24360,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24474,7 +24474,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24588,7 +24588,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:18 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24616,10 +24616,10 @@
         <v>1</v>
       </c>
       <c r="I209" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J209" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K209" t="inlineStr">
         <is>
@@ -24711,7 +24711,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:18 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24739,10 +24739,10 @@
         <v>1</v>
       </c>
       <c r="I210" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J210" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K210" t="inlineStr">
         <is>
@@ -24834,7 +24834,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24948,7 +24948,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:15 PM PT</t>
+          <t>2026-07-12 03:19:30 PM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -25062,7 +25062,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -25176,7 +25176,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -25290,7 +25290,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25404,7 +25404,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25518,7 +25518,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25632,7 +25632,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25660,10 +25660,10 @@
         <v>0</v>
       </c>
       <c r="I218" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J218" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K218" t="inlineStr">
         <is>
@@ -25755,7 +25755,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25869,7 +25869,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25983,7 +25983,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -26097,7 +26097,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -26211,7 +26211,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:18 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26224,7 +26224,7 @@
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 1 out</t>
         </is>
       </c>
       <c r="F223" t="n">
@@ -26236,13 +26236,13 @@
         </is>
       </c>
       <c r="H223" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I223" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J223" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K223" t="inlineStr">
         <is>
@@ -26334,7 +26334,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26448,7 +26448,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:18 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26476,10 +26476,10 @@
         <v>1</v>
       </c>
       <c r="I225" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J225" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K225" t="inlineStr">
         <is>
@@ -26571,7 +26571,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:18 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26599,10 +26599,10 @@
         <v>1</v>
       </c>
       <c r="I226" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J226" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K226" t="inlineStr">
         <is>
@@ -26694,7 +26694,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:18 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26722,10 +26722,10 @@
         <v>1</v>
       </c>
       <c r="I227" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J227" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K227" t="inlineStr">
         <is>
@@ -26817,7 +26817,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:18 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26845,10 +26845,10 @@
         <v>1</v>
       </c>
       <c r="I228" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J228" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K228" t="inlineStr">
         <is>
@@ -26884,10 +26884,10 @@
         </is>
       </c>
       <c r="R228" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S228" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T228" t="n">
         <v>0</v>
@@ -26940,7 +26940,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -27054,7 +27054,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -27168,7 +27168,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -27282,7 +27282,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27396,7 +27396,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27510,7 +27510,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27624,7 +27624,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -27738,7 +27738,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -27852,7 +27852,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -27966,7 +27966,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -28080,7 +28080,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -28194,7 +28194,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -28308,7 +28308,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -28336,10 +28336,10 @@
         <v>0</v>
       </c>
       <c r="I241" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J241" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K241" t="inlineStr">
         <is>
@@ -28431,7 +28431,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -28459,10 +28459,10 @@
         <v>0</v>
       </c>
       <c r="I242" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J242" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K242" t="inlineStr">
         <is>
@@ -28554,7 +28554,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -28582,10 +28582,10 @@
         <v>0</v>
       </c>
       <c r="I243" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J243" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K243" t="inlineStr">
         <is>
@@ -28677,7 +28677,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -28705,10 +28705,10 @@
         <v>0</v>
       </c>
       <c r="I244" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J244" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K244" t="inlineStr">
         <is>
@@ -28800,7 +28800,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -28914,7 +28914,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -29028,7 +29028,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -29142,7 +29142,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -29256,7 +29256,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -29370,7 +29370,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -29484,7 +29484,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -29598,7 +29598,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -29712,7 +29712,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -29826,7 +29826,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -29940,7 +29940,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -30054,7 +30054,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -30168,7 +30168,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -30282,7 +30282,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -30396,7 +30396,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -30510,7 +30510,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -30624,7 +30624,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:18 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -30652,10 +30652,10 @@
         <v>1</v>
       </c>
       <c r="I261" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J261" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K261" t="inlineStr">
         <is>
@@ -30747,7 +30747,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:18 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -30775,10 +30775,10 @@
         <v>1</v>
       </c>
       <c r="I262" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J262" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K262" t="inlineStr">
         <is>
@@ -30870,7 +30870,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:18 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -30898,10 +30898,10 @@
         <v>1</v>
       </c>
       <c r="I263" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J263" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K263" t="inlineStr">
         <is>
@@ -30993,7 +30993,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:18 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -31021,10 +31021,10 @@
         <v>1</v>
       </c>
       <c r="I264" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J264" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K264" t="inlineStr">
         <is>
@@ -31116,7 +31116,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -31230,7 +31230,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -31344,7 +31344,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -31458,7 +31458,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -31572,7 +31572,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -31686,7 +31686,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -31800,7 +31800,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:15 PM PT</t>
+          <t>2026-07-12 03:19:30 PM PT</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -31914,7 +31914,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:15 PM PT</t>
+          <t>2026-07-12 03:19:30 PM PT</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -32028,7 +32028,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:15 PM PT</t>
+          <t>2026-07-12 03:19:30 PM PT</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -32142,7 +32142,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -32256,7 +32256,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -32370,7 +32370,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -32598,7 +32598,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -32712,7 +32712,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C279" t="n">
@@ -32826,7 +32826,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -32940,7 +32940,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C281" t="n">
@@ -33054,7 +33054,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C282" t="n">
@@ -33168,7 +33168,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -33282,7 +33282,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -33396,7 +33396,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -33510,7 +33510,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -33624,7 +33624,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -33738,7 +33738,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -33852,7 +33852,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -33966,7 +33966,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:15 PM PT</t>
+          <t>2026-07-12 03:19:30 PM PT</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -34080,7 +34080,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:15 PM PT</t>
+          <t>2026-07-12 03:19:30 PM PT</t>
         </is>
       </c>
       <c r="C291" t="n">
@@ -34194,7 +34194,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:15 PM PT</t>
+          <t>2026-07-12 03:19:30 PM PT</t>
         </is>
       </c>
       <c r="C292" t="n">
@@ -34308,7 +34308,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:18 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C293" t="n">
@@ -34321,7 +34321,7 @@
       </c>
       <c r="E293" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 1 out</t>
         </is>
       </c>
       <c r="F293" t="n">
@@ -34333,13 +34333,13 @@
         </is>
       </c>
       <c r="H293" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I293" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J293" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K293" t="inlineStr">
         <is>
@@ -34431,7 +34431,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:18 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C294" t="n">
@@ -34444,7 +34444,7 @@
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 1 out</t>
         </is>
       </c>
       <c r="F294" t="n">
@@ -34456,13 +34456,13 @@
         </is>
       </c>
       <c r="H294" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I294" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J294" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K294" t="inlineStr">
         <is>
@@ -34554,7 +34554,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:18 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C295" t="n">
@@ -34567,7 +34567,7 @@
       </c>
       <c r="E295" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 1 out</t>
         </is>
       </c>
       <c r="F295" t="n">
@@ -34579,13 +34579,13 @@
         </is>
       </c>
       <c r="H295" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I295" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J295" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K295" t="inlineStr">
         <is>
@@ -34677,7 +34677,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:18 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C296" t="n">
@@ -34690,7 +34690,7 @@
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 1 out</t>
         </is>
       </c>
       <c r="F296" t="n">
@@ -34702,13 +34702,13 @@
         </is>
       </c>
       <c r="H296" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I296" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J296" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K296" t="inlineStr">
         <is>
@@ -34800,7 +34800,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -34914,7 +34914,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -34942,10 +34942,10 @@
         <v>0</v>
       </c>
       <c r="I298" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J298" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K298" t="inlineStr">
         <is>
@@ -35037,7 +35037,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C299" t="n">
@@ -35151,7 +35151,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C300" t="n">
@@ -35265,7 +35265,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C301" t="n">
@@ -35379,7 +35379,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C302" t="n">
@@ -35493,7 +35493,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C303" t="n">
@@ -35607,7 +35607,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C304" t="n">
@@ -35721,7 +35721,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C305" t="n">
@@ -35835,7 +35835,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C306" t="n">
@@ -35949,7 +35949,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C307" t="n">
@@ -36063,7 +36063,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C308" t="n">
@@ -36177,7 +36177,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:17 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C309" t="n">
@@ -36291,7 +36291,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:18 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -36304,7 +36304,7 @@
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 1 out</t>
         </is>
       </c>
       <c r="F310" t="n">
@@ -36316,13 +36316,13 @@
         </is>
       </c>
       <c r="H310" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I310" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J310" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K310" t="inlineStr">
         <is>
@@ -36414,7 +36414,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:18 PM PT</t>
+          <t>2026-07-12 03:19:32 PM PT</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -36427,7 +36427,7 @@
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 1 out</t>
         </is>
       </c>
       <c r="F311" t="n">
@@ -36439,13 +36439,13 @@
         </is>
       </c>
       <c r="H311" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I311" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J311" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K311" t="inlineStr">
         <is>
@@ -36537,7 +36537,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -36651,7 +36651,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -36765,7 +36765,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -36879,7 +36879,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C315" t="n">
@@ -36993,7 +36993,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>2026-07-12 03:18:16 PM PT</t>
+          <t>2026-07-12 03:19:31 PM PT</t>
         </is>
       </c>
       <c r="C316" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-12 03:25:35 PM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
@@ -487,7 +487,7 @@
     <col width="27" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
@@ -693,7 +693,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -807,7 +807,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -921,7 +921,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1405,7 +1405,7 @@
         <v>2</v>
       </c>
       <c r="I8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J8" t="n">
         <v>2</v>
@@ -1500,7 +1500,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1513,7 +1513,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Top 7 | 2 out</t>
+          <t>Bottom 7 | 0 out</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -1521,17 +1521,17 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -1623,7 +1623,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1737,7 +1737,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1851,7 +1851,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1965,7 +1965,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2079,7 +2079,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2193,7 +2193,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2307,7 +2307,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2421,7 +2421,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2535,7 +2535,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2649,7 +2649,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2763,7 +2763,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2877,7 +2877,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2991,7 +2991,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3105,7 +3105,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3219,7 +3219,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3333,7 +3333,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3447,7 +3447,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3460,7 +3460,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Top 8 | 2 out</t>
+          <t>Bottom 8 | 0 out</t>
         </is>
       </c>
       <c r="F26" t="n">
@@ -3468,17 +3468,17 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H26" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I26" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
@@ -3570,7 +3570,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3684,7 +3684,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3798,7 +3798,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3912,7 +3912,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -4026,7 +4026,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4140,7 +4140,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4254,7 +4254,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4368,7 +4368,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4482,7 +4482,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4596,7 +4596,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4710,7 +4710,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4824,7 +4824,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4938,7 +4938,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5052,7 +5052,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5166,7 +5166,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5280,7 +5280,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5394,7 +5394,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5508,7 +5508,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5521,7 +5521,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Top 8 | 2 out</t>
+          <t>Bottom 8 | 0 out</t>
         </is>
       </c>
       <c r="F44" t="n">
@@ -5529,17 +5529,17 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H44" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I44" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J44" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K44" t="inlineStr">
         <is>
@@ -5631,7 +5631,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5745,7 +5745,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5859,7 +5859,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5973,7 +5973,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6087,7 +6087,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6201,7 +6201,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6315,7 +6315,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6328,7 +6328,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Top 7 | 2 out</t>
+          <t>Bottom 7 | 0 out</t>
         </is>
       </c>
       <c r="F51" t="n">
@@ -6336,17 +6336,17 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H51" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I51" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J51" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K51" t="inlineStr">
         <is>
@@ -6438,7 +6438,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6552,7 +6552,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6666,7 +6666,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6780,7 +6780,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6894,7 +6894,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -7008,7 +7008,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7122,7 +7122,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7150,7 +7150,7 @@
         <v>2</v>
       </c>
       <c r="I58" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J58" t="n">
         <v>2</v>
@@ -7245,7 +7245,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7359,7 +7359,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7473,7 +7473,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7587,7 +7587,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7701,7 +7701,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7815,7 +7815,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7929,7 +7929,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -8043,7 +8043,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8157,7 +8157,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8170,7 +8170,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Top 8 | 2 out</t>
+          <t>Bottom 8 | 0 out</t>
         </is>
       </c>
       <c r="F67" t="n">
@@ -8178,17 +8178,17 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H67" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I67" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J67" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K67" t="inlineStr">
         <is>
@@ -8280,7 +8280,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8293,7 +8293,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Top 8 | 2 out</t>
+          <t>Bottom 8 | 0 out</t>
         </is>
       </c>
       <c r="F68" t="n">
@@ -8301,17 +8301,17 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H68" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I68" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K68" t="inlineStr">
         <is>
@@ -8403,7 +8403,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8517,7 +8517,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8530,7 +8530,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Top 7 | 2 out</t>
+          <t>Bottom 7 | 0 out</t>
         </is>
       </c>
       <c r="F70" t="n">
@@ -8538,17 +8538,17 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H70" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I70" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J70" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K70" t="inlineStr">
         <is>
@@ -8640,7 +8640,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8653,7 +8653,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Top 7 | 2 out</t>
+          <t>Bottom 7 | 0 out</t>
         </is>
       </c>
       <c r="F71" t="n">
@@ -8661,17 +8661,17 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H71" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I71" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J71" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K71" t="inlineStr">
         <is>
@@ -8763,7 +8763,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8877,7 +8877,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8991,7 +8991,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9105,7 +9105,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9219,7 +9219,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9333,7 +9333,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9447,7 +9447,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9561,7 +9561,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9675,7 +9675,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9789,7 +9789,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9903,7 +9903,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -10017,7 +10017,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10131,7 +10131,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10245,7 +10245,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10359,7 +10359,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10473,7 +10473,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10486,7 +10486,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Top 8 | 2 out</t>
+          <t>Bottom 8 | 0 out</t>
         </is>
       </c>
       <c r="F87" t="n">
@@ -10494,17 +10494,17 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H87" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I87" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J87" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K87" t="inlineStr">
         <is>
@@ -10596,7 +10596,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10710,7 +10710,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10723,7 +10723,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Top 8 | 2 out</t>
+          <t>Bottom 8 | 0 out</t>
         </is>
       </c>
       <c r="F89" t="n">
@@ -10731,17 +10731,17 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H89" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I89" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J89" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K89" t="inlineStr">
         <is>
@@ -10833,7 +10833,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10846,7 +10846,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Top 7 | 2 out</t>
+          <t>Bottom 7 | 0 out</t>
         </is>
       </c>
       <c r="F90" t="n">
@@ -10854,17 +10854,17 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H90" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I90" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J90" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K90" t="inlineStr">
         <is>
@@ -10956,7 +10956,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -11070,7 +11070,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11184,7 +11184,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11298,7 +11298,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11412,7 +11412,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11526,7 +11526,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11539,7 +11539,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Top 7 | 2 out</t>
+          <t>Bottom 7 | 0 out</t>
         </is>
       </c>
       <c r="F96" t="n">
@@ -11547,17 +11547,17 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H96" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I96" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J96" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K96" t="inlineStr">
         <is>
@@ -11649,7 +11649,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11763,7 +11763,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11877,7 +11877,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11991,7 +11991,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -12105,7 +12105,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12219,7 +12219,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12333,7 +12333,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12447,7 +12447,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12561,7 +12561,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12574,7 +12574,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Top 8 | 2 out</t>
+          <t>Bottom 8 | 0 out</t>
         </is>
       </c>
       <c r="F105" t="n">
@@ -12582,17 +12582,17 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H105" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I105" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J105" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K105" t="inlineStr">
         <is>
@@ -12684,7 +12684,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12712,7 +12712,7 @@
         <v>2</v>
       </c>
       <c r="I106" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J106" t="n">
         <v>2</v>
@@ -12807,7 +12807,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12835,7 +12835,7 @@
         <v>2</v>
       </c>
       <c r="I107" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J107" t="n">
         <v>2</v>
@@ -12930,7 +12930,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -13044,7 +13044,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13158,7 +13158,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13272,7 +13272,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13285,7 +13285,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>Top 8 | 2 out</t>
+          <t>Bottom 8 | 0 out</t>
         </is>
       </c>
       <c r="F111" t="n">
@@ -13293,17 +13293,17 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H111" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I111" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J111" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K111" t="inlineStr">
         <is>
@@ -13339,10 +13339,10 @@
         </is>
       </c>
       <c r="R111" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S111" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T111" t="n">
         <v>1</v>
@@ -13395,7 +13395,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13509,7 +13509,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13623,7 +13623,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13737,7 +13737,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13765,7 +13765,7 @@
         <v>2</v>
       </c>
       <c r="I115" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J115" t="n">
         <v>2</v>
@@ -13860,7 +13860,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13974,7 +13974,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -14088,7 +14088,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14202,7 +14202,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14230,7 +14230,7 @@
         <v>2</v>
       </c>
       <c r="I119" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J119" t="n">
         <v>2</v>
@@ -14325,7 +14325,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14439,7 +14439,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14553,7 +14553,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14667,7 +14667,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14781,7 +14781,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14895,7 +14895,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -15009,7 +15009,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -15123,7 +15123,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15237,7 +15237,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15351,7 +15351,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15465,7 +15465,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15579,7 +15579,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15693,7 +15693,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15807,7 +15807,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15921,7 +15921,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -16035,7 +16035,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16149,7 +16149,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16263,7 +16263,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16377,7 +16377,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16491,7 +16491,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16605,7 +16605,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16719,7 +16719,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16833,7 +16833,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16947,7 +16947,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -17061,7 +17061,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17175,7 +17175,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17289,7 +17289,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17403,7 +17403,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17517,7 +17517,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17631,7 +17631,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17644,7 +17644,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>Top 8 | 2 out</t>
+          <t>Bottom 8 | 0 out</t>
         </is>
       </c>
       <c r="F149" t="n">
@@ -17652,17 +17652,17 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H149" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I149" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J149" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K149" t="inlineStr">
         <is>
@@ -17754,7 +17754,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17868,7 +17868,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17896,7 +17896,7 @@
         <v>2</v>
       </c>
       <c r="I151" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J151" t="n">
         <v>2</v>
@@ -17991,7 +17991,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -18105,7 +18105,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18219,7 +18219,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18232,7 +18232,7 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>Top 7 | 2 out</t>
+          <t>Bottom 7 | 0 out</t>
         </is>
       </c>
       <c r="F154" t="n">
@@ -18240,17 +18240,17 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H154" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I154" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J154" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K154" t="inlineStr">
         <is>
@@ -18286,10 +18286,10 @@
         </is>
       </c>
       <c r="R154" t="n">
+        <v>4</v>
+      </c>
+      <c r="S154" t="n">
         <v>3</v>
-      </c>
-      <c r="S154" t="n">
-        <v>2</v>
       </c>
       <c r="T154" t="n">
         <v>0</v>
@@ -18342,7 +18342,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18456,7 +18456,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18570,7 +18570,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18684,7 +18684,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18697,7 +18697,7 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>Top 7 | 2 out</t>
+          <t>Bottom 7 | 0 out</t>
         </is>
       </c>
       <c r="F158" t="n">
@@ -18705,17 +18705,17 @@
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H158" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I158" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J158" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K158" t="inlineStr">
         <is>
@@ -18807,7 +18807,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18921,7 +18921,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -19035,7 +19035,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19048,7 +19048,7 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>Top 8 | 2 out</t>
+          <t>Bottom 8 | 0 out</t>
         </is>
       </c>
       <c r="F161" t="n">
@@ -19056,17 +19056,17 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H161" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I161" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J161" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K161" t="inlineStr">
         <is>
@@ -19158,7 +19158,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19171,7 +19171,7 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>Top 8 | 2 out</t>
+          <t>Bottom 8 | 0 out</t>
         </is>
       </c>
       <c r="F162" t="n">
@@ -19179,17 +19179,17 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H162" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I162" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J162" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K162" t="inlineStr">
         <is>
@@ -19281,7 +19281,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19395,7 +19395,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19423,7 +19423,7 @@
         <v>2</v>
       </c>
       <c r="I164" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J164" t="n">
         <v>2</v>
@@ -19518,7 +19518,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19546,7 +19546,7 @@
         <v>2</v>
       </c>
       <c r="I165" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J165" t="n">
         <v>2</v>
@@ -19641,7 +19641,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19755,7 +19755,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19869,7 +19869,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19983,7 +19983,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -20097,7 +20097,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -20211,7 +20211,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20325,7 +20325,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20439,7 +20439,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20553,7 +20553,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20667,7 +20667,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20781,7 +20781,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20809,7 +20809,7 @@
         <v>2</v>
       </c>
       <c r="I176" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J176" t="n">
         <v>2</v>
@@ -20904,7 +20904,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -21018,7 +21018,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -21132,7 +21132,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21246,7 +21246,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21360,7 +21360,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21474,7 +21474,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21588,7 +21588,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21702,7 +21702,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21730,7 +21730,7 @@
         <v>2</v>
       </c>
       <c r="I184" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J184" t="n">
         <v>2</v>
@@ -21825,7 +21825,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21939,7 +21939,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -22053,7 +22053,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -22167,7 +22167,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22180,7 +22180,7 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>Top 8 | 2 out</t>
+          <t>Bottom 8 | 0 out</t>
         </is>
       </c>
       <c r="F188" t="n">
@@ -22188,17 +22188,17 @@
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H188" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I188" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J188" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K188" t="inlineStr">
         <is>
@@ -22225,7 +22225,7 @@
       </c>
       <c r="P188" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>1B</t>
         </is>
       </c>
       <c r="Q188" t="inlineStr">
@@ -22290,7 +22290,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22404,7 +22404,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22518,7 +22518,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22632,7 +22632,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22746,7 +22746,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22860,7 +22860,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22974,7 +22974,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -23088,7 +23088,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -23202,7 +23202,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23316,7 +23316,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23430,7 +23430,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23458,7 +23458,7 @@
         <v>2</v>
       </c>
       <c r="I199" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J199" t="n">
         <v>2</v>
@@ -23553,7 +23553,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23581,7 +23581,7 @@
         <v>2</v>
       </c>
       <c r="I200" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J200" t="n">
         <v>2</v>
@@ -23676,7 +23676,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23790,7 +23790,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23904,7 +23904,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -24018,7 +24018,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -24132,7 +24132,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -24246,7 +24246,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24360,7 +24360,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24474,7 +24474,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24588,7 +24588,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24601,7 +24601,7 @@
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>Top 7 | 2 out</t>
+          <t>Bottom 7 | 0 out</t>
         </is>
       </c>
       <c r="F209" t="n">
@@ -24609,17 +24609,17 @@
       </c>
       <c r="G209" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H209" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I209" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J209" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K209" t="inlineStr">
         <is>
@@ -24711,7 +24711,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24724,7 +24724,7 @@
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>Top 7 | 2 out</t>
+          <t>Bottom 7 | 0 out</t>
         </is>
       </c>
       <c r="F210" t="n">
@@ -24732,17 +24732,17 @@
       </c>
       <c r="G210" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H210" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I210" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J210" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K210" t="inlineStr">
         <is>
@@ -24834,7 +24834,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24948,7 +24948,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -25062,7 +25062,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -25176,7 +25176,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -25290,7 +25290,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25404,7 +25404,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25518,7 +25518,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25632,7 +25632,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25660,7 +25660,7 @@
         <v>2</v>
       </c>
       <c r="I218" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J218" t="n">
         <v>2</v>
@@ -25755,7 +25755,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25869,7 +25869,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25983,7 +25983,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -26097,7 +26097,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -26211,7 +26211,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26224,7 +26224,7 @@
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>Top 8 | 2 out</t>
+          <t>Bottom 8 | 0 out</t>
         </is>
       </c>
       <c r="F223" t="n">
@@ -26232,17 +26232,17 @@
       </c>
       <c r="G223" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H223" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I223" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J223" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K223" t="inlineStr">
         <is>
@@ -26334,7 +26334,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26347,7 +26347,7 @@
       </c>
       <c r="E224" t="inlineStr">
         <is>
-          <t>Top 8 | 2 out</t>
+          <t>Bottom 8 | 0 out</t>
         </is>
       </c>
       <c r="F224" t="n">
@@ -26355,17 +26355,17 @@
       </c>
       <c r="G224" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H224" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I224" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J224" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K224" t="inlineStr">
         <is>
@@ -26392,7 +26392,7 @@
       </c>
       <c r="P224" t="inlineStr">
         <is>
-          <t>PH</t>
+          <t>C</t>
         </is>
       </c>
       <c r="Q224" t="inlineStr">
@@ -26457,7 +26457,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26571,7 +26571,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26584,7 +26584,7 @@
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>Top 7 | 2 out</t>
+          <t>Bottom 7 | 0 out</t>
         </is>
       </c>
       <c r="F226" t="n">
@@ -26592,17 +26592,17 @@
       </c>
       <c r="G226" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H226" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I226" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J226" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K226" t="inlineStr">
         <is>
@@ -26694,7 +26694,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26707,7 +26707,7 @@
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>Top 7 | 2 out</t>
+          <t>Bottom 7 | 0 out</t>
         </is>
       </c>
       <c r="F227" t="n">
@@ -26715,17 +26715,17 @@
       </c>
       <c r="G227" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H227" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I227" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J227" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K227" t="inlineStr">
         <is>
@@ -26817,7 +26817,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26830,7 +26830,7 @@
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>Top 7 | 2 out</t>
+          <t>Bottom 7 | 0 out</t>
         </is>
       </c>
       <c r="F228" t="n">
@@ -26838,17 +26838,17 @@
       </c>
       <c r="G228" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H228" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I228" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J228" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K228" t="inlineStr">
         <is>
@@ -26940,7 +26940,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26953,7 +26953,7 @@
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>Top 7 | 2 out</t>
+          <t>Bottom 7 | 0 out</t>
         </is>
       </c>
       <c r="F229" t="n">
@@ -26961,17 +26961,17 @@
       </c>
       <c r="G229" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H229" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I229" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J229" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K229" t="inlineStr">
         <is>
@@ -27063,7 +27063,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -27177,7 +27177,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -27291,7 +27291,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27405,7 +27405,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27519,7 +27519,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27633,7 +27633,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -27747,7 +27747,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -27861,7 +27861,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -27975,7 +27975,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -28089,7 +28089,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -28203,7 +28203,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -28317,7 +28317,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -28431,7 +28431,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -28459,7 +28459,7 @@
         <v>2</v>
       </c>
       <c r="I242" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J242" t="n">
         <v>2</v>
@@ -28554,7 +28554,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -28582,7 +28582,7 @@
         <v>2</v>
       </c>
       <c r="I243" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J243" t="n">
         <v>2</v>
@@ -28677,7 +28677,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -28705,7 +28705,7 @@
         <v>2</v>
       </c>
       <c r="I244" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J244" t="n">
         <v>2</v>
@@ -28800,7 +28800,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -28828,7 +28828,7 @@
         <v>2</v>
       </c>
       <c r="I245" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J245" t="n">
         <v>2</v>
@@ -28923,7 +28923,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -29037,7 +29037,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -29151,7 +29151,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -29265,7 +29265,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -29379,7 +29379,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -29493,7 +29493,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -29607,7 +29607,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -29721,7 +29721,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -29835,7 +29835,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -29949,7 +29949,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -30063,7 +30063,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -30177,7 +30177,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -30291,7 +30291,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -30405,7 +30405,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -30519,7 +30519,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -30633,7 +30633,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -30747,7 +30747,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -30760,7 +30760,7 @@
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t>Top 7 | 2 out</t>
+          <t>Bottom 7 | 0 out</t>
         </is>
       </c>
       <c r="F262" t="n">
@@ -30768,17 +30768,17 @@
       </c>
       <c r="G262" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H262" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I262" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J262" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K262" t="inlineStr">
         <is>
@@ -30870,7 +30870,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -30883,7 +30883,7 @@
       </c>
       <c r="E263" t="inlineStr">
         <is>
-          <t>Top 7 | 2 out</t>
+          <t>Bottom 7 | 0 out</t>
         </is>
       </c>
       <c r="F263" t="n">
@@ -30891,17 +30891,17 @@
       </c>
       <c r="G263" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H263" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I263" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J263" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K263" t="inlineStr">
         <is>
@@ -30993,7 +30993,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -31006,7 +31006,7 @@
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t>Top 7 | 2 out</t>
+          <t>Bottom 7 | 0 out</t>
         </is>
       </c>
       <c r="F264" t="n">
@@ -31014,17 +31014,17 @@
       </c>
       <c r="G264" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H264" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I264" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J264" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K264" t="inlineStr">
         <is>
@@ -31116,7 +31116,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -31129,7 +31129,7 @@
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t>Top 7 | 2 out</t>
+          <t>Bottom 7 | 0 out</t>
         </is>
       </c>
       <c r="F265" t="n">
@@ -31137,17 +31137,17 @@
       </c>
       <c r="G265" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H265" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I265" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J265" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K265" t="inlineStr">
         <is>
@@ -31239,7 +31239,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -31353,7 +31353,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -31467,7 +31467,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -31581,7 +31581,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -31695,7 +31695,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -31809,7 +31809,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -31923,7 +31923,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -32037,7 +32037,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -32151,7 +32151,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -32265,7 +32265,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -32379,7 +32379,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -32493,7 +32493,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -32607,7 +32607,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -32721,7 +32721,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C279" t="n">
@@ -32835,7 +32835,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -32949,7 +32949,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C281" t="n">
@@ -33063,7 +33063,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C282" t="n">
@@ -33177,7 +33177,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -33291,7 +33291,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -33405,7 +33405,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -33519,7 +33519,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -33633,7 +33633,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -33747,7 +33747,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -33861,7 +33861,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -33975,7 +33975,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -34089,7 +34089,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C291" t="n">
@@ -34203,7 +34203,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C292" t="n">
@@ -34317,7 +34317,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:30 PM PT</t>
+          <t>2026-07-12 03:25:30 PM PT</t>
         </is>
       </c>
       <c r="C293" t="n">
@@ -34431,7 +34431,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C294" t="n">
@@ -34444,7 +34444,7 @@
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>Top 8 | 2 out</t>
+          <t>Bottom 8 | 0 out</t>
         </is>
       </c>
       <c r="F294" t="n">
@@ -34452,17 +34452,17 @@
       </c>
       <c r="G294" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H294" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I294" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J294" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K294" t="inlineStr">
         <is>
@@ -34554,7 +34554,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C295" t="n">
@@ -34567,7 +34567,7 @@
       </c>
       <c r="E295" t="inlineStr">
         <is>
-          <t>Top 8 | 2 out</t>
+          <t>Bottom 8 | 0 out</t>
         </is>
       </c>
       <c r="F295" t="n">
@@ -34575,17 +34575,17 @@
       </c>
       <c r="G295" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H295" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I295" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J295" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K295" t="inlineStr">
         <is>
@@ -34677,7 +34677,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C296" t="n">
@@ -34690,7 +34690,7 @@
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t>Top 8 | 2 out</t>
+          <t>Bottom 8 | 0 out</t>
         </is>
       </c>
       <c r="F296" t="n">
@@ -34698,17 +34698,17 @@
       </c>
       <c r="G296" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H296" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I296" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J296" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K296" t="inlineStr">
         <is>
@@ -34800,7 +34800,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -34813,7 +34813,7 @@
       </c>
       <c r="E297" t="inlineStr">
         <is>
-          <t>Top 8 | 2 out</t>
+          <t>Bottom 8 | 0 out</t>
         </is>
       </c>
       <c r="F297" t="n">
@@ -34821,17 +34821,17 @@
       </c>
       <c r="G297" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H297" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I297" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J297" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K297" t="inlineStr">
         <is>
@@ -34923,7 +34923,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -35037,7 +35037,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C299" t="n">
@@ -35065,7 +35065,7 @@
         <v>2</v>
       </c>
       <c r="I299" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J299" t="n">
         <v>2</v>
@@ -35160,7 +35160,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C300" t="n">
@@ -35274,7 +35274,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C301" t="n">
@@ -35388,7 +35388,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C302" t="n">
@@ -35502,7 +35502,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C303" t="n">
@@ -35616,7 +35616,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C304" t="n">
@@ -35730,7 +35730,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C305" t="n">
@@ -35844,7 +35844,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C306" t="n">
@@ -35958,7 +35958,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C307" t="n">
@@ -36072,7 +36072,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C308" t="n">
@@ -36186,7 +36186,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C309" t="n">
@@ -36300,7 +36300,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -36414,7 +36414,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -36427,7 +36427,7 @@
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t>Top 8 | 2 out</t>
+          <t>Bottom 8 | 0 out</t>
         </is>
       </c>
       <c r="F311" t="n">
@@ -36435,17 +36435,17 @@
       </c>
       <c r="G311" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H311" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I311" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J311" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K311" t="inlineStr">
         <is>
@@ -36537,7 +36537,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:32 PM PT</t>
+          <t>2026-07-12 03:25:32 PM PT</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -36550,7 +36550,7 @@
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>Top 8 | 2 out</t>
+          <t>Bottom 8 | 0 out</t>
         </is>
       </c>
       <c r="F312" t="n">
@@ -36558,17 +36558,17 @@
       </c>
       <c r="G312" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H312" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I312" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J312" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K312" t="inlineStr">
         <is>
@@ -36660,7 +36660,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -36774,7 +36774,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -36888,7 +36888,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C315" t="n">
@@ -37002,7 +37002,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C316" t="n">
@@ -37116,7 +37116,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>2026-07-12 03:23:31 PM PT</t>
+          <t>2026-07-12 03:25:31 PM PT</t>
         </is>
       </c>
       <c r="C317" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-12 03:27:33 PM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -807,7 +807,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -921,7 +921,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1405,7 +1405,7 @@
         <v>2</v>
       </c>
       <c r="I8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J8" t="n">
         <v>2</v>
@@ -1500,7 +1500,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:32 PM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1513,7 +1513,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Bottom 7 | 0 out</t>
+          <t>Bottom 7 | 1 out</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -1525,7 +1525,7 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
@@ -1623,7 +1623,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1737,7 +1737,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1851,7 +1851,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1965,7 +1965,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2079,7 +2079,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2193,7 +2193,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2307,7 +2307,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2421,7 +2421,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2535,7 +2535,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2649,7 +2649,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2763,7 +2763,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2877,7 +2877,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2991,7 +2991,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3105,7 +3105,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3219,7 +3219,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3333,7 +3333,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3447,7 +3447,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:32 PM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3475,10 +3475,10 @@
         <v>0</v>
       </c>
       <c r="I26" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J26" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
@@ -3570,7 +3570,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3684,7 +3684,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3798,7 +3798,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3912,7 +3912,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -4026,7 +4026,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4140,7 +4140,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4254,7 +4254,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4368,7 +4368,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4482,7 +4482,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4596,7 +4596,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4710,7 +4710,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4824,7 +4824,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4938,7 +4938,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5052,7 +5052,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5166,7 +5166,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5280,7 +5280,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5394,7 +5394,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5508,7 +5508,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:32 PM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5536,10 +5536,10 @@
         <v>0</v>
       </c>
       <c r="I44" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J44" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K44" t="inlineStr">
         <is>
@@ -5631,7 +5631,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5745,7 +5745,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5859,7 +5859,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5973,7 +5973,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6087,7 +6087,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6201,7 +6201,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6315,7 +6315,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:32 PM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6328,7 +6328,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Bottom 7 | 0 out</t>
+          <t>Bottom 7 | 1 out</t>
         </is>
       </c>
       <c r="F51" t="n">
@@ -6340,7 +6340,7 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I51" t="n">
         <v>0</v>
@@ -6438,7 +6438,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6552,7 +6552,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6666,7 +6666,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6780,7 +6780,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6894,7 +6894,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -7008,7 +7008,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7122,7 +7122,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7150,7 +7150,7 @@
         <v>2</v>
       </c>
       <c r="I58" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J58" t="n">
         <v>2</v>
@@ -7245,7 +7245,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7359,7 +7359,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7473,7 +7473,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7587,7 +7587,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7701,7 +7701,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7815,7 +7815,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7929,7 +7929,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -8043,7 +8043,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8157,7 +8157,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:32 PM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8185,10 +8185,10 @@
         <v>0</v>
       </c>
       <c r="I67" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J67" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K67" t="inlineStr">
         <is>
@@ -8280,7 +8280,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:32 PM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8308,10 +8308,10 @@
         <v>0</v>
       </c>
       <c r="I68" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J68" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K68" t="inlineStr">
         <is>
@@ -8403,7 +8403,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8517,7 +8517,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:32 PM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8530,7 +8530,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Bottom 7 | 0 out</t>
+          <t>Bottom 7 | 1 out</t>
         </is>
       </c>
       <c r="F70" t="n">
@@ -8542,7 +8542,7 @@
         </is>
       </c>
       <c r="H70" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I70" t="n">
         <v>0</v>
@@ -8640,7 +8640,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:32 PM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8653,7 +8653,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Bottom 7 | 0 out</t>
+          <t>Bottom 7 | 1 out</t>
         </is>
       </c>
       <c r="F71" t="n">
@@ -8665,7 +8665,7 @@
         </is>
       </c>
       <c r="H71" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I71" t="n">
         <v>0</v>
@@ -8763,7 +8763,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8877,7 +8877,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8991,7 +8991,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9105,7 +9105,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9219,7 +9219,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9333,7 +9333,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9447,7 +9447,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9561,7 +9561,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9675,7 +9675,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9789,7 +9789,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9903,7 +9903,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -10017,7 +10017,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10131,7 +10131,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10245,7 +10245,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10359,7 +10359,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10473,7 +10473,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:32 PM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10501,10 +10501,10 @@
         <v>0</v>
       </c>
       <c r="I87" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J87" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K87" t="inlineStr">
         <is>
@@ -10596,7 +10596,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10710,7 +10710,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:32 PM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10738,10 +10738,10 @@
         <v>0</v>
       </c>
       <c r="I89" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J89" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K89" t="inlineStr">
         <is>
@@ -10833,7 +10833,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:32 PM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10846,7 +10846,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Bottom 7 | 0 out</t>
+          <t>Bottom 7 | 1 out</t>
         </is>
       </c>
       <c r="F90" t="n">
@@ -10858,7 +10858,7 @@
         </is>
       </c>
       <c r="H90" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I90" t="n">
         <v>0</v>
@@ -10956,7 +10956,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -11070,7 +11070,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11184,7 +11184,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11298,7 +11298,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11412,7 +11412,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11526,7 +11526,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:32 PM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11539,7 +11539,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Bottom 7 | 0 out</t>
+          <t>Bottom 7 | 1 out</t>
         </is>
       </c>
       <c r="F96" t="n">
@@ -11551,7 +11551,7 @@
         </is>
       </c>
       <c r="H96" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I96" t="n">
         <v>0</v>
@@ -11649,7 +11649,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11763,7 +11763,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11877,7 +11877,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11991,7 +11991,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -12105,7 +12105,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12219,7 +12219,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12333,7 +12333,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12447,7 +12447,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12561,7 +12561,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:32 PM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12589,10 +12589,10 @@
         <v>0</v>
       </c>
       <c r="I105" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J105" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K105" t="inlineStr">
         <is>
@@ -12684,7 +12684,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12712,7 +12712,7 @@
         <v>2</v>
       </c>
       <c r="I106" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J106" t="n">
         <v>2</v>
@@ -12807,7 +12807,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12835,7 +12835,7 @@
         <v>2</v>
       </c>
       <c r="I107" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J107" t="n">
         <v>2</v>
@@ -12930,7 +12930,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -13044,7 +13044,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13158,7 +13158,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13272,7 +13272,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:32 PM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13300,10 +13300,10 @@
         <v>0</v>
       </c>
       <c r="I111" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J111" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K111" t="inlineStr">
         <is>
@@ -13395,7 +13395,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13509,7 +13509,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13623,7 +13623,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13737,7 +13737,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13765,7 +13765,7 @@
         <v>2</v>
       </c>
       <c r="I115" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J115" t="n">
         <v>2</v>
@@ -13860,7 +13860,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13974,7 +13974,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -14088,7 +14088,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14202,7 +14202,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14230,7 +14230,7 @@
         <v>2</v>
       </c>
       <c r="I119" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J119" t="n">
         <v>2</v>
@@ -14325,7 +14325,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14439,7 +14439,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14553,7 +14553,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14667,7 +14667,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14781,7 +14781,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14895,7 +14895,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -15009,7 +15009,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -15123,7 +15123,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15237,7 +15237,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15351,7 +15351,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15465,7 +15465,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15579,7 +15579,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15693,7 +15693,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15807,7 +15807,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15921,7 +15921,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -16035,7 +16035,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16149,7 +16149,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16263,7 +16263,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16377,7 +16377,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16491,7 +16491,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16605,7 +16605,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16719,7 +16719,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16833,7 +16833,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16947,7 +16947,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -17061,7 +17061,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17175,7 +17175,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17289,7 +17289,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17403,7 +17403,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17517,7 +17517,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17631,7 +17631,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:32 PM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17659,10 +17659,10 @@
         <v>0</v>
       </c>
       <c r="I149" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J149" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K149" t="inlineStr">
         <is>
@@ -17754,7 +17754,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17868,7 +17868,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17896,7 +17896,7 @@
         <v>2</v>
       </c>
       <c r="I151" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J151" t="n">
         <v>2</v>
@@ -17991,7 +17991,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -18105,7 +18105,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18219,7 +18219,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:32 PM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18232,7 +18232,7 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>Bottom 7 | 0 out</t>
+          <t>Bottom 7 | 1 out</t>
         </is>
       </c>
       <c r="F154" t="n">
@@ -18244,7 +18244,7 @@
         </is>
       </c>
       <c r="H154" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I154" t="n">
         <v>0</v>
@@ -18342,7 +18342,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18456,7 +18456,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18570,7 +18570,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18684,7 +18684,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:32 PM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18697,7 +18697,7 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>Bottom 7 | 0 out</t>
+          <t>Bottom 7 | 1 out</t>
         </is>
       </c>
       <c r="F158" t="n">
@@ -18709,7 +18709,7 @@
         </is>
       </c>
       <c r="H158" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I158" t="n">
         <v>0</v>
@@ -18807,7 +18807,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18921,7 +18921,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -19035,7 +19035,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:32 PM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19063,10 +19063,10 @@
         <v>0</v>
       </c>
       <c r="I161" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J161" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K161" t="inlineStr">
         <is>
@@ -19158,7 +19158,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:32 PM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19186,10 +19186,10 @@
         <v>0</v>
       </c>
       <c r="I162" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J162" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K162" t="inlineStr">
         <is>
@@ -19281,7 +19281,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19395,7 +19395,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19423,7 +19423,7 @@
         <v>2</v>
       </c>
       <c r="I164" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J164" t="n">
         <v>2</v>
@@ -19518,7 +19518,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19546,7 +19546,7 @@
         <v>2</v>
       </c>
       <c r="I165" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J165" t="n">
         <v>2</v>
@@ -19641,7 +19641,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19755,7 +19755,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19869,7 +19869,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19983,7 +19983,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -20097,7 +20097,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -20211,7 +20211,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20325,7 +20325,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20439,7 +20439,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20553,7 +20553,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20667,7 +20667,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20781,7 +20781,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20809,7 +20809,7 @@
         <v>2</v>
       </c>
       <c r="I176" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J176" t="n">
         <v>2</v>
@@ -20904,7 +20904,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -21018,7 +21018,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -21132,7 +21132,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21246,7 +21246,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21360,7 +21360,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21474,7 +21474,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21588,7 +21588,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21702,7 +21702,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21730,7 +21730,7 @@
         <v>2</v>
       </c>
       <c r="I184" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J184" t="n">
         <v>2</v>
@@ -21825,7 +21825,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21939,7 +21939,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -22053,7 +22053,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -22167,7 +22167,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:32 PM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22195,10 +22195,10 @@
         <v>0</v>
       </c>
       <c r="I188" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J188" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K188" t="inlineStr">
         <is>
@@ -22290,7 +22290,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22404,7 +22404,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22518,7 +22518,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22632,7 +22632,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22746,7 +22746,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22860,7 +22860,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22974,7 +22974,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -23088,7 +23088,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -23202,7 +23202,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23316,7 +23316,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23430,7 +23430,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23458,7 +23458,7 @@
         <v>2</v>
       </c>
       <c r="I199" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J199" t="n">
         <v>2</v>
@@ -23553,7 +23553,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23581,7 +23581,7 @@
         <v>2</v>
       </c>
       <c r="I200" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J200" t="n">
         <v>2</v>
@@ -23676,7 +23676,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23790,7 +23790,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23904,7 +23904,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -24018,7 +24018,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -24132,7 +24132,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -24246,7 +24246,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24360,7 +24360,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24474,7 +24474,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24588,7 +24588,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:32 PM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24601,7 +24601,7 @@
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>Bottom 7 | 0 out</t>
+          <t>Bottom 7 | 1 out</t>
         </is>
       </c>
       <c r="F209" t="n">
@@ -24613,7 +24613,7 @@
         </is>
       </c>
       <c r="H209" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I209" t="n">
         <v>0</v>
@@ -24655,10 +24655,10 @@
         </is>
       </c>
       <c r="R209" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S209" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T209" t="n">
         <v>0</v>
@@ -24691,7 +24691,7 @@
         <v>0</v>
       </c>
       <c r="AD209" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AE209" s="5" t="n">
         <v>2</v>
@@ -24711,7 +24711,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:32 PM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24724,7 +24724,7 @@
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>Bottom 7 | 0 out</t>
+          <t>Bottom 7 | 1 out</t>
         </is>
       </c>
       <c r="F210" t="n">
@@ -24736,7 +24736,7 @@
         </is>
       </c>
       <c r="H210" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I210" t="n">
         <v>0</v>
@@ -24834,7 +24834,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24948,7 +24948,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -25062,7 +25062,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -25176,7 +25176,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -25290,7 +25290,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25404,7 +25404,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25518,7 +25518,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25632,7 +25632,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25660,7 +25660,7 @@
         <v>2</v>
       </c>
       <c r="I218" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J218" t="n">
         <v>2</v>
@@ -25755,7 +25755,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25869,7 +25869,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25983,7 +25983,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -26097,7 +26097,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -26211,7 +26211,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:32 PM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26239,10 +26239,10 @@
         <v>0</v>
       </c>
       <c r="I223" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J223" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K223" t="inlineStr">
         <is>
@@ -26334,7 +26334,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:32 PM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26362,10 +26362,10 @@
         <v>0</v>
       </c>
       <c r="I224" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J224" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K224" t="inlineStr">
         <is>
@@ -26457,7 +26457,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26571,7 +26571,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:32 PM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26584,7 +26584,7 @@
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>Bottom 7 | 0 out</t>
+          <t>Bottom 7 | 1 out</t>
         </is>
       </c>
       <c r="F226" t="n">
@@ -26596,7 +26596,7 @@
         </is>
       </c>
       <c r="H226" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I226" t="n">
         <v>0</v>
@@ -26694,7 +26694,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:32 PM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26707,7 +26707,7 @@
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>Bottom 7 | 0 out</t>
+          <t>Bottom 7 | 1 out</t>
         </is>
       </c>
       <c r="F227" t="n">
@@ -26719,7 +26719,7 @@
         </is>
       </c>
       <c r="H227" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I227" t="n">
         <v>0</v>
@@ -26817,7 +26817,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:32 PM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26830,7 +26830,7 @@
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>Bottom 7 | 0 out</t>
+          <t>Bottom 7 | 1 out</t>
         </is>
       </c>
       <c r="F228" t="n">
@@ -26842,7 +26842,7 @@
         </is>
       </c>
       <c r="H228" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I228" t="n">
         <v>0</v>
@@ -26940,7 +26940,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:32 PM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26953,7 +26953,7 @@
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>Bottom 7 | 0 out</t>
+          <t>Bottom 7 | 1 out</t>
         </is>
       </c>
       <c r="F229" t="n">
@@ -26965,7 +26965,7 @@
         </is>
       </c>
       <c r="H229" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I229" t="n">
         <v>0</v>
@@ -27063,7 +27063,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -27177,7 +27177,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -27291,7 +27291,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27405,7 +27405,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27519,7 +27519,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27633,7 +27633,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -27747,7 +27747,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -27861,7 +27861,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -27975,7 +27975,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -28089,7 +28089,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -28203,7 +28203,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -28317,7 +28317,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -28431,7 +28431,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -28459,7 +28459,7 @@
         <v>2</v>
       </c>
       <c r="I242" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J242" t="n">
         <v>2</v>
@@ -28554,7 +28554,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -28582,7 +28582,7 @@
         <v>2</v>
       </c>
       <c r="I243" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J243" t="n">
         <v>2</v>
@@ -28677,7 +28677,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -28705,7 +28705,7 @@
         <v>2</v>
       </c>
       <c r="I244" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J244" t="n">
         <v>2</v>
@@ -28800,7 +28800,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -28828,7 +28828,7 @@
         <v>2</v>
       </c>
       <c r="I245" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J245" t="n">
         <v>2</v>
@@ -28923,7 +28923,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -29037,7 +29037,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -29151,7 +29151,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -29265,7 +29265,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -29379,7 +29379,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -29493,7 +29493,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -29607,7 +29607,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -29721,7 +29721,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -29835,7 +29835,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -29949,7 +29949,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -30063,7 +30063,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -30177,7 +30177,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -30291,7 +30291,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -30405,7 +30405,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -30519,7 +30519,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -30633,7 +30633,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -30747,7 +30747,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:32 PM PT</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -30760,7 +30760,7 @@
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t>Bottom 7 | 0 out</t>
+          <t>Bottom 7 | 1 out</t>
         </is>
       </c>
       <c r="F262" t="n">
@@ -30772,7 +30772,7 @@
         </is>
       </c>
       <c r="H262" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I262" t="n">
         <v>0</v>
@@ -30870,7 +30870,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:32 PM PT</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -30883,7 +30883,7 @@
       </c>
       <c r="E263" t="inlineStr">
         <is>
-          <t>Bottom 7 | 0 out</t>
+          <t>Bottom 7 | 1 out</t>
         </is>
       </c>
       <c r="F263" t="n">
@@ -30895,7 +30895,7 @@
         </is>
       </c>
       <c r="H263" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I263" t="n">
         <v>0</v>
@@ -30993,7 +30993,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:32 PM PT</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -31006,7 +31006,7 @@
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t>Bottom 7 | 0 out</t>
+          <t>Bottom 7 | 1 out</t>
         </is>
       </c>
       <c r="F264" t="n">
@@ -31018,7 +31018,7 @@
         </is>
       </c>
       <c r="H264" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I264" t="n">
         <v>0</v>
@@ -31116,7 +31116,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:32 PM PT</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -31129,7 +31129,7 @@
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t>Bottom 7 | 0 out</t>
+          <t>Bottom 7 | 1 out</t>
         </is>
       </c>
       <c r="F265" t="n">
@@ -31141,7 +31141,7 @@
         </is>
       </c>
       <c r="H265" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I265" t="n">
         <v>0</v>
@@ -31239,7 +31239,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -31353,7 +31353,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -31467,7 +31467,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -31581,7 +31581,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -31695,7 +31695,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -31809,7 +31809,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -31923,7 +31923,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -32037,7 +32037,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -32151,7 +32151,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -32265,7 +32265,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -32379,7 +32379,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -32493,7 +32493,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -32607,7 +32607,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -32721,7 +32721,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C279" t="n">
@@ -32835,7 +32835,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -32949,7 +32949,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C281" t="n">
@@ -33063,7 +33063,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C282" t="n">
@@ -33177,7 +33177,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -33291,7 +33291,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -33405,7 +33405,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -33519,7 +33519,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -33633,7 +33633,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -33747,7 +33747,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -33861,7 +33861,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -33975,7 +33975,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -34089,7 +34089,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C291" t="n">
@@ -34203,7 +34203,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C292" t="n">
@@ -34317,7 +34317,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:30 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C293" t="n">
@@ -34431,7 +34431,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:32 PM PT</t>
         </is>
       </c>
       <c r="C294" t="n">
@@ -34459,10 +34459,10 @@
         <v>0</v>
       </c>
       <c r="I294" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J294" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K294" t="inlineStr">
         <is>
@@ -34554,7 +34554,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:32 PM PT</t>
         </is>
       </c>
       <c r="C295" t="n">
@@ -34582,10 +34582,10 @@
         <v>0</v>
       </c>
       <c r="I295" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J295" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K295" t="inlineStr">
         <is>
@@ -34677,7 +34677,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:32 PM PT</t>
         </is>
       </c>
       <c r="C296" t="n">
@@ -34705,10 +34705,10 @@
         <v>0</v>
       </c>
       <c r="I296" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J296" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K296" t="inlineStr">
         <is>
@@ -34800,7 +34800,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:32 PM PT</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -34828,10 +34828,10 @@
         <v>0</v>
       </c>
       <c r="I297" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J297" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K297" t="inlineStr">
         <is>
@@ -34923,7 +34923,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -35037,7 +35037,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C299" t="n">
@@ -35065,7 +35065,7 @@
         <v>2</v>
       </c>
       <c r="I299" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J299" t="n">
         <v>2</v>
@@ -35160,7 +35160,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C300" t="n">
@@ -35274,7 +35274,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C301" t="n">
@@ -35388,7 +35388,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C302" t="n">
@@ -35502,7 +35502,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C303" t="n">
@@ -35616,7 +35616,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C304" t="n">
@@ -35730,7 +35730,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C305" t="n">
@@ -35844,7 +35844,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C306" t="n">
@@ -35958,7 +35958,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C307" t="n">
@@ -36072,7 +36072,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C308" t="n">
@@ -36186,7 +36186,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C309" t="n">
@@ -36300,7 +36300,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:31 PM PT</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -36414,7 +36414,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:32 PM PT</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -36442,10 +36442,10 @@
         <v>0</v>
       </c>
       <c r="I311" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J311" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K311" t="inlineStr">
         <is>
@@ -36537,7 +36537,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:32 PM PT</t>
+          <t>2026-07-12 03:27:32 PM PT</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -36565,10 +36565,10 @@
         <v>0</v>
       </c>
       <c r="I312" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J312" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K312" t="inlineStr">
         <is>
@@ -36660,7 +36660,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -36774,7 +36774,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -36888,7 +36888,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C315" t="n">
@@ -37002,7 +37002,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C316" t="n">
@@ -37116,7 +37116,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>2026-07-12 03:25:31 PM PT</t>
+          <t>2026-07-12 03:27:30 PM PT</t>
         </is>
       </c>
       <c r="C317" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-12 03:31:35 PM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -807,7 +807,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:30 PM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -921,7 +921,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1519,10 +1519,10 @@
         <v>2</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -1614,7 +1614,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1728,7 +1728,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1842,7 +1842,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:30 PM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1956,7 +1956,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2070,7 +2070,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:30 PM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2184,7 +2184,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2298,7 +2298,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:30 PM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2412,7 +2412,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2640,7 +2640,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2754,7 +2754,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2868,7 +2868,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2982,7 +2982,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:30 PM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3096,7 +3096,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3324,7 +3324,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3438,7 +3438,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:32 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3466,10 +3466,10 @@
         <v>0</v>
       </c>
       <c r="I26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
@@ -3561,7 +3561,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3675,7 +3675,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3789,7 +3789,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3903,7 +3903,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -4017,7 +4017,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4131,7 +4131,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4245,7 +4245,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4359,7 +4359,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4473,7 +4473,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4587,7 +4587,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4701,7 +4701,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:30 PM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4815,7 +4815,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4929,7 +4929,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:30 PM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5043,7 +5043,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:30 PM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5157,7 +5157,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5271,7 +5271,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5385,7 +5385,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5499,7 +5499,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:32 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5527,10 +5527,10 @@
         <v>0</v>
       </c>
       <c r="I44" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K44" t="inlineStr">
         <is>
@@ -5622,7 +5622,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5736,7 +5736,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5850,7 +5850,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5964,7 +5964,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6078,7 +6078,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6192,7 +6192,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:30 PM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6306,7 +6306,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6334,10 +6334,10 @@
         <v>2</v>
       </c>
       <c r="I51" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J51" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K51" t="inlineStr">
         <is>
@@ -6429,7 +6429,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6543,7 +6543,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6657,7 +6657,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6771,7 +6771,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6885,7 +6885,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:30 PM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -6999,7 +6999,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7113,7 +7113,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7227,7 +7227,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7341,7 +7341,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7455,7 +7455,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7569,7 +7569,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7683,7 +7683,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7797,7 +7797,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7911,7 +7911,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -8025,7 +8025,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8139,7 +8139,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:32 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8167,10 +8167,10 @@
         <v>0</v>
       </c>
       <c r="I67" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J67" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K67" t="inlineStr">
         <is>
@@ -8262,7 +8262,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:32 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8290,10 +8290,10 @@
         <v>0</v>
       </c>
       <c r="I68" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K68" t="inlineStr">
         <is>
@@ -8385,7 +8385,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8499,7 +8499,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8527,10 +8527,10 @@
         <v>2</v>
       </c>
       <c r="I70" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J70" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K70" t="inlineStr">
         <is>
@@ -8622,7 +8622,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8650,10 +8650,10 @@
         <v>2</v>
       </c>
       <c r="I71" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J71" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K71" t="inlineStr">
         <is>
@@ -8745,7 +8745,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8859,7 +8859,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8973,7 +8973,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9087,7 +9087,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9201,7 +9201,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9315,7 +9315,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9429,7 +9429,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9543,7 +9543,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9657,7 +9657,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9771,7 +9771,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9885,7 +9885,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -9999,7 +9999,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10113,7 +10113,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10227,7 +10227,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10341,7 +10341,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10455,7 +10455,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:32 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10483,10 +10483,10 @@
         <v>0</v>
       </c>
       <c r="I87" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J87" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K87" t="inlineStr">
         <is>
@@ -10578,7 +10578,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:32 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10606,10 +10606,10 @@
         <v>0</v>
       </c>
       <c r="I88" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J88" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K88" t="inlineStr">
         <is>
@@ -10701,7 +10701,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10815,7 +10815,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:32 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10843,10 +10843,10 @@
         <v>0</v>
       </c>
       <c r="I90" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J90" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K90" t="inlineStr">
         <is>
@@ -10938,7 +10938,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -10966,10 +10966,10 @@
         <v>2</v>
       </c>
       <c r="I91" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J91" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K91" t="inlineStr">
         <is>
@@ -11061,7 +11061,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11175,7 +11175,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11289,7 +11289,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11403,7 +11403,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11517,7 +11517,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11631,7 +11631,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11659,10 +11659,10 @@
         <v>2</v>
       </c>
       <c r="I97" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J97" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K97" t="inlineStr">
         <is>
@@ -11754,7 +11754,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11868,7 +11868,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:30 PM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11982,7 +11982,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:30 PM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -12096,7 +12096,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:30 PM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12210,7 +12210,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:30 PM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12324,7 +12324,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12438,7 +12438,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12552,7 +12552,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12666,7 +12666,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:32 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12694,10 +12694,10 @@
         <v>0</v>
       </c>
       <c r="I106" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J106" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K106" t="inlineStr">
         <is>
@@ -12789,7 +12789,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12903,7 +12903,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -13017,7 +13017,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13131,7 +13131,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13245,7 +13245,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13359,7 +13359,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:32 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13387,10 +13387,10 @@
         <v>0</v>
       </c>
       <c r="I112" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J112" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K112" t="inlineStr">
         <is>
@@ -13482,7 +13482,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13596,7 +13596,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13710,7 +13710,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13824,7 +13824,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13938,7 +13938,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -14052,7 +14052,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14166,7 +14166,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14280,7 +14280,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14394,7 +14394,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14508,7 +14508,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14622,7 +14622,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14736,7 +14736,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14850,7 +14850,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14964,7 +14964,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -15078,7 +15078,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15192,7 +15192,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15306,7 +15306,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15420,7 +15420,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15534,7 +15534,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15648,7 +15648,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15762,7 +15762,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15876,7 +15876,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -15990,7 +15990,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16104,7 +16104,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16218,7 +16218,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16332,7 +16332,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16446,7 +16446,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16560,7 +16560,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16674,7 +16674,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16788,7 +16788,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16902,7 +16902,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -17016,7 +17016,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17130,7 +17130,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17244,7 +17244,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17358,7 +17358,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17472,7 +17472,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17586,7 +17586,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:30 PM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17700,7 +17700,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:32 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17728,10 +17728,10 @@
         <v>0</v>
       </c>
       <c r="I150" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J150" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K150" t="inlineStr">
         <is>
@@ -17823,7 +17823,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17937,7 +17937,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -18051,7 +18051,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18165,7 +18165,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18279,7 +18279,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18307,10 +18307,10 @@
         <v>2</v>
       </c>
       <c r="I155" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J155" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K155" t="inlineStr">
         <is>
@@ -18402,7 +18402,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18516,7 +18516,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18630,7 +18630,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18744,7 +18744,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18772,10 +18772,10 @@
         <v>2</v>
       </c>
       <c r="I159" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J159" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K159" t="inlineStr">
         <is>
@@ -18867,7 +18867,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18981,7 +18981,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19095,7 +19095,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:32 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19123,10 +19123,10 @@
         <v>0</v>
       </c>
       <c r="I162" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J162" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K162" t="inlineStr">
         <is>
@@ -19218,7 +19218,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:32 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19246,10 +19246,10 @@
         <v>0</v>
       </c>
       <c r="I163" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J163" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K163" t="inlineStr">
         <is>
@@ -19341,7 +19341,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19455,7 +19455,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19569,7 +19569,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19683,7 +19683,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19797,7 +19797,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19911,7 +19911,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -20025,7 +20025,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -20139,7 +20139,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20253,7 +20253,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20367,7 +20367,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20481,7 +20481,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20595,7 +20595,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20709,7 +20709,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20823,7 +20823,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20937,7 +20937,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -21051,7 +21051,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21165,7 +21165,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21279,7 +21279,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21393,7 +21393,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:30 PM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21507,7 +21507,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21621,7 +21621,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21735,7 +21735,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21849,7 +21849,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21963,7 +21963,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -22077,7 +22077,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22191,7 +22191,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:32 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22219,10 +22219,10 @@
         <v>0</v>
       </c>
       <c r="I189" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J189" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K189" t="inlineStr">
         <is>
@@ -22314,7 +22314,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22428,7 +22428,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22542,7 +22542,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22656,7 +22656,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22770,7 +22770,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22884,7 +22884,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -22998,7 +22998,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -23112,7 +23112,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23226,7 +23226,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23340,7 +23340,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23454,7 +23454,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23568,7 +23568,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23682,7 +23682,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23796,7 +23796,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23910,7 +23910,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -24024,7 +24024,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -24138,7 +24138,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24252,7 +24252,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24366,7 +24366,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24480,7 +24480,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24594,7 +24594,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24622,10 +24622,10 @@
         <v>2</v>
       </c>
       <c r="I210" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J210" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K210" t="inlineStr">
         <is>
@@ -24717,7 +24717,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24745,10 +24745,10 @@
         <v>2</v>
       </c>
       <c r="I211" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J211" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K211" t="inlineStr">
         <is>
@@ -24840,7 +24840,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -24954,7 +24954,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:30 PM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -25068,7 +25068,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -25182,7 +25182,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25296,7 +25296,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25410,7 +25410,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25524,7 +25524,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25638,7 +25638,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25752,7 +25752,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25866,7 +25866,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -25980,7 +25980,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -26094,7 +26094,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26208,7 +26208,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:32 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26236,10 +26236,10 @@
         <v>0</v>
       </c>
       <c r="I224" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J224" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K224" t="inlineStr">
         <is>
@@ -26331,7 +26331,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:32 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26359,10 +26359,10 @@
         <v>0</v>
       </c>
       <c r="I225" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J225" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K225" t="inlineStr">
         <is>
@@ -26454,7 +26454,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26568,7 +26568,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26596,10 +26596,10 @@
         <v>2</v>
       </c>
       <c r="I227" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J227" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K227" t="inlineStr">
         <is>
@@ -26691,7 +26691,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26719,10 +26719,10 @@
         <v>2</v>
       </c>
       <c r="I228" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J228" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K228" t="inlineStr">
         <is>
@@ -26814,7 +26814,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26842,10 +26842,10 @@
         <v>2</v>
       </c>
       <c r="I229" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J229" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K229" t="inlineStr">
         <is>
@@ -26937,7 +26937,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -26965,10 +26965,10 @@
         <v>2</v>
       </c>
       <c r="I230" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J230" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K230" t="inlineStr">
         <is>
@@ -27060,7 +27060,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -27174,7 +27174,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27288,7 +27288,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27402,7 +27402,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27516,7 +27516,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -27630,7 +27630,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -27744,7 +27744,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -27858,7 +27858,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -27972,7 +27972,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -28086,7 +28086,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -28200,7 +28200,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -28314,7 +28314,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -28428,7 +28428,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -28542,7 +28542,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -28656,7 +28656,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -28770,7 +28770,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -28884,7 +28884,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -28998,7 +28998,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -29112,7 +29112,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -29226,7 +29226,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -29340,7 +29340,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -29454,7 +29454,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -29568,7 +29568,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -29682,7 +29682,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -29796,7 +29796,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -29910,7 +29910,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -30024,7 +30024,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -30138,7 +30138,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -30252,7 +30252,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -30366,7 +30366,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -30480,7 +30480,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -30594,7 +30594,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -30708,7 +30708,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -30736,10 +30736,10 @@
         <v>2</v>
       </c>
       <c r="I263" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J263" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K263" t="inlineStr">
         <is>
@@ -30831,7 +30831,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -30859,10 +30859,10 @@
         <v>2</v>
       </c>
       <c r="I264" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J264" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K264" t="inlineStr">
         <is>
@@ -30954,7 +30954,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -30982,10 +30982,10 @@
         <v>2</v>
       </c>
       <c r="I265" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J265" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K265" t="inlineStr">
         <is>
@@ -31077,7 +31077,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -31105,10 +31105,10 @@
         <v>2</v>
       </c>
       <c r="I266" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J266" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K266" t="inlineStr">
         <is>
@@ -31200,7 +31200,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -31228,10 +31228,10 @@
         <v>2</v>
       </c>
       <c r="I267" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J267" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K267" t="inlineStr">
         <is>
@@ -31323,7 +31323,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -31437,7 +31437,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -31551,7 +31551,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -31665,7 +31665,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -31779,7 +31779,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -31893,7 +31893,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -32007,7 +32007,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:30 PM PT</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -32121,7 +32121,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:30 PM PT</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -32235,7 +32235,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:30 PM PT</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -32349,7 +32349,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -32463,7 +32463,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -32577,7 +32577,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C279" t="n">
@@ -32691,7 +32691,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -32805,7 +32805,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C281" t="n">
@@ -32919,7 +32919,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C282" t="n">
@@ -33033,7 +33033,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -33147,7 +33147,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -33261,7 +33261,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -33375,7 +33375,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -33489,7 +33489,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -33603,7 +33603,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -33717,7 +33717,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -33831,7 +33831,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -33945,7 +33945,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C291" t="n">
@@ -34059,7 +34059,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C292" t="n">
@@ -34173,7 +34173,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:30 PM PT</t>
         </is>
       </c>
       <c r="C293" t="n">
@@ -34287,7 +34287,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:30 PM PT</t>
         </is>
       </c>
       <c r="C294" t="n">
@@ -34401,7 +34401,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:30 PM PT</t>
         </is>
       </c>
       <c r="C295" t="n">
@@ -34515,7 +34515,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:32 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C296" t="n">
@@ -34543,10 +34543,10 @@
         <v>0</v>
       </c>
       <c r="I296" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J296" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K296" t="inlineStr">
         <is>
@@ -34638,7 +34638,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:32 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -34666,10 +34666,10 @@
         <v>0</v>
       </c>
       <c r="I297" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J297" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K297" t="inlineStr">
         <is>
@@ -34761,7 +34761,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:32 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -34789,10 +34789,10 @@
         <v>0</v>
       </c>
       <c r="I298" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J298" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K298" t="inlineStr">
         <is>
@@ -34884,7 +34884,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C299" t="n">
@@ -34998,7 +34998,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C300" t="n">
@@ -35112,7 +35112,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C301" t="n">
@@ -35226,7 +35226,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C302" t="n">
@@ -35340,7 +35340,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C303" t="n">
@@ -35454,7 +35454,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C304" t="n">
@@ -35568,7 +35568,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C305" t="n">
@@ -35682,7 +35682,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C306" t="n">
@@ -35796,7 +35796,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C307" t="n">
@@ -35910,7 +35910,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C308" t="n">
@@ -36024,7 +36024,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C309" t="n">
@@ -36138,7 +36138,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -36252,7 +36252,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:31 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -36366,7 +36366,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:32 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -36394,10 +36394,10 @@
         <v>0</v>
       </c>
       <c r="I312" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J312" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K312" t="inlineStr">
         <is>
@@ -36489,7 +36489,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:32 PM PT</t>
+          <t>2026-07-12 03:31:32 PM PT</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -36517,10 +36517,10 @@
         <v>0</v>
       </c>
       <c r="I313" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J313" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K313" t="inlineStr">
         <is>
@@ -36612,7 +36612,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -36726,7 +36726,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C315" t="n">
@@ -36840,7 +36840,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C316" t="n">
@@ -36954,7 +36954,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C317" t="n">
@@ -37068,7 +37068,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>2026-07-12 03:29:30 PM PT</t>
+          <t>2026-07-12 03:31:31 PM PT</t>
         </is>
       </c>
       <c r="C318" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-12 03:39:36 PM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -807,7 +807,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -921,7 +921,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 1 out</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -1516,13 +1516,13 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -1614,7 +1614,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1728,7 +1728,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1842,7 +1842,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1956,7 +1956,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2070,7 +2070,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2184,7 +2184,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2298,7 +2298,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2412,7 +2412,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2640,7 +2640,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2754,7 +2754,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2868,7 +2868,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2982,7 +2982,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3096,7 +3096,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3324,7 +3324,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3438,7 +3438,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3451,7 +3451,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Bottom 8 | 3 out</t>
         </is>
       </c>
       <c r="F26" t="n">
@@ -3463,13 +3463,13 @@
         </is>
       </c>
       <c r="H26" t="n">
+        <v>3</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" t="n">
         <v>2</v>
-      </c>
-      <c r="I26" t="n">
-        <v>0</v>
-      </c>
-      <c r="J26" t="n">
-        <v>1</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
@@ -3561,7 +3561,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3675,7 +3675,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3789,7 +3789,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3903,7 +3903,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -4017,7 +4017,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4131,7 +4131,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4245,7 +4245,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4359,7 +4359,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4473,7 +4473,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4587,7 +4587,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4701,7 +4701,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4815,7 +4815,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4929,7 +4929,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5043,7 +5043,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5157,7 +5157,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5271,7 +5271,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5385,7 +5385,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5499,7 +5499,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5512,7 +5512,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Bottom 8 | 3 out</t>
         </is>
       </c>
       <c r="F44" t="n">
@@ -5524,13 +5524,13 @@
         </is>
       </c>
       <c r="H44" t="n">
+        <v>3</v>
+      </c>
+      <c r="I44" t="n">
+        <v>0</v>
+      </c>
+      <c r="J44" t="n">
         <v>2</v>
-      </c>
-      <c r="I44" t="n">
-        <v>0</v>
-      </c>
-      <c r="J44" t="n">
-        <v>1</v>
       </c>
       <c r="K44" t="inlineStr">
         <is>
@@ -5622,7 +5622,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5736,7 +5736,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5850,7 +5850,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5964,7 +5964,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6078,7 +6078,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6192,7 +6192,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6306,7 +6306,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6319,7 +6319,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Bottom 8 | 3 out</t>
         </is>
       </c>
       <c r="F51" t="n">
@@ -6331,13 +6331,13 @@
         </is>
       </c>
       <c r="H51" t="n">
+        <v>3</v>
+      </c>
+      <c r="I51" t="n">
+        <v>0</v>
+      </c>
+      <c r="J51" t="n">
         <v>2</v>
-      </c>
-      <c r="I51" t="n">
-        <v>0</v>
-      </c>
-      <c r="J51" t="n">
-        <v>1</v>
       </c>
       <c r="K51" t="inlineStr">
         <is>
@@ -6429,7 +6429,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6442,7 +6442,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 1 out</t>
         </is>
       </c>
       <c r="F52" t="n">
@@ -6454,13 +6454,13 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I52" t="n">
         <v>0</v>
       </c>
       <c r="J52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K52" t="inlineStr">
         <is>
@@ -6552,7 +6552,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6666,7 +6666,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6780,7 +6780,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6894,7 +6894,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -7008,7 +7008,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7122,7 +7122,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7236,7 +7236,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7350,7 +7350,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7578,7 +7578,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7692,7 +7692,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7806,7 +7806,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7920,7 +7920,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -8034,7 +8034,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8148,7 +8148,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8161,7 +8161,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Bottom 8 | 3 out</t>
         </is>
       </c>
       <c r="F67" t="n">
@@ -8173,13 +8173,13 @@
         </is>
       </c>
       <c r="H67" t="n">
+        <v>3</v>
+      </c>
+      <c r="I67" t="n">
+        <v>0</v>
+      </c>
+      <c r="J67" t="n">
         <v>2</v>
-      </c>
-      <c r="I67" t="n">
-        <v>0</v>
-      </c>
-      <c r="J67" t="n">
-        <v>1</v>
       </c>
       <c r="K67" t="inlineStr">
         <is>
@@ -8271,7 +8271,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8385,7 +8385,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8398,7 +8398,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Bottom 8 | 3 out</t>
         </is>
       </c>
       <c r="F69" t="n">
@@ -8410,13 +8410,13 @@
         </is>
       </c>
       <c r="H69" t="n">
+        <v>3</v>
+      </c>
+      <c r="I69" t="n">
+        <v>0</v>
+      </c>
+      <c r="J69" t="n">
         <v>2</v>
-      </c>
-      <c r="I69" t="n">
-        <v>0</v>
-      </c>
-      <c r="J69" t="n">
-        <v>1</v>
       </c>
       <c r="K69" t="inlineStr">
         <is>
@@ -8508,7 +8508,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8521,7 +8521,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Bottom 8 | 3 out</t>
         </is>
       </c>
       <c r="F70" t="n">
@@ -8533,13 +8533,13 @@
         </is>
       </c>
       <c r="H70" t="n">
+        <v>3</v>
+      </c>
+      <c r="I70" t="n">
+        <v>0</v>
+      </c>
+      <c r="J70" t="n">
         <v>2</v>
-      </c>
-      <c r="I70" t="n">
-        <v>0</v>
-      </c>
-      <c r="J70" t="n">
-        <v>1</v>
       </c>
       <c r="K70" t="inlineStr">
         <is>
@@ -8631,7 +8631,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8745,7 +8745,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8758,7 +8758,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 1 out</t>
         </is>
       </c>
       <c r="F72" t="n">
@@ -8770,13 +8770,13 @@
         </is>
       </c>
       <c r="H72" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I72" t="n">
         <v>0</v>
       </c>
       <c r="J72" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K72" t="inlineStr">
         <is>
@@ -8868,7 +8868,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8881,7 +8881,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 1 out</t>
         </is>
       </c>
       <c r="F73" t="n">
@@ -8893,13 +8893,13 @@
         </is>
       </c>
       <c r="H73" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I73" t="n">
         <v>0</v>
       </c>
       <c r="J73" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K73" t="inlineStr">
         <is>
@@ -8991,7 +8991,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9105,7 +9105,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9219,7 +9219,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9333,7 +9333,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9447,7 +9447,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9561,7 +9561,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9675,7 +9675,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9789,7 +9789,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9802,7 +9802,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Bottom 8 | 3 out</t>
         </is>
       </c>
       <c r="F81" t="n">
@@ -9814,13 +9814,13 @@
         </is>
       </c>
       <c r="H81" t="n">
+        <v>3</v>
+      </c>
+      <c r="I81" t="n">
+        <v>0</v>
+      </c>
+      <c r="J81" t="n">
         <v>2</v>
-      </c>
-      <c r="I81" t="n">
-        <v>0</v>
-      </c>
-      <c r="J81" t="n">
-        <v>1</v>
       </c>
       <c r="K81" t="inlineStr">
         <is>
@@ -9912,7 +9912,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -10026,7 +10026,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10140,7 +10140,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10254,7 +10254,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10368,7 +10368,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10482,7 +10482,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10596,7 +10596,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10710,7 +10710,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10824,7 +10824,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10837,7 +10837,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Bottom 8 | 3 out</t>
         </is>
       </c>
       <c r="F90" t="n">
@@ -10849,13 +10849,13 @@
         </is>
       </c>
       <c r="H90" t="n">
+        <v>3</v>
+      </c>
+      <c r="I90" t="n">
+        <v>0</v>
+      </c>
+      <c r="J90" t="n">
         <v>2</v>
-      </c>
-      <c r="I90" t="n">
-        <v>0</v>
-      </c>
-      <c r="J90" t="n">
-        <v>1</v>
       </c>
       <c r="K90" t="inlineStr">
         <is>
@@ -10947,7 +10947,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -11061,7 +11061,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11074,7 +11074,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Bottom 8 | 3 out</t>
         </is>
       </c>
       <c r="F92" t="n">
@@ -11086,13 +11086,13 @@
         </is>
       </c>
       <c r="H92" t="n">
+        <v>3</v>
+      </c>
+      <c r="I92" t="n">
+        <v>0</v>
+      </c>
+      <c r="J92" t="n">
         <v>2</v>
-      </c>
-      <c r="I92" t="n">
-        <v>0</v>
-      </c>
-      <c r="J92" t="n">
-        <v>1</v>
       </c>
       <c r="K92" t="inlineStr">
         <is>
@@ -11184,7 +11184,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11197,7 +11197,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 1 out</t>
         </is>
       </c>
       <c r="F93" t="n">
@@ -11209,13 +11209,13 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I93" t="n">
         <v>0</v>
       </c>
       <c r="J93" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K93" t="inlineStr">
         <is>
@@ -11307,7 +11307,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11421,7 +11421,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11535,7 +11535,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11649,7 +11649,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11763,7 +11763,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11877,7 +11877,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11890,7 +11890,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 1 out</t>
         </is>
       </c>
       <c r="F99" t="n">
@@ -11902,13 +11902,13 @@
         </is>
       </c>
       <c r="H99" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I99" t="n">
         <v>0</v>
       </c>
       <c r="J99" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K99" t="inlineStr">
         <is>
@@ -12000,7 +12000,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -12114,7 +12114,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12228,7 +12228,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12342,7 +12342,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12456,7 +12456,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12570,7 +12570,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12684,7 +12684,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12798,7 +12798,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12912,7 +12912,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12925,7 +12925,7 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Bottom 8 | 3 out</t>
         </is>
       </c>
       <c r="F108" t="n">
@@ -12937,13 +12937,13 @@
         </is>
       </c>
       <c r="H108" t="n">
+        <v>3</v>
+      </c>
+      <c r="I108" t="n">
+        <v>0</v>
+      </c>
+      <c r="J108" t="n">
         <v>2</v>
-      </c>
-      <c r="I108" t="n">
-        <v>0</v>
-      </c>
-      <c r="J108" t="n">
-        <v>1</v>
       </c>
       <c r="K108" t="inlineStr">
         <is>
@@ -13035,7 +13035,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13149,7 +13149,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13263,7 +13263,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13377,7 +13377,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13491,7 +13491,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13605,7 +13605,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13618,7 +13618,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Bottom 8 | 3 out</t>
         </is>
       </c>
       <c r="F114" t="n">
@@ -13630,13 +13630,13 @@
         </is>
       </c>
       <c r="H114" t="n">
+        <v>3</v>
+      </c>
+      <c r="I114" t="n">
+        <v>0</v>
+      </c>
+      <c r="J114" t="n">
         <v>2</v>
-      </c>
-      <c r="I114" t="n">
-        <v>0</v>
-      </c>
-      <c r="J114" t="n">
-        <v>1</v>
       </c>
       <c r="K114" t="inlineStr">
         <is>
@@ -13728,7 +13728,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13842,7 +13842,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13956,7 +13956,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -14070,7 +14070,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14184,7 +14184,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14298,7 +14298,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14412,7 +14412,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14526,7 +14526,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14640,7 +14640,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14754,7 +14754,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14868,7 +14868,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14982,7 +14982,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -15096,7 +15096,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15210,7 +15210,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15324,7 +15324,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15438,7 +15438,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15552,7 +15552,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15666,7 +15666,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15780,7 +15780,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15894,7 +15894,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -16008,7 +16008,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16122,7 +16122,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16236,7 +16236,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16350,7 +16350,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16464,7 +16464,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16578,7 +16578,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16692,7 +16692,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16806,7 +16806,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16920,7 +16920,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -17034,7 +17034,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17148,7 +17148,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17262,7 +17262,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17376,7 +17376,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17490,7 +17490,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17604,7 +17604,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17718,7 +17718,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17832,7 +17832,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17946,7 +17946,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -18060,7 +18060,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18174,7 +18174,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18288,7 +18288,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18402,7 +18402,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18415,7 +18415,7 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 1 out</t>
         </is>
       </c>
       <c r="F156" t="n">
@@ -18427,13 +18427,13 @@
         </is>
       </c>
       <c r="H156" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I156" t="n">
         <v>0</v>
       </c>
       <c r="J156" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K156" t="inlineStr">
         <is>
@@ -18525,7 +18525,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18639,7 +18639,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18753,7 +18753,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18867,7 +18867,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18880,7 +18880,7 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 1 out</t>
         </is>
       </c>
       <c r="F160" t="n">
@@ -18892,13 +18892,13 @@
         </is>
       </c>
       <c r="H160" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I160" t="n">
         <v>0</v>
       </c>
       <c r="J160" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K160" t="inlineStr">
         <is>
@@ -18990,7 +18990,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19104,7 +19104,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19218,7 +19218,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19231,7 +19231,7 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Bottom 8 | 3 out</t>
         </is>
       </c>
       <c r="F163" t="n">
@@ -19243,13 +19243,13 @@
         </is>
       </c>
       <c r="H163" t="n">
+        <v>3</v>
+      </c>
+      <c r="I163" t="n">
+        <v>0</v>
+      </c>
+      <c r="J163" t="n">
         <v>2</v>
-      </c>
-      <c r="I163" t="n">
-        <v>0</v>
-      </c>
-      <c r="J163" t="n">
-        <v>1</v>
       </c>
       <c r="K163" t="inlineStr">
         <is>
@@ -19341,7 +19341,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19354,7 +19354,7 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Bottom 8 | 3 out</t>
         </is>
       </c>
       <c r="F164" t="n">
@@ -19366,13 +19366,13 @@
         </is>
       </c>
       <c r="H164" t="n">
+        <v>3</v>
+      </c>
+      <c r="I164" t="n">
+        <v>0</v>
+      </c>
+      <c r="J164" t="n">
         <v>2</v>
-      </c>
-      <c r="I164" t="n">
-        <v>0</v>
-      </c>
-      <c r="J164" t="n">
-        <v>1</v>
       </c>
       <c r="K164" t="inlineStr">
         <is>
@@ -19464,7 +19464,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19578,7 +19578,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19692,7 +19692,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19806,7 +19806,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19920,7 +19920,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -20034,7 +20034,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -20148,7 +20148,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20262,7 +20262,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20376,7 +20376,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20490,7 +20490,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20604,7 +20604,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20718,7 +20718,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20832,7 +20832,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20946,7 +20946,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -21060,7 +21060,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21174,7 +21174,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21288,7 +21288,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21402,7 +21402,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21516,7 +21516,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21630,7 +21630,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21744,7 +21744,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21858,7 +21858,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21972,7 +21972,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -22086,7 +22086,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22200,7 +22200,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22314,7 +22314,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22327,7 +22327,7 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Bottom 8 | 3 out</t>
         </is>
       </c>
       <c r="F190" t="n">
@@ -22339,13 +22339,13 @@
         </is>
       </c>
       <c r="H190" t="n">
+        <v>3</v>
+      </c>
+      <c r="I190" t="n">
+        <v>0</v>
+      </c>
+      <c r="J190" t="n">
         <v>2</v>
-      </c>
-      <c r="I190" t="n">
-        <v>0</v>
-      </c>
-      <c r="J190" t="n">
-        <v>1</v>
       </c>
       <c r="K190" t="inlineStr">
         <is>
@@ -22437,7 +22437,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22551,7 +22551,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22665,7 +22665,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22779,7 +22779,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22893,7 +22893,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -23007,7 +23007,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -23121,7 +23121,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23235,7 +23235,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23349,7 +23349,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23463,7 +23463,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23577,7 +23577,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23691,7 +23691,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23805,7 +23805,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23919,7 +23919,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -24033,7 +24033,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -24147,7 +24147,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24261,7 +24261,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24375,7 +24375,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24489,7 +24489,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24603,7 +24603,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24717,7 +24717,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24730,7 +24730,7 @@
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 1 out</t>
         </is>
       </c>
       <c r="F211" t="n">
@@ -24742,13 +24742,13 @@
         </is>
       </c>
       <c r="H211" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I211" t="n">
         <v>0</v>
       </c>
       <c r="J211" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K211" t="inlineStr">
         <is>
@@ -24840,7 +24840,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -24853,7 +24853,7 @@
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 1 out</t>
         </is>
       </c>
       <c r="F212" t="n">
@@ -24865,13 +24865,13 @@
         </is>
       </c>
       <c r="H212" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I212" t="n">
         <v>0</v>
       </c>
       <c r="J212" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K212" t="inlineStr">
         <is>
@@ -24963,7 +24963,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -24976,7 +24976,7 @@
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 1 out</t>
         </is>
       </c>
       <c r="F213" t="n">
@@ -24988,13 +24988,13 @@
         </is>
       </c>
       <c r="H213" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I213" t="n">
         <v>0</v>
       </c>
       <c r="J213" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K213" t="inlineStr">
         <is>
@@ -25086,7 +25086,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -25200,7 +25200,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25314,7 +25314,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25428,7 +25428,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25542,7 +25542,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25656,7 +25656,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25770,7 +25770,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25884,7 +25884,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -25998,7 +25998,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -26112,7 +26112,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26226,7 +26226,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26340,7 +26340,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26454,7 +26454,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26467,7 +26467,7 @@
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Bottom 8 | 3 out</t>
         </is>
       </c>
       <c r="F226" t="n">
@@ -26479,13 +26479,13 @@
         </is>
       </c>
       <c r="H226" t="n">
+        <v>3</v>
+      </c>
+      <c r="I226" t="n">
+        <v>0</v>
+      </c>
+      <c r="J226" t="n">
         <v>2</v>
-      </c>
-      <c r="I226" t="n">
-        <v>0</v>
-      </c>
-      <c r="J226" t="n">
-        <v>1</v>
       </c>
       <c r="K226" t="inlineStr">
         <is>
@@ -26577,7 +26577,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26590,7 +26590,7 @@
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Bottom 8 | 3 out</t>
         </is>
       </c>
       <c r="F227" t="n">
@@ -26602,13 +26602,13 @@
         </is>
       </c>
       <c r="H227" t="n">
+        <v>3</v>
+      </c>
+      <c r="I227" t="n">
+        <v>0</v>
+      </c>
+      <c r="J227" t="n">
         <v>2</v>
-      </c>
-      <c r="I227" t="n">
-        <v>0</v>
-      </c>
-      <c r="J227" t="n">
-        <v>1</v>
       </c>
       <c r="K227" t="inlineStr">
         <is>
@@ -26700,7 +26700,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26814,7 +26814,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26827,7 +26827,7 @@
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 1 out</t>
         </is>
       </c>
       <c r="F229" t="n">
@@ -26839,13 +26839,13 @@
         </is>
       </c>
       <c r="H229" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I229" t="n">
         <v>0</v>
       </c>
       <c r="J229" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K229" t="inlineStr">
         <is>
@@ -26937,7 +26937,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -26950,7 +26950,7 @@
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 1 out</t>
         </is>
       </c>
       <c r="F230" t="n">
@@ -26962,13 +26962,13 @@
         </is>
       </c>
       <c r="H230" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I230" t="n">
         <v>0</v>
       </c>
       <c r="J230" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K230" t="inlineStr">
         <is>
@@ -27004,10 +27004,10 @@
         </is>
       </c>
       <c r="R230" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S230" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T230" t="n">
         <v>0</v>
@@ -27060,7 +27060,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -27073,7 +27073,7 @@
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 1 out</t>
         </is>
       </c>
       <c r="F231" t="n">
@@ -27085,13 +27085,13 @@
         </is>
       </c>
       <c r="H231" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I231" t="n">
         <v>0</v>
       </c>
       <c r="J231" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K231" t="inlineStr">
         <is>
@@ -27183,7 +27183,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27196,7 +27196,7 @@
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 1 out</t>
         </is>
       </c>
       <c r="F232" t="n">
@@ -27208,13 +27208,13 @@
         </is>
       </c>
       <c r="H232" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I232" t="n">
         <v>0</v>
       </c>
       <c r="J232" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K232" t="inlineStr">
         <is>
@@ -27306,7 +27306,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27420,7 +27420,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27534,7 +27534,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -27648,7 +27648,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -27762,7 +27762,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -27876,7 +27876,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -27990,7 +27990,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -28104,7 +28104,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -28218,7 +28218,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -28332,7 +28332,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -28446,7 +28446,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -28560,7 +28560,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -28674,7 +28674,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -28788,7 +28788,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -28902,7 +28902,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -29016,7 +29016,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -29130,7 +29130,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -29244,7 +29244,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -29358,7 +29358,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -29472,7 +29472,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -29586,7 +29586,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -29700,7 +29700,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -29814,7 +29814,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -29928,7 +29928,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -30042,7 +30042,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -30156,7 +30156,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -30270,7 +30270,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -30384,7 +30384,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -30498,7 +30498,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -30612,7 +30612,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -30726,7 +30726,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -30840,7 +30840,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -30954,7 +30954,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -30967,7 +30967,7 @@
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 1 out</t>
         </is>
       </c>
       <c r="F265" t="n">
@@ -30979,13 +30979,13 @@
         </is>
       </c>
       <c r="H265" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I265" t="n">
         <v>0</v>
       </c>
       <c r="J265" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K265" t="inlineStr">
         <is>
@@ -31077,7 +31077,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -31090,7 +31090,7 @@
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 1 out</t>
         </is>
       </c>
       <c r="F266" t="n">
@@ -31102,13 +31102,13 @@
         </is>
       </c>
       <c r="H266" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I266" t="n">
         <v>0</v>
       </c>
       <c r="J266" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K266" t="inlineStr">
         <is>
@@ -31200,7 +31200,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -31213,7 +31213,7 @@
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 1 out</t>
         </is>
       </c>
       <c r="F267" t="n">
@@ -31225,13 +31225,13 @@
         </is>
       </c>
       <c r="H267" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I267" t="n">
         <v>0</v>
       </c>
       <c r="J267" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K267" t="inlineStr">
         <is>
@@ -31323,7 +31323,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -31336,7 +31336,7 @@
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>Top 8 | 0 out</t>
+          <t>Top 8 | 1 out</t>
         </is>
       </c>
       <c r="F268" t="n">
@@ -31348,13 +31348,13 @@
         </is>
       </c>
       <c r="H268" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I268" t="n">
         <v>0</v>
       </c>
       <c r="J268" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K268" t="inlineStr">
         <is>
@@ -31446,7 +31446,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -31560,7 +31560,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -31674,7 +31674,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -31788,7 +31788,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -31902,7 +31902,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -32016,7 +32016,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -32130,7 +32130,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -32244,7 +32244,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -32358,7 +32358,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -32472,7 +32472,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -32586,7 +32586,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C279" t="n">
@@ -32700,7 +32700,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -32814,7 +32814,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C281" t="n">
@@ -32928,7 +32928,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C282" t="n">
@@ -33042,7 +33042,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -33156,7 +33156,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -33270,7 +33270,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -33384,7 +33384,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -33498,7 +33498,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -33612,7 +33612,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -33726,7 +33726,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -33840,7 +33840,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -33954,7 +33954,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C291" t="n">
@@ -34068,7 +34068,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C292" t="n">
@@ -34182,7 +34182,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C293" t="n">
@@ -34296,7 +34296,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C294" t="n">
@@ -34410,7 +34410,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C295" t="n">
@@ -34524,7 +34524,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:30 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C296" t="n">
@@ -34638,7 +34638,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -34651,7 +34651,7 @@
       </c>
       <c r="E297" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Bottom 8 | 3 out</t>
         </is>
       </c>
       <c r="F297" t="n">
@@ -34663,13 +34663,13 @@
         </is>
       </c>
       <c r="H297" t="n">
+        <v>3</v>
+      </c>
+      <c r="I297" t="n">
+        <v>0</v>
+      </c>
+      <c r="J297" t="n">
         <v>2</v>
-      </c>
-      <c r="I297" t="n">
-        <v>0</v>
-      </c>
-      <c r="J297" t="n">
-        <v>1</v>
       </c>
       <c r="K297" t="inlineStr">
         <is>
@@ -34761,7 +34761,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -34774,7 +34774,7 @@
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Bottom 8 | 3 out</t>
         </is>
       </c>
       <c r="F298" t="n">
@@ -34786,13 +34786,13 @@
         </is>
       </c>
       <c r="H298" t="n">
+        <v>3</v>
+      </c>
+      <c r="I298" t="n">
+        <v>0</v>
+      </c>
+      <c r="J298" t="n">
         <v>2</v>
-      </c>
-      <c r="I298" t="n">
-        <v>0</v>
-      </c>
-      <c r="J298" t="n">
-        <v>1</v>
       </c>
       <c r="K298" t="inlineStr">
         <is>
@@ -34884,7 +34884,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C299" t="n">
@@ -34897,7 +34897,7 @@
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Bottom 8 | 3 out</t>
         </is>
       </c>
       <c r="F299" t="n">
@@ -34909,13 +34909,13 @@
         </is>
       </c>
       <c r="H299" t="n">
+        <v>3</v>
+      </c>
+      <c r="I299" t="n">
+        <v>0</v>
+      </c>
+      <c r="J299" t="n">
         <v>2</v>
-      </c>
-      <c r="I299" t="n">
-        <v>0</v>
-      </c>
-      <c r="J299" t="n">
-        <v>1</v>
       </c>
       <c r="K299" t="inlineStr">
         <is>
@@ -34951,10 +34951,10 @@
         </is>
       </c>
       <c r="R299" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S299" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T299" t="n">
         <v>0</v>
@@ -35007,7 +35007,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C300" t="n">
@@ -35121,7 +35121,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C301" t="n">
@@ -35235,7 +35235,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C302" t="n">
@@ -35349,7 +35349,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C303" t="n">
@@ -35463,7 +35463,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C304" t="n">
@@ -35577,7 +35577,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C305" t="n">
@@ -35691,7 +35691,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:33 PM PT</t>
         </is>
       </c>
       <c r="C306" t="n">
@@ -35805,7 +35805,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C307" t="n">
@@ -35919,7 +35919,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C308" t="n">
@@ -36033,7 +36033,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:32 PM PT</t>
         </is>
       </c>
       <c r="C309" t="n">
@@ -36147,7 +36147,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -36261,7 +36261,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -36375,7 +36375,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -36489,7 +36489,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -36502,7 +36502,7 @@
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Bottom 8 | 3 out</t>
         </is>
       </c>
       <c r="F313" t="n">
@@ -36514,13 +36514,13 @@
         </is>
       </c>
       <c r="H313" t="n">
+        <v>3</v>
+      </c>
+      <c r="I313" t="n">
+        <v>0</v>
+      </c>
+      <c r="J313" t="n">
         <v>2</v>
-      </c>
-      <c r="I313" t="n">
-        <v>0</v>
-      </c>
-      <c r="J313" t="n">
-        <v>1</v>
       </c>
       <c r="K313" t="inlineStr">
         <is>
@@ -36612,7 +36612,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:32 PM PT</t>
+          <t>2026-07-12 03:39:34 PM PT</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -36625,7 +36625,7 @@
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Bottom 8 | 3 out</t>
         </is>
       </c>
       <c r="F314" t="n">
@@ -36637,13 +36637,13 @@
         </is>
       </c>
       <c r="H314" t="n">
+        <v>3</v>
+      </c>
+      <c r="I314" t="n">
+        <v>0</v>
+      </c>
+      <c r="J314" t="n">
         <v>2</v>
-      </c>
-      <c r="I314" t="n">
-        <v>0</v>
-      </c>
-      <c r="J314" t="n">
-        <v>1</v>
       </c>
       <c r="K314" t="inlineStr">
         <is>
@@ -36735,7 +36735,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C315" t="n">
@@ -36849,7 +36849,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C316" t="n">
@@ -36963,7 +36963,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C317" t="n">
@@ -37077,7 +37077,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C318" t="n">
@@ -37191,7 +37191,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>2026-07-12 03:37:31 PM PT</t>
+          <t>2026-07-12 03:39:31 PM PT</t>
         </is>
       </c>
       <c r="C319" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-12 03:41:36 PM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
@@ -487,7 +487,7 @@
     <col width="27" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
@@ -693,7 +693,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -807,7 +807,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -921,7 +921,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -1516,13 +1516,13 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -1614,7 +1614,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1728,7 +1728,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1842,7 +1842,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1956,7 +1956,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2070,7 +2070,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2184,7 +2184,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2298,7 +2298,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2412,7 +2412,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2640,7 +2640,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2754,7 +2754,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2868,7 +2868,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2982,7 +2982,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3096,7 +3096,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3324,7 +3324,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3438,7 +3438,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:35 PM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3451,25 +3451,25 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H26" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J26" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
@@ -3561,7 +3561,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3675,7 +3675,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3789,7 +3789,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3903,7 +3903,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -4017,7 +4017,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4131,7 +4131,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4245,7 +4245,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4359,7 +4359,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4473,7 +4473,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4587,7 +4587,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4701,7 +4701,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4815,7 +4815,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4929,7 +4929,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5043,7 +5043,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5157,7 +5157,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5271,7 +5271,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5385,7 +5385,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5499,7 +5499,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:35 PM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5512,25 +5512,25 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F44" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H44" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J44" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K44" t="inlineStr">
         <is>
@@ -5622,7 +5622,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5736,7 +5736,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5850,7 +5850,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5964,7 +5964,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6078,7 +6078,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6192,7 +6192,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6306,7 +6306,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:35 PM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6319,25 +6319,25 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F51" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H51" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I51" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J51" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K51" t="inlineStr">
         <is>
@@ -6429,7 +6429,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6442,7 +6442,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F52" t="n">
@@ -6454,13 +6454,13 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I52" t="n">
         <v>0</v>
       </c>
       <c r="J52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K52" t="inlineStr">
         <is>
@@ -6552,7 +6552,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6666,7 +6666,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6780,7 +6780,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6894,7 +6894,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -7008,7 +7008,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7122,7 +7122,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7236,7 +7236,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7350,7 +7350,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7578,7 +7578,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7692,7 +7692,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7806,7 +7806,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7920,7 +7920,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -8034,7 +8034,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8148,7 +8148,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:35 PM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8161,25 +8161,25 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F67" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H67" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I67" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J67" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K67" t="inlineStr">
         <is>
@@ -8271,7 +8271,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8385,7 +8385,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:35 PM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8398,25 +8398,25 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F69" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H69" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I69" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J69" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K69" t="inlineStr">
         <is>
@@ -8508,7 +8508,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:35 PM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8521,25 +8521,25 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F70" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H70" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I70" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J70" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K70" t="inlineStr">
         <is>
@@ -8631,7 +8631,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8745,7 +8745,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8758,7 +8758,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F72" t="n">
@@ -8770,13 +8770,13 @@
         </is>
       </c>
       <c r="H72" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I72" t="n">
         <v>0</v>
       </c>
       <c r="J72" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K72" t="inlineStr">
         <is>
@@ -8868,7 +8868,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8881,7 +8881,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F73" t="n">
@@ -8893,13 +8893,13 @@
         </is>
       </c>
       <c r="H73" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I73" t="n">
         <v>0</v>
       </c>
       <c r="J73" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K73" t="inlineStr">
         <is>
@@ -8991,7 +8991,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9105,7 +9105,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9219,7 +9219,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9333,7 +9333,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9447,7 +9447,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9561,7 +9561,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9675,7 +9675,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9789,7 +9789,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:35 PM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9802,25 +9802,25 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F81" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H81" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I81" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J81" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K81" t="inlineStr">
         <is>
@@ -9912,7 +9912,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -10026,7 +10026,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10140,7 +10140,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10254,7 +10254,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10368,7 +10368,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10482,7 +10482,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10596,7 +10596,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10710,7 +10710,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10824,7 +10824,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:35 PM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10837,25 +10837,25 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F90" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H90" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I90" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J90" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K90" t="inlineStr">
         <is>
@@ -10947,7 +10947,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -11061,7 +11061,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:35 PM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11074,25 +11074,25 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F92" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H92" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I92" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J92" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K92" t="inlineStr">
         <is>
@@ -11184,7 +11184,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11197,7 +11197,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F93" t="n">
@@ -11209,13 +11209,13 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I93" t="n">
         <v>0</v>
       </c>
       <c r="J93" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K93" t="inlineStr">
         <is>
@@ -11251,11 +11251,11 @@
         </is>
       </c>
       <c r="R93" t="n">
+        <v>4</v>
+      </c>
+      <c r="S93" t="n">
         <v>3</v>
       </c>
-      <c r="S93" t="n">
-        <v>2</v>
-      </c>
       <c r="T93" t="n">
         <v>1</v>
       </c>
@@ -11287,7 +11287,7 @@
         <v>0</v>
       </c>
       <c r="AD93" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE93" s="5" t="n">
         <v>7</v>
@@ -11307,7 +11307,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11421,7 +11421,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11535,7 +11535,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11649,7 +11649,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11763,7 +11763,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11877,7 +11877,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11890,7 +11890,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F99" t="n">
@@ -11902,13 +11902,13 @@
         </is>
       </c>
       <c r="H99" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I99" t="n">
         <v>0</v>
       </c>
       <c r="J99" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K99" t="inlineStr">
         <is>
@@ -12000,7 +12000,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -12114,7 +12114,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12228,7 +12228,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12342,7 +12342,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12456,7 +12456,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12570,7 +12570,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12684,7 +12684,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12798,7 +12798,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12912,7 +12912,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:35 PM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12925,25 +12925,25 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F108" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H108" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I108" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J108" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K108" t="inlineStr">
         <is>
@@ -12970,7 +12970,7 @@
       </c>
       <c r="P108" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>DH</t>
         </is>
       </c>
       <c r="Q108" t="inlineStr">
@@ -13035,7 +13035,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13149,7 +13149,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13263,7 +13263,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13377,7 +13377,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13491,7 +13491,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13605,7 +13605,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:35 PM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13618,25 +13618,25 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F114" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H114" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I114" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J114" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K114" t="inlineStr">
         <is>
@@ -13728,7 +13728,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13842,7 +13842,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13956,7 +13956,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -14070,7 +14070,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14184,7 +14184,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14298,7 +14298,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14412,7 +14412,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14526,7 +14526,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14640,7 +14640,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14754,7 +14754,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14868,7 +14868,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14982,7 +14982,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -15096,7 +15096,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15210,7 +15210,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15324,7 +15324,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15438,7 +15438,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15552,7 +15552,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15666,7 +15666,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15780,7 +15780,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15894,7 +15894,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -16008,7 +16008,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16122,7 +16122,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16236,7 +16236,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16350,7 +16350,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16464,7 +16464,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16578,7 +16578,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16692,7 +16692,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16806,7 +16806,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16920,7 +16920,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -17034,7 +17034,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17148,7 +17148,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17262,7 +17262,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17376,7 +17376,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17490,7 +17490,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17604,7 +17604,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17718,7 +17718,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17832,7 +17832,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17946,7 +17946,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -18060,7 +18060,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18174,7 +18174,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18288,7 +18288,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18402,7 +18402,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18415,7 +18415,7 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F156" t="n">
@@ -18427,13 +18427,13 @@
         </is>
       </c>
       <c r="H156" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I156" t="n">
         <v>0</v>
       </c>
       <c r="J156" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K156" t="inlineStr">
         <is>
@@ -18525,7 +18525,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18639,7 +18639,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18753,7 +18753,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18867,7 +18867,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18880,7 +18880,7 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F160" t="n">
@@ -18892,13 +18892,13 @@
         </is>
       </c>
       <c r="H160" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I160" t="n">
         <v>0</v>
       </c>
       <c r="J160" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K160" t="inlineStr">
         <is>
@@ -18990,7 +18990,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19104,7 +19104,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19218,7 +19218,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:35 PM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19231,25 +19231,25 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F163" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H163" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I163" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J163" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K163" t="inlineStr">
         <is>
@@ -19341,7 +19341,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:35 PM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19354,25 +19354,25 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F164" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H164" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I164" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J164" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K164" t="inlineStr">
         <is>
@@ -19464,7 +19464,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19578,7 +19578,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19692,7 +19692,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19806,7 +19806,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19920,7 +19920,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -20034,7 +20034,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -20148,7 +20148,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20262,7 +20262,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20376,7 +20376,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20490,7 +20490,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20604,7 +20604,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20718,7 +20718,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20832,7 +20832,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20946,7 +20946,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -21060,7 +21060,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21174,7 +21174,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21288,7 +21288,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21402,7 +21402,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21516,7 +21516,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21630,7 +21630,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21744,7 +21744,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21858,7 +21858,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21972,7 +21972,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -22086,7 +22086,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22200,7 +22200,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22314,7 +22314,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:35 PM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22327,25 +22327,25 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F190" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H190" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I190" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J190" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K190" t="inlineStr">
         <is>
@@ -22437,7 +22437,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22551,7 +22551,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22665,7 +22665,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22779,7 +22779,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22893,7 +22893,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -23007,7 +23007,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -23121,7 +23121,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23235,7 +23235,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23349,7 +23349,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23463,7 +23463,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23577,7 +23577,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23691,7 +23691,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23805,7 +23805,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23919,7 +23919,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -24033,7 +24033,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -24147,7 +24147,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24261,7 +24261,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24375,7 +24375,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24489,7 +24489,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24603,7 +24603,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24717,7 +24717,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24730,7 +24730,7 @@
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F211" t="n">
@@ -24742,13 +24742,13 @@
         </is>
       </c>
       <c r="H211" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I211" t="n">
         <v>0</v>
       </c>
       <c r="J211" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K211" t="inlineStr">
         <is>
@@ -24840,7 +24840,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -24853,7 +24853,7 @@
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F212" t="n">
@@ -24865,13 +24865,13 @@
         </is>
       </c>
       <c r="H212" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I212" t="n">
         <v>0</v>
       </c>
       <c r="J212" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K212" t="inlineStr">
         <is>
@@ -24963,7 +24963,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -24976,7 +24976,7 @@
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F213" t="n">
@@ -24988,13 +24988,13 @@
         </is>
       </c>
       <c r="H213" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I213" t="n">
         <v>0</v>
       </c>
       <c r="J213" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K213" t="inlineStr">
         <is>
@@ -25086,7 +25086,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -25200,7 +25200,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25314,7 +25314,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25428,7 +25428,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25542,7 +25542,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25656,7 +25656,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25770,7 +25770,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25884,7 +25884,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -25998,7 +25998,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -26112,7 +26112,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26226,7 +26226,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26340,7 +26340,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26454,7 +26454,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:35 PM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26467,25 +26467,25 @@
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F226" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G226" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H226" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I226" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J226" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K226" t="inlineStr">
         <is>
@@ -26577,7 +26577,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:35 PM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26590,25 +26590,25 @@
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F227" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G227" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H227" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I227" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J227" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K227" t="inlineStr">
         <is>
@@ -26700,7 +26700,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26814,7 +26814,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26827,7 +26827,7 @@
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F229" t="n">
@@ -26839,13 +26839,13 @@
         </is>
       </c>
       <c r="H229" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I229" t="n">
         <v>0</v>
       </c>
       <c r="J229" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K229" t="inlineStr">
         <is>
@@ -26937,7 +26937,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -26950,7 +26950,7 @@
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F230" t="n">
@@ -26962,13 +26962,13 @@
         </is>
       </c>
       <c r="H230" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I230" t="n">
         <v>0</v>
       </c>
       <c r="J230" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K230" t="inlineStr">
         <is>
@@ -27060,7 +27060,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -27073,7 +27073,7 @@
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F231" t="n">
@@ -27085,13 +27085,13 @@
         </is>
       </c>
       <c r="H231" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I231" t="n">
         <v>0</v>
       </c>
       <c r="J231" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K231" t="inlineStr">
         <is>
@@ -27127,10 +27127,10 @@
         </is>
       </c>
       <c r="R231" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S231" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T231" t="n">
         <v>0</v>
@@ -27183,7 +27183,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27196,7 +27196,7 @@
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F232" t="n">
@@ -27208,13 +27208,13 @@
         </is>
       </c>
       <c r="H232" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I232" t="n">
         <v>0</v>
       </c>
       <c r="J232" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K232" t="inlineStr">
         <is>
@@ -27306,7 +27306,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27420,7 +27420,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27534,7 +27534,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -27648,7 +27648,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -27762,7 +27762,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -27876,7 +27876,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -27990,7 +27990,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -28104,7 +28104,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -28218,7 +28218,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -28332,7 +28332,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -28446,7 +28446,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -28560,7 +28560,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -28674,7 +28674,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -28788,7 +28788,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -28902,7 +28902,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -29016,7 +29016,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -29130,7 +29130,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -29244,7 +29244,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -29358,7 +29358,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -29472,7 +29472,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -29586,7 +29586,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -29700,7 +29700,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -29814,7 +29814,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -29928,7 +29928,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -30042,7 +30042,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -30156,7 +30156,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -30270,7 +30270,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -30384,7 +30384,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -30498,7 +30498,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -30612,7 +30612,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -30726,7 +30726,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -30840,7 +30840,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -30954,7 +30954,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -30967,7 +30967,7 @@
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F265" t="n">
@@ -30979,13 +30979,13 @@
         </is>
       </c>
       <c r="H265" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I265" t="n">
         <v>0</v>
       </c>
       <c r="J265" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K265" t="inlineStr">
         <is>
@@ -31077,7 +31077,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -31090,7 +31090,7 @@
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F266" t="n">
@@ -31102,13 +31102,13 @@
         </is>
       </c>
       <c r="H266" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I266" t="n">
         <v>0</v>
       </c>
       <c r="J266" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K266" t="inlineStr">
         <is>
@@ -31200,7 +31200,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -31213,7 +31213,7 @@
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F267" t="n">
@@ -31225,13 +31225,13 @@
         </is>
       </c>
       <c r="H267" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I267" t="n">
         <v>0</v>
       </c>
       <c r="J267" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K267" t="inlineStr">
         <is>
@@ -31323,7 +31323,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -31336,7 +31336,7 @@
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>Top 8 | 1 out</t>
+          <t>Top 8 | 2 out</t>
         </is>
       </c>
       <c r="F268" t="n">
@@ -31348,13 +31348,13 @@
         </is>
       </c>
       <c r="H268" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I268" t="n">
         <v>0</v>
       </c>
       <c r="J268" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K268" t="inlineStr">
         <is>
@@ -31446,7 +31446,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -31560,7 +31560,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -31674,7 +31674,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -31788,7 +31788,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -31902,7 +31902,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -32016,7 +32016,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -32130,7 +32130,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -32244,7 +32244,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -32358,7 +32358,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -32472,7 +32472,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -32586,7 +32586,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C279" t="n">
@@ -32700,7 +32700,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -32814,7 +32814,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C281" t="n">
@@ -32928,7 +32928,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C282" t="n">
@@ -33042,7 +33042,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -33156,7 +33156,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -33270,7 +33270,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -33384,7 +33384,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -33498,7 +33498,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -33612,7 +33612,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -33726,7 +33726,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -33840,7 +33840,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -33954,7 +33954,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C291" t="n">
@@ -34068,7 +34068,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C292" t="n">
@@ -34182,7 +34182,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C293" t="n">
@@ -34296,7 +34296,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C294" t="n">
@@ -34410,7 +34410,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C295" t="n">
@@ -34524,7 +34524,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C296" t="n">
@@ -34638,7 +34638,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:35 PM PT</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -34651,25 +34651,25 @@
       </c>
       <c r="E297" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F297" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G297" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H297" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I297" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J297" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K297" t="inlineStr">
         <is>
@@ -34761,7 +34761,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:35 PM PT</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -34774,25 +34774,25 @@
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F298" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G298" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H298" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I298" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J298" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K298" t="inlineStr">
         <is>
@@ -34884,7 +34884,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:35 PM PT</t>
         </is>
       </c>
       <c r="C299" t="n">
@@ -34897,25 +34897,25 @@
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F299" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G299" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H299" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I299" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J299" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K299" t="inlineStr">
         <is>
@@ -35007,7 +35007,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C300" t="n">
@@ -35121,7 +35121,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C301" t="n">
@@ -35235,7 +35235,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C302" t="n">
@@ -35349,7 +35349,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C303" t="n">
@@ -35463,7 +35463,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C304" t="n">
@@ -35577,7 +35577,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C305" t="n">
@@ -35691,7 +35691,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:33 PM PT</t>
+          <t>2026-07-12 03:41:33 PM PT</t>
         </is>
       </c>
       <c r="C306" t="n">
@@ -35805,7 +35805,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C307" t="n">
@@ -35919,7 +35919,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C308" t="n">
@@ -36033,7 +36033,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:32 PM PT</t>
+          <t>2026-07-12 03:41:32 PM PT</t>
         </is>
       </c>
       <c r="C309" t="n">
@@ -36147,7 +36147,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -36261,7 +36261,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -36375,7 +36375,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:34 PM PT</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -36489,7 +36489,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:35 PM PT</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -36502,25 +36502,25 @@
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F313" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G313" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H313" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I313" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J313" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K313" t="inlineStr">
         <is>
@@ -36612,7 +36612,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:34 PM PT</t>
+          <t>2026-07-12 03:41:35 PM PT</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -36625,25 +36625,25 @@
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>Bottom 8 | 3 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F314" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G314" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H314" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I314" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J314" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K314" t="inlineStr">
         <is>
@@ -36735,7 +36735,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C315" t="n">
@@ -36849,7 +36849,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C316" t="n">
@@ -36963,7 +36963,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C317" t="n">
@@ -37077,7 +37077,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C318" t="n">
@@ -37191,7 +37191,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>2026-07-12 03:39:31 PM PT</t>
+          <t>2026-07-12 03:41:31 PM PT</t>
         </is>
       </c>
       <c r="C319" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-12 03:43:34 PM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
@@ -487,7 +487,7 @@
     <col width="27" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
@@ -693,7 +693,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -807,7 +807,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:30 PM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -921,7 +921,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Top 8 | 2 out</t>
+          <t>Bottom 8 | 0 out</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -1512,11 +1512,11 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
@@ -1614,7 +1614,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1728,7 +1728,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1842,7 +1842,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:30 PM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1956,7 +1956,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2070,7 +2070,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:30 PM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2184,7 +2184,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2298,7 +2298,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:30 PM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2412,7 +2412,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2640,7 +2640,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2754,7 +2754,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2868,7 +2868,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2982,7 +2982,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:30 PM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3096,7 +3096,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3324,7 +3324,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3438,7 +3438,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:35 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3451,7 +3451,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F26" t="n">
@@ -3463,13 +3463,13 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
@@ -3505,10 +3505,10 @@
         </is>
       </c>
       <c r="R26" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S26" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T26" t="n">
         <v>1</v>
@@ -3561,7 +3561,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3675,7 +3675,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3789,7 +3789,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3903,7 +3903,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -4017,7 +4017,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4131,7 +4131,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4245,7 +4245,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4359,7 +4359,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4473,7 +4473,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4587,7 +4587,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4701,7 +4701,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:30 PM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4815,7 +4815,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4929,7 +4929,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:30 PM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5043,7 +5043,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:30 PM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5157,7 +5157,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5271,7 +5271,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5385,7 +5385,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5499,7 +5499,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:35 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5512,7 +5512,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F44" t="n">
@@ -5524,13 +5524,13 @@
         </is>
       </c>
       <c r="H44" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I44" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K44" t="inlineStr">
         <is>
@@ -5622,7 +5622,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5736,7 +5736,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5850,7 +5850,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5964,7 +5964,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6078,7 +6078,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6192,7 +6192,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:30 PM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6306,7 +6306,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:35 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6319,7 +6319,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F51" t="n">
@@ -6331,13 +6331,13 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I51" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J51" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K51" t="inlineStr">
         <is>
@@ -6429,7 +6429,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6442,7 +6442,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Top 8 | 2 out</t>
+          <t>Bottom 8 | 0 out</t>
         </is>
       </c>
       <c r="F52" t="n">
@@ -6450,11 +6450,11 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H52" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I52" t="n">
         <v>0</v>
@@ -6552,7 +6552,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6666,7 +6666,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6780,7 +6780,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6894,7 +6894,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -7008,7 +7008,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:30 PM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7122,7 +7122,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7236,7 +7236,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7350,7 +7350,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7578,7 +7578,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7692,7 +7692,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7806,7 +7806,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7920,7 +7920,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -8034,7 +8034,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8148,7 +8148,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:35 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8161,7 +8161,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F67" t="n">
@@ -8173,13 +8173,13 @@
         </is>
       </c>
       <c r="H67" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I67" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J67" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K67" t="inlineStr">
         <is>
@@ -8271,7 +8271,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8385,7 +8385,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:35 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8398,7 +8398,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F69" t="n">
@@ -8410,13 +8410,13 @@
         </is>
       </c>
       <c r="H69" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I69" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J69" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K69" t="inlineStr">
         <is>
@@ -8508,7 +8508,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:35 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8521,7 +8521,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F70" t="n">
@@ -8533,13 +8533,13 @@
         </is>
       </c>
       <c r="H70" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I70" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J70" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K70" t="inlineStr">
         <is>
@@ -8631,7 +8631,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8745,7 +8745,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8758,7 +8758,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Top 8 | 2 out</t>
+          <t>Bottom 8 | 0 out</t>
         </is>
       </c>
       <c r="F72" t="n">
@@ -8766,11 +8766,11 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H72" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I72" t="n">
         <v>0</v>
@@ -8868,7 +8868,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8881,7 +8881,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Top 8 | 2 out</t>
+          <t>Bottom 8 | 0 out</t>
         </is>
       </c>
       <c r="F73" t="n">
@@ -8889,11 +8889,11 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H73" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I73" t="n">
         <v>0</v>
@@ -8991,7 +8991,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9105,7 +9105,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9219,7 +9219,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9333,7 +9333,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9447,7 +9447,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9561,7 +9561,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9675,7 +9675,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9789,7 +9789,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:35 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9802,7 +9802,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F81" t="n">
@@ -9814,13 +9814,13 @@
         </is>
       </c>
       <c r="H81" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I81" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J81" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K81" t="inlineStr">
         <is>
@@ -9912,7 +9912,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -10026,7 +10026,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10140,7 +10140,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10254,7 +10254,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10368,7 +10368,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10482,7 +10482,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10596,7 +10596,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10710,7 +10710,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10824,7 +10824,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:35 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10837,7 +10837,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F90" t="n">
@@ -10849,13 +10849,13 @@
         </is>
       </c>
       <c r="H90" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I90" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J90" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K90" t="inlineStr">
         <is>
@@ -10947,7 +10947,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -11061,7 +11061,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:35 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11074,7 +11074,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F92" t="n">
@@ -11086,13 +11086,13 @@
         </is>
       </c>
       <c r="H92" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I92" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J92" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K92" t="inlineStr">
         <is>
@@ -11184,7 +11184,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11197,7 +11197,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Top 8 | 2 out</t>
+          <t>Bottom 8 | 0 out</t>
         </is>
       </c>
       <c r="F93" t="n">
@@ -11205,11 +11205,11 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H93" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I93" t="n">
         <v>0</v>
@@ -11307,7 +11307,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11421,7 +11421,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11535,7 +11535,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11649,7 +11649,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11763,7 +11763,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11877,7 +11877,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11890,7 +11890,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Top 8 | 2 out</t>
+          <t>Bottom 8 | 0 out</t>
         </is>
       </c>
       <c r="F99" t="n">
@@ -11898,11 +11898,11 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H99" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I99" t="n">
         <v>0</v>
@@ -12000,7 +12000,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -12114,7 +12114,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:30 PM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12228,7 +12228,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:30 PM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12342,7 +12342,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:30 PM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12456,7 +12456,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:30 PM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12570,7 +12570,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12684,7 +12684,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12798,7 +12798,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12912,7 +12912,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:35 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12925,7 +12925,7 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F108" t="n">
@@ -12937,13 +12937,13 @@
         </is>
       </c>
       <c r="H108" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I108" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J108" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K108" t="inlineStr">
         <is>
@@ -13035,7 +13035,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13149,7 +13149,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13263,7 +13263,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13377,7 +13377,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13491,7 +13491,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13605,7 +13605,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:35 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13618,7 +13618,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F114" t="n">
@@ -13630,13 +13630,13 @@
         </is>
       </c>
       <c r="H114" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I114" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J114" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K114" t="inlineStr">
         <is>
@@ -13728,7 +13728,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13842,7 +13842,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13956,7 +13956,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -14070,7 +14070,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14184,7 +14184,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14298,7 +14298,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14412,7 +14412,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14526,7 +14526,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14640,7 +14640,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14754,7 +14754,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14868,7 +14868,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14982,7 +14982,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -15096,7 +15096,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15210,7 +15210,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15324,7 +15324,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15438,7 +15438,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15552,7 +15552,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15666,7 +15666,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15780,7 +15780,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15894,7 +15894,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -16008,7 +16008,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16122,7 +16122,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16236,7 +16236,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16350,7 +16350,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16464,7 +16464,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16578,7 +16578,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16692,7 +16692,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16806,7 +16806,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16920,7 +16920,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -17034,7 +17034,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17148,7 +17148,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17262,7 +17262,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17376,7 +17376,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17490,7 +17490,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17604,7 +17604,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17718,7 +17718,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17832,7 +17832,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:30 PM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17946,7 +17946,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -18060,7 +18060,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18174,7 +18174,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18288,7 +18288,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18402,7 +18402,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18415,7 +18415,7 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>Top 8 | 2 out</t>
+          <t>Bottom 8 | 0 out</t>
         </is>
       </c>
       <c r="F156" t="n">
@@ -18423,11 +18423,11 @@
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H156" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I156" t="n">
         <v>0</v>
@@ -18525,7 +18525,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18639,7 +18639,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18753,7 +18753,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18867,7 +18867,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18880,7 +18880,7 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>Top 8 | 2 out</t>
+          <t>Bottom 8 | 0 out</t>
         </is>
       </c>
       <c r="F160" t="n">
@@ -18888,11 +18888,11 @@
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H160" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I160" t="n">
         <v>0</v>
@@ -18990,7 +18990,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19104,7 +19104,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19218,7 +19218,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:35 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19231,7 +19231,7 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F163" t="n">
@@ -19243,13 +19243,13 @@
         </is>
       </c>
       <c r="H163" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I163" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J163" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K163" t="inlineStr">
         <is>
@@ -19341,7 +19341,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:35 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19354,7 +19354,7 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F164" t="n">
@@ -19366,13 +19366,13 @@
         </is>
       </c>
       <c r="H164" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I164" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J164" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K164" t="inlineStr">
         <is>
@@ -19464,7 +19464,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19578,7 +19578,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19692,7 +19692,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19806,7 +19806,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19920,7 +19920,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -20034,7 +20034,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -20148,7 +20148,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20262,7 +20262,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20376,7 +20376,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20490,7 +20490,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20604,7 +20604,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20718,7 +20718,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20832,7 +20832,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20946,7 +20946,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -21060,7 +21060,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21174,7 +21174,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21288,7 +21288,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21402,7 +21402,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21516,7 +21516,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:30 PM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21630,7 +21630,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21744,7 +21744,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21858,7 +21858,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21972,7 +21972,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -22086,7 +22086,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22200,7 +22200,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22314,7 +22314,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:35 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22327,7 +22327,7 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F190" t="n">
@@ -22339,13 +22339,13 @@
         </is>
       </c>
       <c r="H190" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I190" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J190" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K190" t="inlineStr">
         <is>
@@ -22437,7 +22437,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22551,7 +22551,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22665,7 +22665,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22779,7 +22779,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22893,7 +22893,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -23007,7 +23007,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -23121,7 +23121,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23235,7 +23235,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23349,7 +23349,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23463,7 +23463,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23577,7 +23577,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23691,7 +23691,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23805,7 +23805,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23919,7 +23919,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -24033,7 +24033,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -24147,7 +24147,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24261,7 +24261,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24375,7 +24375,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24489,7 +24489,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24603,7 +24603,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24717,7 +24717,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24730,7 +24730,7 @@
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>Top 8 | 2 out</t>
+          <t>Bottom 8 | 0 out</t>
         </is>
       </c>
       <c r="F211" t="n">
@@ -24738,11 +24738,11 @@
       </c>
       <c r="G211" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H211" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I211" t="n">
         <v>0</v>
@@ -24840,7 +24840,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -24853,7 +24853,7 @@
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>Top 8 | 2 out</t>
+          <t>Bottom 8 | 0 out</t>
         </is>
       </c>
       <c r="F212" t="n">
@@ -24861,11 +24861,11 @@
       </c>
       <c r="G212" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H212" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I212" t="n">
         <v>0</v>
@@ -24963,7 +24963,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -24976,7 +24976,7 @@
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>Top 8 | 2 out</t>
+          <t>Bottom 8 | 0 out</t>
         </is>
       </c>
       <c r="F213" t="n">
@@ -24984,11 +24984,11 @@
       </c>
       <c r="G213" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H213" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I213" t="n">
         <v>0</v>
@@ -25086,7 +25086,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -25200,7 +25200,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:30 PM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25314,7 +25314,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25428,7 +25428,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25542,7 +25542,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25656,7 +25656,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25770,7 +25770,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25884,7 +25884,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -25998,7 +25998,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -26112,7 +26112,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26226,7 +26226,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26340,7 +26340,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26454,7 +26454,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:35 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26467,7 +26467,7 @@
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F226" t="n">
@@ -26479,13 +26479,13 @@
         </is>
       </c>
       <c r="H226" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I226" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J226" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K226" t="inlineStr">
         <is>
@@ -26577,7 +26577,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:35 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26590,7 +26590,7 @@
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F227" t="n">
@@ -26602,13 +26602,13 @@
         </is>
       </c>
       <c r="H227" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I227" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J227" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K227" t="inlineStr">
         <is>
@@ -26700,7 +26700,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26814,7 +26814,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26827,7 +26827,7 @@
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>Top 8 | 2 out</t>
+          <t>Bottom 8 | 0 out</t>
         </is>
       </c>
       <c r="F229" t="n">
@@ -26835,11 +26835,11 @@
       </c>
       <c r="G229" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H229" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I229" t="n">
         <v>0</v>
@@ -26937,7 +26937,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -26950,7 +26950,7 @@
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>Top 8 | 2 out</t>
+          <t>Bottom 8 | 0 out</t>
         </is>
       </c>
       <c r="F230" t="n">
@@ -26958,11 +26958,11 @@
       </c>
       <c r="G230" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H230" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I230" t="n">
         <v>0</v>
@@ -27060,7 +27060,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -27073,7 +27073,7 @@
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>Top 8 | 2 out</t>
+          <t>Bottom 8 | 0 out</t>
         </is>
       </c>
       <c r="F231" t="n">
@@ -27081,11 +27081,11 @@
       </c>
       <c r="G231" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H231" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I231" t="n">
         <v>0</v>
@@ -27183,7 +27183,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27196,7 +27196,7 @@
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>Top 8 | 2 out</t>
+          <t>Bottom 8 | 0 out</t>
         </is>
       </c>
       <c r="F232" t="n">
@@ -27204,11 +27204,11 @@
       </c>
       <c r="G232" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H232" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I232" t="n">
         <v>0</v>
@@ -27306,7 +27306,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27420,7 +27420,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27534,7 +27534,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -27648,7 +27648,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -27762,7 +27762,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -27876,7 +27876,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -27990,7 +27990,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -28104,7 +28104,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -28218,7 +28218,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -28332,7 +28332,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -28446,7 +28446,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -28560,7 +28560,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -28674,7 +28674,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -28788,7 +28788,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -28902,7 +28902,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -29016,7 +29016,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -29130,7 +29130,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -29244,7 +29244,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -29358,7 +29358,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -29472,7 +29472,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -29586,7 +29586,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -29700,7 +29700,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -29814,7 +29814,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -29928,7 +29928,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -30042,7 +30042,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -30156,7 +30156,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -30270,7 +30270,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -30384,7 +30384,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -30498,7 +30498,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -30612,7 +30612,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -30726,7 +30726,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -30840,7 +30840,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -30954,7 +30954,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -30967,7 +30967,7 @@
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t>Top 8 | 2 out</t>
+          <t>Bottom 8 | 0 out</t>
         </is>
       </c>
       <c r="F265" t="n">
@@ -30975,11 +30975,11 @@
       </c>
       <c r="G265" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H265" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I265" t="n">
         <v>0</v>
@@ -31077,7 +31077,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -31090,7 +31090,7 @@
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>Top 8 | 2 out</t>
+          <t>Bottom 8 | 0 out</t>
         </is>
       </c>
       <c r="F266" t="n">
@@ -31098,11 +31098,11 @@
       </c>
       <c r="G266" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H266" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I266" t="n">
         <v>0</v>
@@ -31200,7 +31200,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -31213,7 +31213,7 @@
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>Top 8 | 2 out</t>
+          <t>Bottom 8 | 0 out</t>
         </is>
       </c>
       <c r="F267" t="n">
@@ -31221,11 +31221,11 @@
       </c>
       <c r="G267" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H267" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I267" t="n">
         <v>0</v>
@@ -31323,7 +31323,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -31336,7 +31336,7 @@
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>Top 8 | 2 out</t>
+          <t>Bottom 8 | 0 out</t>
         </is>
       </c>
       <c r="F268" t="n">
@@ -31344,11 +31344,11 @@
       </c>
       <c r="G268" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H268" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I268" t="n">
         <v>0</v>
@@ -31446,7 +31446,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -31560,7 +31560,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -31674,7 +31674,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -31788,7 +31788,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -31902,7 +31902,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -32016,7 +32016,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -32130,7 +32130,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:30 PM PT</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -32244,7 +32244,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:30 PM PT</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -32358,7 +32358,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:30 PM PT</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -32472,7 +32472,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -32586,7 +32586,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C279" t="n">
@@ -32700,7 +32700,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -32814,7 +32814,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C281" t="n">
@@ -32928,7 +32928,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C282" t="n">
@@ -33042,7 +33042,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -33156,7 +33156,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -33270,7 +33270,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -33384,7 +33384,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -33498,7 +33498,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -33612,7 +33612,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -33726,7 +33726,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -33840,7 +33840,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -33954,7 +33954,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C291" t="n">
@@ -34068,7 +34068,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C292" t="n">
@@ -34182,7 +34182,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C293" t="n">
@@ -34296,7 +34296,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:30 PM PT</t>
         </is>
       </c>
       <c r="C294" t="n">
@@ -34410,7 +34410,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:30 PM PT</t>
         </is>
       </c>
       <c r="C295" t="n">
@@ -34524,7 +34524,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:30 PM PT</t>
         </is>
       </c>
       <c r="C296" t="n">
@@ -34638,7 +34638,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:35 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -34651,7 +34651,7 @@
       </c>
       <c r="E297" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F297" t="n">
@@ -34663,13 +34663,13 @@
         </is>
       </c>
       <c r="H297" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I297" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J297" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K297" t="inlineStr">
         <is>
@@ -34761,7 +34761,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:35 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -34774,7 +34774,7 @@
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F298" t="n">
@@ -34786,13 +34786,13 @@
         </is>
       </c>
       <c r="H298" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I298" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J298" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K298" t="inlineStr">
         <is>
@@ -34884,7 +34884,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:35 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C299" t="n">
@@ -34897,7 +34897,7 @@
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F299" t="n">
@@ -34909,13 +34909,13 @@
         </is>
       </c>
       <c r="H299" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I299" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J299" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K299" t="inlineStr">
         <is>
@@ -35007,7 +35007,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C300" t="n">
@@ -35121,7 +35121,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C301" t="n">
@@ -35235,7 +35235,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C302" t="n">
@@ -35349,7 +35349,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C303" t="n">
@@ -35463,7 +35463,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C304" t="n">
@@ -35577,7 +35577,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C305" t="n">
@@ -35691,7 +35691,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:33 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C306" t="n">
@@ -35805,7 +35805,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C307" t="n">
@@ -35919,7 +35919,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C308" t="n">
@@ -36033,7 +36033,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:32 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C309" t="n">
@@ -36147,7 +36147,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -36261,7 +36261,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -36375,7 +36375,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:34 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -36489,7 +36489,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:35 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -36502,7 +36502,7 @@
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F313" t="n">
@@ -36514,13 +36514,13 @@
         </is>
       </c>
       <c r="H313" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I313" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J313" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K313" t="inlineStr">
         <is>
@@ -36556,10 +36556,10 @@
         </is>
       </c>
       <c r="R313" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S313" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T313" t="n">
         <v>0</v>
@@ -36612,7 +36612,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:35 PM PT</t>
+          <t>2026-07-12 03:43:32 PM PT</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -36625,7 +36625,7 @@
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F314" t="n">
@@ -36637,13 +36637,13 @@
         </is>
       </c>
       <c r="H314" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I314" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J314" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K314" t="inlineStr">
         <is>
@@ -36735,7 +36735,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C315" t="n">
@@ -36849,7 +36849,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C316" t="n">
@@ -36963,7 +36963,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C317" t="n">
@@ -37077,7 +37077,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C318" t="n">
@@ -37191,7 +37191,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>2026-07-12 03:41:31 PM PT</t>
+          <t>2026-07-12 03:43:31 PM PT</t>
         </is>
       </c>
       <c r="C319" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-12 03:49:35 PM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
@@ -487,7 +487,7 @@
     <col width="27" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
@@ -693,7 +693,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -807,7 +807,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:30 PM PT</t>
+          <t>2026-07-12 03:49:30 PM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -921,7 +921,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1504,25 +1504,25 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -1614,7 +1614,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1728,7 +1728,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1842,7 +1842,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:30 PM PT</t>
+          <t>2026-07-12 03:49:30 PM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1956,7 +1956,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2070,7 +2070,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:30 PM PT</t>
+          <t>2026-07-12 03:49:30 PM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2184,7 +2184,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2298,7 +2298,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:30 PM PT</t>
+          <t>2026-07-12 03:49:30 PM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2412,7 +2412,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2640,7 +2640,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2754,7 +2754,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2868,7 +2868,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2982,7 +2982,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:30 PM PT</t>
+          <t>2026-07-12 03:49:30 PM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3096,7 +3096,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3324,7 +3324,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3438,7 +3438,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:33 PM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3451,7 +3451,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F26" t="n">
@@ -3552,7 +3552,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3666,7 +3666,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3780,7 +3780,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3894,7 +3894,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -4008,7 +4008,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4122,7 +4122,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4236,7 +4236,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4350,7 +4350,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4464,7 +4464,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4578,7 +4578,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4692,7 +4692,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:30 PM PT</t>
+          <t>2026-07-12 03:49:30 PM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4806,7 +4806,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4920,7 +4920,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:30 PM PT</t>
+          <t>2026-07-12 03:49:30 PM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5034,7 +5034,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:30 PM PT</t>
+          <t>2026-07-12 03:49:30 PM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5148,7 +5148,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5262,7 +5262,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5376,7 +5376,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5490,7 +5490,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:33 PM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5503,7 +5503,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F44" t="n">
@@ -5604,7 +5604,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5718,7 +5718,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5832,7 +5832,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5946,7 +5946,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6060,7 +6060,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6174,7 +6174,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:30 PM PT</t>
+          <t>2026-07-12 03:49:30 PM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:33 PM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6301,7 +6301,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F51" t="n">
@@ -6402,7 +6402,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6415,25 +6415,25 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F52" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H52" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I52" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K52" t="inlineStr">
         <is>
@@ -6525,7 +6525,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6639,7 +6639,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6753,7 +6753,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6867,7 +6867,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -6981,7 +6981,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:30 PM PT</t>
+          <t>2026-07-12 03:49:30 PM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7095,7 +7095,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7209,7 +7209,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7323,7 +7323,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7437,7 +7437,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7551,7 +7551,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7665,7 +7665,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7779,7 +7779,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7893,7 +7893,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -8007,7 +8007,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8121,7 +8121,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:33 PM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8134,7 +8134,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F67" t="n">
@@ -8235,7 +8235,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8349,7 +8349,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:33 PM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8362,7 +8362,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F69" t="n">
@@ -8463,7 +8463,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:33 PM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8476,7 +8476,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F70" t="n">
@@ -8577,7 +8577,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8691,7 +8691,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8704,25 +8704,25 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F72" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H72" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I72" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J72" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K72" t="inlineStr">
         <is>
@@ -8814,7 +8814,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8827,25 +8827,25 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F73" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H73" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I73" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J73" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K73" t="inlineStr">
         <is>
@@ -8937,7 +8937,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9051,7 +9051,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9165,7 +9165,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9279,7 +9279,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9393,7 +9393,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9507,7 +9507,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9621,7 +9621,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9735,7 +9735,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:33 PM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9748,7 +9748,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F81" t="n">
@@ -9849,7 +9849,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -9963,7 +9963,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10077,7 +10077,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10191,7 +10191,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10305,7 +10305,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10419,7 +10419,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10533,7 +10533,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10647,7 +10647,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10761,7 +10761,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:33 PM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10774,7 +10774,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F90" t="n">
@@ -10875,7 +10875,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -10989,7 +10989,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:33 PM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11002,7 +11002,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F92" t="n">
@@ -11103,7 +11103,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11116,25 +11116,25 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F93" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H93" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I93" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J93" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K93" t="inlineStr">
         <is>
@@ -11226,7 +11226,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11340,7 +11340,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11454,7 +11454,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11568,7 +11568,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11682,7 +11682,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11796,7 +11796,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11809,25 +11809,25 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F99" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H99" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I99" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J99" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K99" t="inlineStr">
         <is>
@@ -11919,7 +11919,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -12033,7 +12033,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:30 PM PT</t>
+          <t>2026-07-12 03:49:30 PM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12147,7 +12147,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:30 PM PT</t>
+          <t>2026-07-12 03:49:30 PM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12261,7 +12261,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:30 PM PT</t>
+          <t>2026-07-12 03:49:30 PM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12375,7 +12375,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:30 PM PT</t>
+          <t>2026-07-12 03:49:30 PM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12489,7 +12489,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12603,7 +12603,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12717,7 +12717,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12831,7 +12831,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:33 PM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12844,7 +12844,7 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F108" t="n">
@@ -12945,7 +12945,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13059,7 +13059,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13173,7 +13173,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13287,7 +13287,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13401,7 +13401,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13515,7 +13515,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:33 PM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13528,7 +13528,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F114" t="n">
@@ -13629,7 +13629,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13743,7 +13743,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13857,7 +13857,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -13971,7 +13971,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14085,7 +14085,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14199,7 +14199,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14313,7 +14313,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14326,25 +14326,25 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F121" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H121" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I121" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J121" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K121" t="inlineStr">
         <is>
@@ -14436,7 +14436,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14550,7 +14550,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14664,7 +14664,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14778,7 +14778,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14892,7 +14892,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -15006,7 +15006,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15120,7 +15120,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15234,7 +15234,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15348,7 +15348,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15462,7 +15462,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15576,7 +15576,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15690,7 +15690,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15804,7 +15804,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -15918,7 +15918,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16032,7 +16032,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16146,7 +16146,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16260,7 +16260,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16374,7 +16374,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16488,7 +16488,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16602,7 +16602,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16716,7 +16716,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16830,7 +16830,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -16944,7 +16944,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17058,7 +17058,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17172,7 +17172,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17286,7 +17286,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17400,7 +17400,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17514,7 +17514,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17628,7 +17628,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17742,7 +17742,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17856,7 +17856,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:30 PM PT</t>
+          <t>2026-07-12 03:49:30 PM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -17970,7 +17970,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18084,7 +18084,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18198,7 +18198,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18312,7 +18312,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18426,7 +18426,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18439,25 +18439,25 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F157" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H157" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I157" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J157" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K157" t="inlineStr">
         <is>
@@ -18549,7 +18549,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18663,7 +18663,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18777,7 +18777,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18891,7 +18891,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19005,7 +19005,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19119,7 +19119,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:33 PM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19132,7 +19132,7 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F163" t="n">
@@ -19233,7 +19233,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:33 PM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19246,7 +19246,7 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F164" t="n">
@@ -19347,7 +19347,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19461,7 +19461,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19575,7 +19575,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19689,7 +19689,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19803,7 +19803,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -19917,7 +19917,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -20031,7 +20031,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20145,7 +20145,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20259,7 +20259,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20373,7 +20373,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20487,7 +20487,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20601,7 +20601,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20715,7 +20715,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20829,7 +20829,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -20943,7 +20943,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21057,7 +21057,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21171,7 +21171,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21285,7 +21285,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21399,7 +21399,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:30 PM PT</t>
+          <t>2026-07-12 03:49:30 PM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21513,7 +21513,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21627,7 +21627,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21741,7 +21741,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21855,7 +21855,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -21969,7 +21969,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22083,7 +22083,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22197,7 +22197,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:33 PM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22210,7 +22210,7 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F190" t="n">
@@ -22311,7 +22311,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22425,7 +22425,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22539,7 +22539,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22653,7 +22653,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22767,7 +22767,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -22881,7 +22881,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -22995,7 +22995,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23109,7 +23109,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23223,7 +23223,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23337,7 +23337,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23451,7 +23451,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23565,7 +23565,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23679,7 +23679,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23793,7 +23793,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -23907,7 +23907,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -24021,7 +24021,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24135,7 +24135,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24249,7 +24249,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24363,7 +24363,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24477,7 +24477,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24591,7 +24591,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24604,25 +24604,25 @@
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F211" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G211" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H211" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I211" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J211" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K211" t="inlineStr">
         <is>
@@ -24714,7 +24714,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -24727,25 +24727,25 @@
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F212" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G212" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H212" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I212" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J212" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K212" t="inlineStr">
         <is>
@@ -24837,7 +24837,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -24850,25 +24850,25 @@
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F213" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G213" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H213" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I213" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J213" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K213" t="inlineStr">
         <is>
@@ -24960,7 +24960,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -25074,7 +25074,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:30 PM PT</t>
+          <t>2026-07-12 03:49:30 PM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25188,7 +25188,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25302,7 +25302,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25416,7 +25416,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25530,7 +25530,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25644,7 +25644,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25758,7 +25758,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -25872,7 +25872,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -25986,7 +25986,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26100,7 +26100,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26214,7 +26214,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26328,7 +26328,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:33 PM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26341,7 +26341,7 @@
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F226" t="n">
@@ -26442,7 +26442,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:33 PM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26455,7 +26455,7 @@
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F227" t="n">
@@ -26556,7 +26556,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26670,7 +26670,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26683,25 +26683,25 @@
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F229" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G229" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H229" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I229" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J229" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K229" t="inlineStr">
         <is>
@@ -26793,7 +26793,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -26806,25 +26806,25 @@
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F230" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G230" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H230" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I230" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J230" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K230" t="inlineStr">
         <is>
@@ -26916,7 +26916,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -26929,25 +26929,25 @@
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F231" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G231" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H231" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I231" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J231" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K231" t="inlineStr">
         <is>
@@ -27039,7 +27039,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27052,25 +27052,25 @@
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F232" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G232" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H232" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I232" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J232" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K232" t="inlineStr">
         <is>
@@ -27162,7 +27162,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27175,25 +27175,25 @@
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F233" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G233" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H233" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I233" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J233" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K233" t="inlineStr">
         <is>
@@ -27285,7 +27285,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27399,7 +27399,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -27513,7 +27513,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -27627,7 +27627,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -27741,7 +27741,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -27855,7 +27855,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -27969,7 +27969,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -28083,7 +28083,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -28197,7 +28197,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -28311,7 +28311,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -28425,7 +28425,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -28539,7 +28539,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -28653,7 +28653,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -28767,7 +28767,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -28881,7 +28881,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -28995,7 +28995,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -29109,7 +29109,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -29223,7 +29223,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -29337,7 +29337,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -29451,7 +29451,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -29565,7 +29565,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -29679,7 +29679,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -29793,7 +29793,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -29907,7 +29907,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -30021,7 +30021,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -30135,7 +30135,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -30249,7 +30249,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -30363,7 +30363,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -30477,7 +30477,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -30591,7 +30591,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -30705,7 +30705,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -30819,7 +30819,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -30933,7 +30933,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -30946,25 +30946,25 @@
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F266" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G266" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H266" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I266" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J266" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K266" t="inlineStr">
         <is>
@@ -31056,7 +31056,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -31069,25 +31069,25 @@
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F267" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G267" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H267" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I267" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J267" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K267" t="inlineStr">
         <is>
@@ -31123,10 +31123,10 @@
         </is>
       </c>
       <c r="R267" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S267" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T267" t="n">
         <v>0</v>
@@ -31179,7 +31179,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -31192,25 +31192,25 @@
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F268" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G268" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H268" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I268" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J268" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K268" t="inlineStr">
         <is>
@@ -31302,7 +31302,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -31315,25 +31315,25 @@
       </c>
       <c r="E269" t="inlineStr">
         <is>
-          <t>Bottom 8 | 2 out</t>
+          <t>Top 9 | 0 out</t>
         </is>
       </c>
       <c r="F269" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G269" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="H269" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I269" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J269" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K269" t="inlineStr">
         <is>
@@ -31425,7 +31425,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -31539,7 +31539,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -31653,7 +31653,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -31767,7 +31767,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -31881,7 +31881,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -31995,7 +31995,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -32109,7 +32109,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:30 PM PT</t>
+          <t>2026-07-12 03:49:30 PM PT</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -32223,7 +32223,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:30 PM PT</t>
+          <t>2026-07-12 03:49:30 PM PT</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -32337,7 +32337,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:30 PM PT</t>
+          <t>2026-07-12 03:49:30 PM PT</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -32451,7 +32451,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C279" t="n">
@@ -32565,7 +32565,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -32679,7 +32679,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C281" t="n">
@@ -32793,7 +32793,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C282" t="n">
@@ -32907,7 +32907,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -33021,7 +33021,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -33135,7 +33135,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -33249,7 +33249,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -33363,7 +33363,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -33477,7 +33477,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -33591,7 +33591,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -33705,7 +33705,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -33819,7 +33819,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C291" t="n">
@@ -33933,7 +33933,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C292" t="n">
@@ -34047,7 +34047,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C293" t="n">
@@ -34161,7 +34161,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C294" t="n">
@@ -34275,7 +34275,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:30 PM PT</t>
+          <t>2026-07-12 03:49:30 PM PT</t>
         </is>
       </c>
       <c r="C295" t="n">
@@ -34389,7 +34389,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:30 PM PT</t>
+          <t>2026-07-12 03:49:30 PM PT</t>
         </is>
       </c>
       <c r="C296" t="n">
@@ -34503,7 +34503,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:30 PM PT</t>
+          <t>2026-07-12 03:49:30 PM PT</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -34617,7 +34617,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:33 PM PT</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -34630,7 +34630,7 @@
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F298" t="n">
@@ -34731,7 +34731,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:33 PM PT</t>
         </is>
       </c>
       <c r="C299" t="n">
@@ -34744,7 +34744,7 @@
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F299" t="n">
@@ -34845,7 +34845,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:33 PM PT</t>
         </is>
       </c>
       <c r="C300" t="n">
@@ -34858,7 +34858,7 @@
       </c>
       <c r="E300" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F300" t="n">
@@ -34959,7 +34959,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C301" t="n">
@@ -35073,7 +35073,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C302" t="n">
@@ -35187,7 +35187,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C303" t="n">
@@ -35301,7 +35301,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C304" t="n">
@@ -35415,7 +35415,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C305" t="n">
@@ -35529,7 +35529,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C306" t="n">
@@ -35643,7 +35643,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C307" t="n">
@@ -35757,7 +35757,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C308" t="n">
@@ -35871,7 +35871,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C309" t="n">
@@ -35985,7 +35985,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -36099,7 +36099,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -36213,7 +36213,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -36327,7 +36327,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:32 PM PT</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -36441,7 +36441,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:33 PM PT</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -36454,7 +36454,7 @@
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F314" t="n">
@@ -36555,7 +36555,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:32 PM PT</t>
+          <t>2026-07-12 03:49:33 PM PT</t>
         </is>
       </c>
       <c r="C315" t="n">
@@ -36568,7 +36568,7 @@
       </c>
       <c r="E315" t="inlineStr">
         <is>
-          <t>Game Over</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="F315" t="n">
@@ -36669,7 +36669,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C316" t="n">
@@ -36783,7 +36783,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C317" t="n">
@@ -36897,7 +36897,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C318" t="n">
@@ -37011,7 +37011,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C319" t="n">
@@ -37125,7 +37125,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>2026-07-12 03:47:31 PM PT</t>
+          <t>2026-07-12 03:49:31 PM PT</t>
         </is>
       </c>
       <c r="C320" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-12 03:51:34 PM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -807,7 +807,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:30 PM PT</t>
+          <t>2026-07-12 03:51:30 PM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -921,7 +921,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1519,10 +1519,10 @@
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -1614,7 +1614,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1728,7 +1728,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1842,7 +1842,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:30 PM PT</t>
+          <t>2026-07-12 03:51:30 PM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1956,7 +1956,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2070,7 +2070,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:30 PM PT</t>
+          <t>2026-07-12 03:51:30 PM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2184,7 +2184,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2298,7 +2298,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:30 PM PT</t>
+          <t>2026-07-12 03:51:30 PM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2412,7 +2412,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2640,7 +2640,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2754,7 +2754,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2868,7 +2868,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2982,7 +2982,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:30 PM PT</t>
+          <t>2026-07-12 03:51:30 PM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3096,7 +3096,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3324,7 +3324,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3438,7 +3438,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:33 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3552,7 +3552,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3666,7 +3666,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3780,7 +3780,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3894,7 +3894,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -4008,7 +4008,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4122,7 +4122,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4236,7 +4236,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4350,7 +4350,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4464,7 +4464,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4578,7 +4578,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4692,7 +4692,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:30 PM PT</t>
+          <t>2026-07-12 03:51:30 PM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4806,7 +4806,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4920,7 +4920,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:30 PM PT</t>
+          <t>2026-07-12 03:51:30 PM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5034,7 +5034,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:30 PM PT</t>
+          <t>2026-07-12 03:51:30 PM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5148,7 +5148,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5262,7 +5262,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5376,7 +5376,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5490,7 +5490,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:33 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5604,7 +5604,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5718,7 +5718,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5832,7 +5832,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5946,7 +5946,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6060,7 +6060,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6174,7 +6174,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:30 PM PT</t>
+          <t>2026-07-12 03:51:30 PM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:33 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6402,7 +6402,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6430,10 +6430,10 @@
         <v>0</v>
       </c>
       <c r="I52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J52" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K52" t="inlineStr">
         <is>
@@ -6525,7 +6525,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6639,7 +6639,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6753,7 +6753,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6867,7 +6867,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -6981,7 +6981,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:30 PM PT</t>
+          <t>2026-07-12 03:51:30 PM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7095,7 +7095,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7209,7 +7209,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7323,7 +7323,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7437,7 +7437,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7551,7 +7551,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7665,7 +7665,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7779,7 +7779,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7893,7 +7893,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -8007,7 +8007,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8121,7 +8121,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:33 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8235,7 +8235,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8349,7 +8349,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:33 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8463,7 +8463,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:33 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8577,7 +8577,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8691,7 +8691,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8719,10 +8719,10 @@
         <v>0</v>
       </c>
       <c r="I72" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J72" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K72" t="inlineStr">
         <is>
@@ -8814,7 +8814,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8842,10 +8842,10 @@
         <v>0</v>
       </c>
       <c r="I73" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J73" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K73" t="inlineStr">
         <is>
@@ -8937,7 +8937,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9051,7 +9051,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9165,7 +9165,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9279,7 +9279,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9393,7 +9393,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9507,7 +9507,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9621,7 +9621,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9735,7 +9735,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:33 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9849,7 +9849,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -9963,7 +9963,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10077,7 +10077,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10191,7 +10191,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10305,7 +10305,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10419,7 +10419,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10533,7 +10533,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10647,7 +10647,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10761,7 +10761,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:33 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10875,7 +10875,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -10989,7 +10989,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:33 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11103,7 +11103,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11131,10 +11131,10 @@
         <v>0</v>
       </c>
       <c r="I93" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J93" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K93" t="inlineStr">
         <is>
@@ -11226,7 +11226,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11340,7 +11340,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11454,7 +11454,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11568,7 +11568,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11682,7 +11682,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11796,7 +11796,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11824,10 +11824,10 @@
         <v>0</v>
       </c>
       <c r="I99" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J99" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K99" t="inlineStr">
         <is>
@@ -11919,7 +11919,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -12033,7 +12033,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:30 PM PT</t>
+          <t>2026-07-12 03:51:30 PM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12147,7 +12147,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:30 PM PT</t>
+          <t>2026-07-12 03:51:30 PM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12261,7 +12261,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:30 PM PT</t>
+          <t>2026-07-12 03:51:30 PM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12375,7 +12375,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:30 PM PT</t>
+          <t>2026-07-12 03:51:30 PM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12489,7 +12489,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12603,7 +12603,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12717,7 +12717,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12831,7 +12831,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:33 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12945,7 +12945,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13059,7 +13059,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13173,7 +13173,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13287,7 +13287,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13401,7 +13401,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13515,7 +13515,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:33 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13629,7 +13629,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13743,7 +13743,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13857,7 +13857,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -13971,7 +13971,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14085,7 +14085,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14199,7 +14199,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14313,7 +14313,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14341,10 +14341,10 @@
         <v>0</v>
       </c>
       <c r="I121" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J121" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K121" t="inlineStr">
         <is>
@@ -14436,7 +14436,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14550,7 +14550,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14664,7 +14664,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14778,7 +14778,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14892,7 +14892,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -15006,7 +15006,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15120,7 +15120,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15234,7 +15234,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15348,7 +15348,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15462,7 +15462,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15576,7 +15576,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15690,7 +15690,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15804,7 +15804,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -15918,7 +15918,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16032,7 +16032,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16146,7 +16146,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16260,7 +16260,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16374,7 +16374,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16488,7 +16488,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16602,7 +16602,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16716,7 +16716,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16830,7 +16830,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -16944,7 +16944,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17058,7 +17058,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17172,7 +17172,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17286,7 +17286,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17400,7 +17400,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17514,7 +17514,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17628,7 +17628,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17742,7 +17742,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17856,7 +17856,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:30 PM PT</t>
+          <t>2026-07-12 03:51:30 PM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -17970,7 +17970,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18084,7 +18084,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18198,7 +18198,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18312,7 +18312,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18426,7 +18426,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18454,10 +18454,10 @@
         <v>0</v>
       </c>
       <c r="I157" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J157" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K157" t="inlineStr">
         <is>
@@ -18549,7 +18549,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18663,7 +18663,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18777,7 +18777,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18891,7 +18891,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19005,7 +19005,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19119,7 +19119,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:33 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19233,7 +19233,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:33 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19347,7 +19347,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19461,7 +19461,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19575,7 +19575,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19689,7 +19689,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19803,7 +19803,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -19917,7 +19917,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -20031,7 +20031,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20145,7 +20145,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20259,7 +20259,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20373,7 +20373,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20487,7 +20487,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20601,7 +20601,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20715,7 +20715,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20829,7 +20829,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -20943,7 +20943,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21057,7 +21057,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21171,7 +21171,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21285,7 +21285,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21399,7 +21399,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:30 PM PT</t>
+          <t>2026-07-12 03:51:30 PM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21513,7 +21513,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21627,7 +21627,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21741,7 +21741,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21855,7 +21855,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -21969,7 +21969,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22083,7 +22083,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22197,7 +22197,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:33 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22311,7 +22311,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22425,7 +22425,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22539,7 +22539,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22653,7 +22653,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22767,7 +22767,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -22881,7 +22881,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -22995,7 +22995,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23109,7 +23109,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23223,7 +23223,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23337,7 +23337,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23451,7 +23451,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23565,7 +23565,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23679,7 +23679,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23793,7 +23793,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -23907,7 +23907,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -24021,7 +24021,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24135,7 +24135,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24249,7 +24249,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24363,7 +24363,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24477,7 +24477,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24591,7 +24591,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24619,10 +24619,10 @@
         <v>0</v>
       </c>
       <c r="I211" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J211" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K211" t="inlineStr">
         <is>
@@ -24714,7 +24714,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -24742,10 +24742,10 @@
         <v>0</v>
       </c>
       <c r="I212" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J212" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K212" t="inlineStr">
         <is>
@@ -24837,7 +24837,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -24865,10 +24865,10 @@
         <v>0</v>
       </c>
       <c r="I213" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J213" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K213" t="inlineStr">
         <is>
@@ -24960,7 +24960,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -25074,7 +25074,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:30 PM PT</t>
+          <t>2026-07-12 03:51:30 PM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25188,7 +25188,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25302,7 +25302,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25416,7 +25416,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25530,7 +25530,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25644,7 +25644,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25758,7 +25758,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -25872,7 +25872,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -25986,7 +25986,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26100,7 +26100,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26214,7 +26214,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26328,7 +26328,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:33 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26442,7 +26442,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:33 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26556,7 +26556,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26670,7 +26670,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26698,10 +26698,10 @@
         <v>0</v>
       </c>
       <c r="I229" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J229" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K229" t="inlineStr">
         <is>
@@ -26793,7 +26793,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -26821,10 +26821,10 @@
         <v>0</v>
       </c>
       <c r="I230" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J230" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K230" t="inlineStr">
         <is>
@@ -26916,7 +26916,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -26944,10 +26944,10 @@
         <v>0</v>
       </c>
       <c r="I231" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J231" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K231" t="inlineStr">
         <is>
@@ -27039,7 +27039,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27067,10 +27067,10 @@
         <v>0</v>
       </c>
       <c r="I232" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J232" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K232" t="inlineStr">
         <is>
@@ -27162,7 +27162,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27190,10 +27190,10 @@
         <v>0</v>
       </c>
       <c r="I233" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J233" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K233" t="inlineStr">
         <is>
@@ -27285,7 +27285,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27399,7 +27399,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -27513,7 +27513,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -27627,7 +27627,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -27741,7 +27741,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -27855,7 +27855,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -27969,7 +27969,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -28083,7 +28083,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -28197,7 +28197,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -28311,7 +28311,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -28425,7 +28425,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -28539,7 +28539,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -28653,7 +28653,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -28767,7 +28767,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -28881,7 +28881,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -28995,7 +28995,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -29109,7 +29109,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -29223,7 +29223,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -29337,7 +29337,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -29451,7 +29451,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -29565,7 +29565,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -29679,7 +29679,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -29793,7 +29793,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -29907,7 +29907,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -30021,7 +30021,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -30135,7 +30135,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -30249,7 +30249,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -30363,7 +30363,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -30477,7 +30477,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -30591,7 +30591,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -30705,7 +30705,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -30819,7 +30819,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -30933,7 +30933,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -30961,10 +30961,10 @@
         <v>0</v>
       </c>
       <c r="I266" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J266" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K266" t="inlineStr">
         <is>
@@ -31056,7 +31056,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -31084,10 +31084,10 @@
         <v>0</v>
       </c>
       <c r="I267" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J267" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K267" t="inlineStr">
         <is>
@@ -31179,7 +31179,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -31207,10 +31207,10 @@
         <v>0</v>
       </c>
       <c r="I268" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J268" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K268" t="inlineStr">
         <is>
@@ -31302,7 +31302,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -31330,10 +31330,10 @@
         <v>0</v>
       </c>
       <c r="I269" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J269" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K269" t="inlineStr">
         <is>
@@ -31425,7 +31425,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -31539,7 +31539,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -31653,7 +31653,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -31767,7 +31767,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -31881,7 +31881,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -31995,7 +31995,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -32109,7 +32109,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:30 PM PT</t>
+          <t>2026-07-12 03:51:30 PM PT</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -32223,7 +32223,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:30 PM PT</t>
+          <t>2026-07-12 03:51:30 PM PT</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -32337,7 +32337,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:30 PM PT</t>
+          <t>2026-07-12 03:51:30 PM PT</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -32451,7 +32451,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C279" t="n">
@@ -32565,7 +32565,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -32679,7 +32679,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C281" t="n">
@@ -32793,7 +32793,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C282" t="n">
@@ -32907,7 +32907,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -33021,7 +33021,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -33135,7 +33135,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -33249,7 +33249,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -33363,7 +33363,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -33477,7 +33477,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -33591,7 +33591,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -33705,7 +33705,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -33819,7 +33819,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C291" t="n">
@@ -33933,7 +33933,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C292" t="n">
@@ -34047,7 +34047,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C293" t="n">
@@ -34161,7 +34161,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C294" t="n">
@@ -34275,7 +34275,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:30 PM PT</t>
+          <t>2026-07-12 03:51:30 PM PT</t>
         </is>
       </c>
       <c r="C295" t="n">
@@ -34389,7 +34389,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:30 PM PT</t>
+          <t>2026-07-12 03:51:30 PM PT</t>
         </is>
       </c>
       <c r="C296" t="n">
@@ -34503,7 +34503,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:30 PM PT</t>
+          <t>2026-07-12 03:51:30 PM PT</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -34617,7 +34617,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:33 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -34731,7 +34731,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:33 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C299" t="n">
@@ -34845,7 +34845,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:33 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C300" t="n">
@@ -34959,7 +34959,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C301" t="n">
@@ -35073,7 +35073,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C302" t="n">
@@ -35187,7 +35187,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C303" t="n">
@@ -35301,7 +35301,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C304" t="n">
@@ -35415,7 +35415,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C305" t="n">
@@ -35529,7 +35529,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C306" t="n">
@@ -35643,7 +35643,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C307" t="n">
@@ -35757,7 +35757,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C308" t="n">
@@ -35871,7 +35871,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C309" t="n">
@@ -35985,7 +35985,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -36099,7 +36099,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -36213,7 +36213,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -36327,7 +36327,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:32 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -36441,7 +36441,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:33 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -36555,7 +36555,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:33 PM PT</t>
+          <t>2026-07-12 03:51:32 PM PT</t>
         </is>
       </c>
       <c r="C315" t="n">
@@ -36669,7 +36669,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C316" t="n">
@@ -36783,7 +36783,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C317" t="n">
@@ -36897,7 +36897,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C318" t="n">
@@ -37011,7 +37011,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C319" t="n">
@@ -37125,7 +37125,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>2026-07-12 03:49:31 PM PT</t>
+          <t>2026-07-12 03:51:31 PM PT</t>
         </is>
       </c>
       <c r="C320" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-12 03:53:34 PM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -807,7 +807,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:30 PM PT</t>
+          <t>2026-07-12 03:53:30 PM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -921,7 +921,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 1 out</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -1516,10 +1516,10 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J9" t="n">
         <v>2</v>
@@ -1614,7 +1614,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1728,7 +1728,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1842,7 +1842,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:30 PM PT</t>
+          <t>2026-07-12 03:53:30 PM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1956,7 +1956,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2070,7 +2070,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:30 PM PT</t>
+          <t>2026-07-12 03:53:30 PM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2184,7 +2184,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2298,7 +2298,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:30 PM PT</t>
+          <t>2026-07-12 03:53:30 PM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2412,7 +2412,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2640,7 +2640,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2754,7 +2754,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2868,7 +2868,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2982,7 +2982,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:30 PM PT</t>
+          <t>2026-07-12 03:53:30 PM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3096,7 +3096,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3324,7 +3324,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3438,7 +3438,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3552,7 +3552,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3666,7 +3666,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3780,7 +3780,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3894,7 +3894,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -4008,7 +4008,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4122,7 +4122,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4236,7 +4236,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4350,7 +4350,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4464,7 +4464,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4578,7 +4578,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4692,7 +4692,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:30 PM PT</t>
+          <t>2026-07-12 03:53:30 PM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4806,7 +4806,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4920,7 +4920,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:30 PM PT</t>
+          <t>2026-07-12 03:53:30 PM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5034,7 +5034,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:30 PM PT</t>
+          <t>2026-07-12 03:53:30 PM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5148,7 +5148,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5262,7 +5262,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5376,7 +5376,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5490,7 +5490,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5604,7 +5604,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5718,7 +5718,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5832,7 +5832,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5946,7 +5946,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6060,7 +6060,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6174,7 +6174,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:30 PM PT</t>
+          <t>2026-07-12 03:53:30 PM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6402,7 +6402,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6415,7 +6415,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 1 out</t>
         </is>
       </c>
       <c r="F52" t="n">
@@ -6427,10 +6427,10 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J52" t="n">
         <v>2</v>
@@ -6469,10 +6469,10 @@
         </is>
       </c>
       <c r="R52" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S52" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T52" t="n">
         <v>2</v>
@@ -6525,7 +6525,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6639,7 +6639,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6753,7 +6753,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6867,7 +6867,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -6981,7 +6981,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:30 PM PT</t>
+          <t>2026-07-12 03:53:30 PM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7095,7 +7095,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7209,7 +7209,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7323,7 +7323,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7437,7 +7437,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7551,7 +7551,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7665,7 +7665,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7779,7 +7779,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7893,7 +7893,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -8007,7 +8007,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8121,7 +8121,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8235,7 +8235,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8349,7 +8349,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8463,7 +8463,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8577,7 +8577,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8691,7 +8691,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8704,7 +8704,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 1 out</t>
         </is>
       </c>
       <c r="F72" t="n">
@@ -8716,10 +8716,10 @@
         </is>
       </c>
       <c r="H72" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I72" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J72" t="n">
         <v>2</v>
@@ -8814,7 +8814,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8827,7 +8827,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 1 out</t>
         </is>
       </c>
       <c r="F73" t="n">
@@ -8839,10 +8839,10 @@
         </is>
       </c>
       <c r="H73" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I73" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J73" t="n">
         <v>2</v>
@@ -8937,7 +8937,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9051,7 +9051,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9165,7 +9165,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9279,7 +9279,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9393,7 +9393,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9507,7 +9507,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9621,7 +9621,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9735,7 +9735,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9849,7 +9849,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -9963,7 +9963,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10077,7 +10077,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10191,7 +10191,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10305,7 +10305,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10419,7 +10419,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10533,7 +10533,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10647,7 +10647,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10761,7 +10761,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10875,7 +10875,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -10989,7 +10989,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11103,7 +11103,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11116,7 +11116,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 1 out</t>
         </is>
       </c>
       <c r="F93" t="n">
@@ -11128,10 +11128,10 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I93" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J93" t="n">
         <v>2</v>
@@ -11226,7 +11226,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11340,7 +11340,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11454,7 +11454,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11568,7 +11568,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11682,7 +11682,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11796,7 +11796,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11809,7 +11809,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 1 out</t>
         </is>
       </c>
       <c r="F99" t="n">
@@ -11821,10 +11821,10 @@
         </is>
       </c>
       <c r="H99" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I99" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J99" t="n">
         <v>2</v>
@@ -11919,7 +11919,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -12033,7 +12033,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:30 PM PT</t>
+          <t>2026-07-12 03:53:30 PM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12147,7 +12147,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:30 PM PT</t>
+          <t>2026-07-12 03:53:30 PM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12261,7 +12261,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:30 PM PT</t>
+          <t>2026-07-12 03:53:30 PM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12375,7 +12375,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:30 PM PT</t>
+          <t>2026-07-12 03:53:30 PM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12489,7 +12489,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12603,7 +12603,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12717,7 +12717,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12831,7 +12831,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12945,7 +12945,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13059,7 +13059,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13173,7 +13173,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13287,7 +13287,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13401,7 +13401,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13515,7 +13515,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13629,7 +13629,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13743,7 +13743,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13857,7 +13857,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -13971,7 +13971,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14085,7 +14085,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14199,7 +14199,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14313,7 +14313,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14326,7 +14326,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 1 out</t>
         </is>
       </c>
       <c r="F121" t="n">
@@ -14338,10 +14338,10 @@
         </is>
       </c>
       <c r="H121" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I121" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J121" t="n">
         <v>2</v>
@@ -14436,7 +14436,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14550,7 +14550,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14664,7 +14664,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14778,7 +14778,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14892,7 +14892,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -15006,7 +15006,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15120,7 +15120,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15234,7 +15234,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15348,7 +15348,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15462,7 +15462,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15576,7 +15576,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15690,7 +15690,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15804,7 +15804,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -15918,7 +15918,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16032,7 +16032,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16146,7 +16146,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16260,7 +16260,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16374,7 +16374,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16488,7 +16488,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16602,7 +16602,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16716,7 +16716,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16830,7 +16830,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -16944,7 +16944,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17058,7 +17058,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17172,7 +17172,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17286,7 +17286,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17400,7 +17400,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17514,7 +17514,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17628,7 +17628,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17742,7 +17742,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17856,7 +17856,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:30 PM PT</t>
+          <t>2026-07-12 03:53:30 PM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -17970,7 +17970,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18084,7 +18084,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18198,7 +18198,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18312,7 +18312,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18426,7 +18426,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18439,7 +18439,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 1 out</t>
         </is>
       </c>
       <c r="F157" t="n">
@@ -18451,10 +18451,10 @@
         </is>
       </c>
       <c r="H157" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I157" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J157" t="n">
         <v>2</v>
@@ -18549,7 +18549,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18663,7 +18663,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18777,7 +18777,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18891,7 +18891,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19005,7 +19005,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19119,7 +19119,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19233,7 +19233,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19347,7 +19347,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19461,7 +19461,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19575,7 +19575,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19689,7 +19689,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19803,7 +19803,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -19917,7 +19917,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -20031,7 +20031,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20145,7 +20145,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20259,7 +20259,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20373,7 +20373,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20487,7 +20487,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20601,7 +20601,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20715,7 +20715,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20829,7 +20829,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -20943,7 +20943,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21057,7 +21057,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21171,7 +21171,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21285,7 +21285,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21399,7 +21399,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:30 PM PT</t>
+          <t>2026-07-12 03:53:30 PM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21513,7 +21513,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21627,7 +21627,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21741,7 +21741,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21855,7 +21855,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -21969,7 +21969,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22083,7 +22083,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22197,7 +22197,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22311,7 +22311,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22425,7 +22425,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22539,7 +22539,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22653,7 +22653,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22767,7 +22767,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -22881,7 +22881,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -22995,7 +22995,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23109,7 +23109,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23223,7 +23223,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23337,7 +23337,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23451,7 +23451,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23565,7 +23565,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23679,7 +23679,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23793,7 +23793,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -23907,7 +23907,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -24021,7 +24021,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24135,7 +24135,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24249,7 +24249,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24363,7 +24363,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24477,7 +24477,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24591,7 +24591,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24604,7 +24604,7 @@
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 1 out</t>
         </is>
       </c>
       <c r="F211" t="n">
@@ -24616,10 +24616,10 @@
         </is>
       </c>
       <c r="H211" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I211" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J211" t="n">
         <v>2</v>
@@ -24714,7 +24714,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -24727,7 +24727,7 @@
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 1 out</t>
         </is>
       </c>
       <c r="F212" t="n">
@@ -24739,10 +24739,10 @@
         </is>
       </c>
       <c r="H212" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I212" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J212" t="n">
         <v>2</v>
@@ -24837,7 +24837,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -24850,7 +24850,7 @@
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 1 out</t>
         </is>
       </c>
       <c r="F213" t="n">
@@ -24862,10 +24862,10 @@
         </is>
       </c>
       <c r="H213" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I213" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J213" t="n">
         <v>2</v>
@@ -24960,7 +24960,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -25074,7 +25074,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:30 PM PT</t>
+          <t>2026-07-12 03:53:30 PM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25188,7 +25188,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25302,7 +25302,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25416,7 +25416,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25530,7 +25530,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25644,7 +25644,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25758,7 +25758,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -25872,7 +25872,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -25986,7 +25986,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26100,7 +26100,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26214,7 +26214,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26328,7 +26328,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26442,7 +26442,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26556,7 +26556,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26670,7 +26670,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26683,7 +26683,7 @@
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 1 out</t>
         </is>
       </c>
       <c r="F229" t="n">
@@ -26695,10 +26695,10 @@
         </is>
       </c>
       <c r="H229" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I229" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J229" t="n">
         <v>2</v>
@@ -26793,7 +26793,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -26806,7 +26806,7 @@
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 1 out</t>
         </is>
       </c>
       <c r="F230" t="n">
@@ -26818,10 +26818,10 @@
         </is>
       </c>
       <c r="H230" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I230" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J230" t="n">
         <v>2</v>
@@ -26916,7 +26916,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -26929,7 +26929,7 @@
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 1 out</t>
         </is>
       </c>
       <c r="F231" t="n">
@@ -26941,10 +26941,10 @@
         </is>
       </c>
       <c r="H231" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I231" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J231" t="n">
         <v>2</v>
@@ -27039,7 +27039,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27052,7 +27052,7 @@
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 1 out</t>
         </is>
       </c>
       <c r="F232" t="n">
@@ -27064,10 +27064,10 @@
         </is>
       </c>
       <c r="H232" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I232" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J232" t="n">
         <v>2</v>
@@ -27162,7 +27162,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27175,7 +27175,7 @@
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 1 out</t>
         </is>
       </c>
       <c r="F233" t="n">
@@ -27187,10 +27187,10 @@
         </is>
       </c>
       <c r="H233" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I233" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J233" t="n">
         <v>2</v>
@@ -27285,7 +27285,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27399,7 +27399,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -27513,7 +27513,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -27627,7 +27627,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -27741,7 +27741,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -27855,7 +27855,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -27969,7 +27969,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -28083,7 +28083,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -28197,7 +28197,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -28311,7 +28311,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -28425,7 +28425,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -28539,7 +28539,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -28653,7 +28653,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -28767,7 +28767,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -28881,7 +28881,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -28995,7 +28995,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -29109,7 +29109,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -29223,7 +29223,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -29337,7 +29337,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -29451,7 +29451,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -29565,7 +29565,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -29679,7 +29679,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -29793,7 +29793,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -29907,7 +29907,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -30021,7 +30021,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -30135,7 +30135,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -30249,7 +30249,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -30363,7 +30363,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -30477,7 +30477,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -30591,7 +30591,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -30705,7 +30705,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -30819,7 +30819,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -30933,7 +30933,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -30946,7 +30946,7 @@
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 1 out</t>
         </is>
       </c>
       <c r="F266" t="n">
@@ -30958,10 +30958,10 @@
         </is>
       </c>
       <c r="H266" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I266" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J266" t="n">
         <v>2</v>
@@ -31056,7 +31056,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -31069,7 +31069,7 @@
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 1 out</t>
         </is>
       </c>
       <c r="F267" t="n">
@@ -31081,10 +31081,10 @@
         </is>
       </c>
       <c r="H267" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I267" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J267" t="n">
         <v>2</v>
@@ -31179,7 +31179,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -31192,7 +31192,7 @@
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 1 out</t>
         </is>
       </c>
       <c r="F268" t="n">
@@ -31204,10 +31204,10 @@
         </is>
       </c>
       <c r="H268" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I268" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J268" t="n">
         <v>2</v>
@@ -31302,7 +31302,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -31315,7 +31315,7 @@
       </c>
       <c r="E269" t="inlineStr">
         <is>
-          <t>Top 9 | 0 out</t>
+          <t>Top 9 | 1 out</t>
         </is>
       </c>
       <c r="F269" t="n">
@@ -31327,10 +31327,10 @@
         </is>
       </c>
       <c r="H269" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I269" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J269" t="n">
         <v>2</v>
@@ -31425,7 +31425,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -31539,7 +31539,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -31653,7 +31653,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -31767,7 +31767,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -31881,7 +31881,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -31995,7 +31995,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -32109,7 +32109,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:30 PM PT</t>
+          <t>2026-07-12 03:53:30 PM PT</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -32223,7 +32223,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:30 PM PT</t>
+          <t>2026-07-12 03:53:30 PM PT</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -32337,7 +32337,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:30 PM PT</t>
+          <t>2026-07-12 03:53:30 PM PT</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -32451,7 +32451,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C279" t="n">
@@ -32565,7 +32565,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -32679,7 +32679,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C281" t="n">
@@ -32793,7 +32793,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C282" t="n">
@@ -32907,7 +32907,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -33021,7 +33021,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -33135,7 +33135,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -33249,7 +33249,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -33363,7 +33363,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -33477,7 +33477,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -33591,7 +33591,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -33705,7 +33705,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -33819,7 +33819,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C291" t="n">
@@ -33933,7 +33933,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C292" t="n">
@@ -34047,7 +34047,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C293" t="n">
@@ -34161,7 +34161,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C294" t="n">
@@ -34275,7 +34275,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:30 PM PT</t>
+          <t>2026-07-12 03:53:30 PM PT</t>
         </is>
       </c>
       <c r="C295" t="n">
@@ -34389,7 +34389,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:30 PM PT</t>
+          <t>2026-07-12 03:53:30 PM PT</t>
         </is>
       </c>
       <c r="C296" t="n">
@@ -34503,7 +34503,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:30 PM PT</t>
+          <t>2026-07-12 03:53:30 PM PT</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -34617,7 +34617,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -34731,7 +34731,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C299" t="n">
@@ -34845,7 +34845,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C300" t="n">
@@ -34959,7 +34959,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C301" t="n">
@@ -35073,7 +35073,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C302" t="n">
@@ -35187,7 +35187,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C303" t="n">
@@ -35301,7 +35301,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C304" t="n">
@@ -35415,7 +35415,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C305" t="n">
@@ -35529,7 +35529,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C306" t="n">
@@ -35643,7 +35643,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C307" t="n">
@@ -35757,7 +35757,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C308" t="n">
@@ -35871,7 +35871,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C309" t="n">
@@ -35985,7 +35985,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -36099,7 +36099,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -36213,7 +36213,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -36327,7 +36327,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -36441,7 +36441,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -36555,7 +36555,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:32 PM PT</t>
+          <t>2026-07-12 03:53:32 PM PT</t>
         </is>
       </c>
       <c r="C315" t="n">
@@ -36669,7 +36669,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C316" t="n">
@@ -36783,7 +36783,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C317" t="n">
@@ -36897,7 +36897,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C318" t="n">
@@ -37011,7 +37011,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C319" t="n">
@@ -37125,7 +37125,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>2026-07-12 03:51:31 PM PT</t>
+          <t>2026-07-12 03:53:31 PM PT</t>
         </is>
       </c>
       <c r="C320" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-12 03:55:34 PM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -807,7 +807,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:30 PM PT</t>
+          <t>2026-07-12 03:55:30 PM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -921,7 +921,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Top 9 | 1 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -1516,10 +1516,10 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J9" t="n">
         <v>2</v>
@@ -1614,7 +1614,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1728,7 +1728,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1842,7 +1842,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:30 PM PT</t>
+          <t>2026-07-12 03:55:30 PM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1956,7 +1956,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2070,7 +2070,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:30 PM PT</t>
+          <t>2026-07-12 03:55:30 PM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2184,7 +2184,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2298,7 +2298,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:30 PM PT</t>
+          <t>2026-07-12 03:55:30 PM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2412,7 +2412,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2640,7 +2640,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2754,7 +2754,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2868,7 +2868,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2982,7 +2982,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:30 PM PT</t>
+          <t>2026-07-12 03:55:30 PM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3096,7 +3096,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3324,7 +3324,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3438,7 +3438,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3552,7 +3552,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3666,7 +3666,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3780,7 +3780,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3894,7 +3894,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -4008,7 +4008,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4122,7 +4122,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4236,7 +4236,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4350,7 +4350,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4464,7 +4464,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4578,7 +4578,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4692,7 +4692,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:30 PM PT</t>
+          <t>2026-07-12 03:55:30 PM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4806,7 +4806,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4920,7 +4920,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:30 PM PT</t>
+          <t>2026-07-12 03:55:30 PM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5034,7 +5034,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:30 PM PT</t>
+          <t>2026-07-12 03:55:30 PM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5148,7 +5148,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5262,7 +5262,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5376,7 +5376,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5490,7 +5490,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5604,7 +5604,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5718,7 +5718,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5832,7 +5832,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5946,7 +5946,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6060,7 +6060,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6174,7 +6174,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:30 PM PT</t>
+          <t>2026-07-12 03:55:30 PM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6288,7 +6288,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6402,7 +6402,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6415,7 +6415,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Top 9 | 1 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F52" t="n">
@@ -6427,10 +6427,10 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J52" t="n">
         <v>2</v>
@@ -6525,7 +6525,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6639,7 +6639,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6753,7 +6753,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6867,7 +6867,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -6981,7 +6981,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:30 PM PT</t>
+          <t>2026-07-12 03:55:30 PM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7095,7 +7095,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7209,7 +7209,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7323,7 +7323,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7437,7 +7437,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7551,7 +7551,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7665,7 +7665,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7779,7 +7779,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7893,7 +7893,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -8007,7 +8007,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8121,7 +8121,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8235,7 +8235,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8349,7 +8349,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8463,7 +8463,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8577,7 +8577,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8691,7 +8691,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8704,7 +8704,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Top 9 | 1 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F72" t="n">
@@ -8716,10 +8716,10 @@
         </is>
       </c>
       <c r="H72" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I72" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J72" t="n">
         <v>2</v>
@@ -8758,10 +8758,10 @@
         </is>
       </c>
       <c r="R72" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S72" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T72" t="n">
         <v>1</v>
@@ -8814,7 +8814,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8827,7 +8827,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Top 9 | 1 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F73" t="n">
@@ -8839,10 +8839,10 @@
         </is>
       </c>
       <c r="H73" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I73" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J73" t="n">
         <v>2</v>
@@ -8937,7 +8937,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -9051,7 +9051,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9165,7 +9165,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9279,7 +9279,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9393,7 +9393,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9507,7 +9507,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9621,7 +9621,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9735,7 +9735,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9849,7 +9849,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -9963,7 +9963,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10077,7 +10077,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10191,7 +10191,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10305,7 +10305,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10419,7 +10419,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10533,7 +10533,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10647,7 +10647,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10761,7 +10761,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10875,7 +10875,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -10989,7 +10989,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11103,7 +11103,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11116,7 +11116,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Top 9 | 1 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F93" t="n">
@@ -11128,10 +11128,10 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I93" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J93" t="n">
         <v>2</v>
@@ -11226,7 +11226,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11340,7 +11340,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11454,7 +11454,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11568,7 +11568,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11682,7 +11682,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11796,7 +11796,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11809,7 +11809,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Top 9 | 1 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F99" t="n">
@@ -11821,10 +11821,10 @@
         </is>
       </c>
       <c r="H99" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I99" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J99" t="n">
         <v>2</v>
@@ -11919,7 +11919,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -12033,7 +12033,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:30 PM PT</t>
+          <t>2026-07-12 03:55:30 PM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12147,7 +12147,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:30 PM PT</t>
+          <t>2026-07-12 03:55:30 PM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12261,7 +12261,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:30 PM PT</t>
+          <t>2026-07-12 03:55:30 PM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12375,7 +12375,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:30 PM PT</t>
+          <t>2026-07-12 03:55:30 PM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12489,7 +12489,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12603,7 +12603,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12717,7 +12717,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12831,7 +12831,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12945,7 +12945,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13059,7 +13059,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13173,7 +13173,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13287,7 +13287,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13401,7 +13401,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13515,7 +13515,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13629,7 +13629,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13743,7 +13743,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13857,7 +13857,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -13971,7 +13971,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14085,7 +14085,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14199,7 +14199,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14313,7 +14313,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14326,7 +14326,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Top 9 | 1 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F121" t="n">
@@ -14338,10 +14338,10 @@
         </is>
       </c>
       <c r="H121" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I121" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J121" t="n">
         <v>2</v>
@@ -14436,7 +14436,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14550,7 +14550,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14664,7 +14664,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14778,7 +14778,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14892,7 +14892,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -15006,7 +15006,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15120,7 +15120,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15234,7 +15234,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15348,7 +15348,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15462,7 +15462,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15576,7 +15576,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15690,7 +15690,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15804,7 +15804,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -15918,7 +15918,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16032,7 +16032,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16146,7 +16146,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16260,7 +16260,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16374,7 +16374,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16488,7 +16488,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16602,7 +16602,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16716,7 +16716,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16830,7 +16830,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -16944,7 +16944,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17058,7 +17058,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17172,7 +17172,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17286,7 +17286,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17400,7 +17400,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17514,7 +17514,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17628,7 +17628,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17742,7 +17742,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17856,7 +17856,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:30 PM PT</t>
+          <t>2026-07-12 03:55:30 PM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -17970,7 +17970,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18084,7 +18084,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18198,7 +18198,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18312,7 +18312,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18426,7 +18426,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18439,7 +18439,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>Top 9 | 1 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F157" t="n">
@@ -18451,10 +18451,10 @@
         </is>
       </c>
       <c r="H157" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I157" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J157" t="n">
         <v>2</v>
@@ -18549,7 +18549,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18663,7 +18663,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18777,7 +18777,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18891,7 +18891,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19005,7 +19005,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19119,7 +19119,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19233,7 +19233,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19347,7 +19347,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19461,7 +19461,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19575,7 +19575,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19689,7 +19689,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19803,7 +19803,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -19917,7 +19917,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -20031,7 +20031,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20145,7 +20145,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20259,7 +20259,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20373,7 +20373,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20487,7 +20487,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20601,7 +20601,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20715,7 +20715,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20829,7 +20829,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -20943,7 +20943,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21057,7 +21057,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21171,7 +21171,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21285,7 +21285,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21399,7 +21399,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:30 PM PT</t>
+          <t>2026-07-12 03:55:30 PM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21513,7 +21513,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21627,7 +21627,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21741,7 +21741,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21855,7 +21855,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -21969,7 +21969,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22083,7 +22083,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22197,7 +22197,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22311,7 +22311,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22425,7 +22425,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22539,7 +22539,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22653,7 +22653,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22767,7 +22767,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -22881,7 +22881,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -22995,7 +22995,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23109,7 +23109,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23223,7 +23223,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23337,7 +23337,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23451,7 +23451,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23565,7 +23565,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23679,7 +23679,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23793,7 +23793,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -23907,7 +23907,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -24021,7 +24021,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24135,7 +24135,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24249,7 +24249,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24363,7 +24363,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24477,7 +24477,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24591,7 +24591,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24604,7 +24604,7 @@
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>Top 9 | 1 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F211" t="n">
@@ -24616,10 +24616,10 @@
         </is>
       </c>
       <c r="H211" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I211" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J211" t="n">
         <v>2</v>
@@ -24714,7 +24714,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -24727,7 +24727,7 @@
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>Top 9 | 1 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F212" t="n">
@@ -24739,10 +24739,10 @@
         </is>
       </c>
       <c r="H212" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I212" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J212" t="n">
         <v>2</v>
@@ -24837,7 +24837,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -24850,7 +24850,7 @@
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>Top 9 | 1 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F213" t="n">
@@ -24862,10 +24862,10 @@
         </is>
       </c>
       <c r="H213" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I213" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J213" t="n">
         <v>2</v>
@@ -24960,7 +24960,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -25074,7 +25074,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:30 PM PT</t>
+          <t>2026-07-12 03:55:30 PM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25188,7 +25188,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25302,7 +25302,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25416,7 +25416,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25530,7 +25530,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25644,7 +25644,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25758,7 +25758,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -25872,7 +25872,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -25986,7 +25986,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26100,7 +26100,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26214,7 +26214,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26328,7 +26328,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26442,7 +26442,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26556,7 +26556,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26670,7 +26670,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26683,7 +26683,7 @@
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>Top 9 | 1 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F229" t="n">
@@ -26695,10 +26695,10 @@
         </is>
       </c>
       <c r="H229" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I229" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J229" t="n">
         <v>2</v>
@@ -26793,7 +26793,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -26806,7 +26806,7 @@
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>Top 9 | 1 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F230" t="n">
@@ -26818,10 +26818,10 @@
         </is>
       </c>
       <c r="H230" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I230" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J230" t="n">
         <v>2</v>
@@ -26916,7 +26916,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -26929,7 +26929,7 @@
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>Top 9 | 1 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F231" t="n">
@@ -26941,10 +26941,10 @@
         </is>
       </c>
       <c r="H231" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I231" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J231" t="n">
         <v>2</v>
@@ -27039,7 +27039,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27052,7 +27052,7 @@
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>Top 9 | 1 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F232" t="n">
@@ -27064,10 +27064,10 @@
         </is>
       </c>
       <c r="H232" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I232" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J232" t="n">
         <v>2</v>
@@ -27162,7 +27162,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27175,7 +27175,7 @@
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>Top 9 | 1 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F233" t="n">
@@ -27187,10 +27187,10 @@
         </is>
       </c>
       <c r="H233" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I233" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J233" t="n">
         <v>2</v>
@@ -27285,7 +27285,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27399,7 +27399,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -27513,7 +27513,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -27627,7 +27627,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -27741,7 +27741,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -27855,7 +27855,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -27969,7 +27969,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -28083,7 +28083,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -28197,7 +28197,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -28311,7 +28311,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -28425,7 +28425,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -28539,7 +28539,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -28653,7 +28653,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -28767,7 +28767,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -28881,7 +28881,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -28995,7 +28995,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -29109,7 +29109,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -29223,7 +29223,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -29337,7 +29337,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -29451,7 +29451,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -29565,7 +29565,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -29679,7 +29679,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -29793,7 +29793,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -29907,7 +29907,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -30021,7 +30021,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -30135,7 +30135,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -30249,7 +30249,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -30363,7 +30363,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -30477,7 +30477,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -30591,7 +30591,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -30705,7 +30705,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -30819,7 +30819,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -30933,7 +30933,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -30946,7 +30946,7 @@
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>Top 9 | 1 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F266" t="n">
@@ -30958,10 +30958,10 @@
         </is>
       </c>
       <c r="H266" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I266" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J266" t="n">
         <v>2</v>
@@ -31056,7 +31056,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -31069,7 +31069,7 @@
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>Top 9 | 1 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F267" t="n">
@@ -31081,10 +31081,10 @@
         </is>
       </c>
       <c r="H267" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I267" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J267" t="n">
         <v>2</v>
@@ -31179,7 +31179,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -31192,7 +31192,7 @@
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>Top 9 | 1 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F268" t="n">
@@ -31204,10 +31204,10 @@
         </is>
       </c>
       <c r="H268" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I268" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J268" t="n">
         <v>2</v>
@@ -31302,7 +31302,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -31315,7 +31315,7 @@
       </c>
       <c r="E269" t="inlineStr">
         <is>
-          <t>Top 9 | 1 out</t>
+          <t>Top 9 | 2 out</t>
         </is>
       </c>
       <c r="F269" t="n">
@@ -31327,10 +31327,10 @@
         </is>
       </c>
       <c r="H269" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I269" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J269" t="n">
         <v>2</v>
@@ -31425,7 +31425,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -31539,7 +31539,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -31653,7 +31653,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -31767,7 +31767,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -31881,7 +31881,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -31995,7 +31995,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -32109,7 +32109,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:30 PM PT</t>
+          <t>2026-07-12 03:55:30 PM PT</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -32223,7 +32223,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:30 PM PT</t>
+          <t>2026-07-12 03:55:30 PM PT</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -32337,7 +32337,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:30 PM PT</t>
+          <t>2026-07-12 03:55:30 PM PT</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -32451,7 +32451,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C279" t="n">
@@ -32565,7 +32565,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -32679,7 +32679,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C281" t="n">
@@ -32793,7 +32793,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C282" t="n">
@@ -32907,7 +32907,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -33021,7 +33021,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -33135,7 +33135,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -33249,7 +33249,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -33363,7 +33363,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -33477,7 +33477,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -33591,7 +33591,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -33705,7 +33705,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -33819,7 +33819,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C291" t="n">
@@ -33933,7 +33933,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C292" t="n">
@@ -34047,7 +34047,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C293" t="n">
@@ -34161,7 +34161,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C294" t="n">
@@ -34275,7 +34275,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:30 PM PT</t>
+          <t>2026-07-12 03:55:30 PM PT</t>
         </is>
       </c>
       <c r="C295" t="n">
@@ -34389,7 +34389,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:30 PM PT</t>
+          <t>2026-07-12 03:55:30 PM PT</t>
         </is>
       </c>
       <c r="C296" t="n">
@@ -34503,7 +34503,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:30 PM PT</t>
+          <t>2026-07-12 03:55:30 PM PT</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -34617,7 +34617,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -34731,7 +34731,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C299" t="n">
@@ -34845,7 +34845,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C300" t="n">
@@ -34959,7 +34959,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C301" t="n">
@@ -35073,7 +35073,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C302" t="n">
@@ -35187,7 +35187,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C303" t="n">
@@ -35301,7 +35301,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C304" t="n">
@@ -35415,7 +35415,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C305" t="n">
@@ -35529,7 +35529,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C306" t="n">
@@ -35643,7 +35643,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C307" t="n">
@@ -35757,7 +35757,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C308" t="n">
@@ -35871,7 +35871,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C309" t="n">
@@ -35985,7 +35985,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -36099,7 +36099,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -36213,7 +36213,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -36327,7 +36327,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -36441,7 +36441,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -36555,7 +36555,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:32 PM PT</t>
+          <t>2026-07-12 03:55:32 PM PT</t>
         </is>
       </c>
       <c r="C315" t="n">
@@ -36669,7 +36669,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C316" t="n">
@@ -36783,7 +36783,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C317" t="n">
@@ -36897,7 +36897,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C318" t="n">
@@ -37011,7 +37011,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C319" t="n">
@@ -37125,7 +37125,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>2026-07-12 03:53:31 PM PT</t>
+          <t>2026-07-12 03:55:31 PM PT</t>
         </is>
       </c>
       <c r="C320" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-12 03:59:33 PM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
@@ -487,7 +487,7 @@
     <col width="27" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
@@ -693,7 +693,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -807,7 +807,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:30 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -921,7 +921,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -1512,17 +1512,17 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -1614,7 +1614,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1728,7 +1728,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1842,7 +1842,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:30 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1956,7 +1956,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2070,7 +2070,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:30 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2184,7 +2184,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2298,7 +2298,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:30 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2412,7 +2412,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2640,7 +2640,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2754,7 +2754,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2868,7 +2868,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2982,7 +2982,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:30 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3096,7 +3096,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3324,7 +3324,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3438,7 +3438,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3552,7 +3552,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3565,7 +3565,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F27" t="n">
@@ -3573,17 +3573,17 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H27" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I27" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
@@ -3675,7 +3675,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3789,7 +3789,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3903,7 +3903,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -4017,7 +4017,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4131,7 +4131,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4245,7 +4245,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4359,7 +4359,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4473,7 +4473,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4587,7 +4587,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4701,7 +4701,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4815,7 +4815,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:30 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4929,7 +4929,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5043,7 +5043,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:30 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5157,7 +5157,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:30 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5271,7 +5271,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5385,7 +5385,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5499,7 +5499,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5613,7 +5613,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5727,7 +5727,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5841,7 +5841,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5955,7 +5955,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6069,7 +6069,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6183,7 +6183,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6297,7 +6297,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:30 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6411,7 +6411,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6525,7 +6525,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6538,7 +6538,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F53" t="n">
@@ -6546,17 +6546,17 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H53" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I53" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J53" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K53" t="inlineStr">
         <is>
@@ -6648,7 +6648,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6762,7 +6762,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6876,7 +6876,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -6990,7 +6990,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7104,7 +7104,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:30 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7218,7 +7218,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7332,7 +7332,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7446,7 +7446,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7560,7 +7560,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7674,7 +7674,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7788,7 +7788,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7902,7 +7902,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -8016,7 +8016,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8130,7 +8130,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8244,7 +8244,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8358,7 +8358,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8472,7 +8472,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8586,7 +8586,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8700,7 +8700,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8827,7 +8827,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F73" t="n">
@@ -8835,17 +8835,17 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H73" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I73" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J73" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K73" t="inlineStr">
         <is>
@@ -8937,7 +8937,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -8950,7 +8950,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F74" t="n">
@@ -8958,17 +8958,17 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H74" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I74" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J74" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K74" t="inlineStr">
         <is>
@@ -9004,10 +9004,10 @@
         </is>
       </c>
       <c r="R74" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S74" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T74" t="n">
         <v>0</v>
@@ -9060,7 +9060,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9174,7 +9174,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9288,7 +9288,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9402,7 +9402,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9516,7 +9516,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9630,7 +9630,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9744,7 +9744,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9858,7 +9858,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -9972,7 +9972,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10086,7 +10086,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10200,7 +10200,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10428,7 +10428,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10542,7 +10542,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10656,7 +10656,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10770,7 +10770,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10884,7 +10884,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -10998,7 +10998,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11112,7 +11112,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11226,7 +11226,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11239,7 +11239,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F94" t="n">
@@ -11247,17 +11247,17 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H94" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I94" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J94" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K94" t="inlineStr">
         <is>
@@ -11349,7 +11349,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11463,7 +11463,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11577,7 +11577,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11691,7 +11691,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11805,7 +11805,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11919,7 +11919,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -11932,7 +11932,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F100" t="n">
@@ -11940,17 +11940,17 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H100" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I100" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J100" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K100" t="inlineStr">
         <is>
@@ -12042,7 +12042,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12156,7 +12156,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:30 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12270,7 +12270,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:30 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12384,7 +12384,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:30 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12498,7 +12498,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:30 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12612,7 +12612,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12726,7 +12726,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12840,7 +12840,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12954,7 +12954,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13068,7 +13068,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13182,7 +13182,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13296,7 +13296,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13410,7 +13410,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13524,7 +13524,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13638,7 +13638,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13752,7 +13752,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13866,7 +13866,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -13980,7 +13980,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14094,7 +14094,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14208,7 +14208,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14322,7 +14322,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14436,7 +14436,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14449,7 +14449,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F122" t="n">
@@ -14457,17 +14457,17 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H122" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I122" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J122" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K122" t="inlineStr">
         <is>
@@ -14559,7 +14559,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14673,7 +14673,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14787,7 +14787,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14901,7 +14901,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -15015,7 +15015,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15129,7 +15129,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15243,7 +15243,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -15357,7 +15357,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -15471,7 +15471,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -15585,7 +15585,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -15699,7 +15699,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -15813,7 +15813,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -15927,7 +15927,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -16041,7 +16041,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -16155,7 +16155,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -16269,7 +16269,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -16383,7 +16383,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -16497,7 +16497,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -16611,7 +16611,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -16725,7 +16725,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -16839,7 +16839,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C143" t="n">
@@ -16953,7 +16953,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -17067,7 +17067,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -17181,7 +17181,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -17295,7 +17295,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -17409,7 +17409,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -17523,7 +17523,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -17637,7 +17637,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -17751,7 +17751,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -17865,7 +17865,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -17979,7 +17979,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:30 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -18093,7 +18093,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -18207,7 +18207,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -18321,7 +18321,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -18435,7 +18435,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -18549,7 +18549,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -18562,7 +18562,7 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F158" t="n">
@@ -18570,17 +18570,17 @@
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H158" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I158" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J158" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K158" t="inlineStr">
         <is>
@@ -18672,7 +18672,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -18786,7 +18786,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -18900,7 +18900,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -19014,7 +19014,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -19128,7 +19128,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -19242,7 +19242,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -19356,7 +19356,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -19470,7 +19470,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -19584,7 +19584,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -19698,7 +19698,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -19812,7 +19812,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -19926,7 +19926,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -20040,7 +20040,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -20154,7 +20154,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -20268,7 +20268,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -20382,7 +20382,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -20496,7 +20496,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -20610,7 +20610,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -20724,7 +20724,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -20838,7 +20838,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -20952,7 +20952,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -21066,7 +21066,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -21180,7 +21180,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -21294,7 +21294,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -21408,7 +21408,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C183" t="n">
@@ -21522,7 +21522,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:30 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C184" t="n">
@@ -21636,7 +21636,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C185" t="n">
@@ -21750,7 +21750,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C186" t="n">
@@ -21864,7 +21864,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C187" t="n">
@@ -21978,7 +21978,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -22092,7 +22092,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C189" t="n">
@@ -22206,7 +22206,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -22320,7 +22320,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -22434,7 +22434,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C192" t="n">
@@ -22548,7 +22548,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -22662,7 +22662,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -22776,7 +22776,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -22890,7 +22890,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -23004,7 +23004,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -23118,7 +23118,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C198" t="n">
@@ -23232,7 +23232,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -23346,7 +23346,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -23460,7 +23460,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -23574,7 +23574,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C202" t="n">
@@ -23688,7 +23688,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C203" t="n">
@@ -23802,7 +23802,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -23916,7 +23916,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C205" t="n">
@@ -24030,7 +24030,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -24144,7 +24144,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -24258,7 +24258,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C208" t="n">
@@ -24372,7 +24372,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -24486,7 +24486,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C210" t="n">
@@ -24600,7 +24600,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C211" t="n">
@@ -24714,7 +24714,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -24727,7 +24727,7 @@
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F212" t="n">
@@ -24735,17 +24735,17 @@
       </c>
       <c r="G212" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H212" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I212" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J212" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K212" t="inlineStr">
         <is>
@@ -24837,7 +24837,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C213" t="n">
@@ -24850,7 +24850,7 @@
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F213" t="n">
@@ -24858,17 +24858,17 @@
       </c>
       <c r="G213" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H213" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I213" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J213" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K213" t="inlineStr">
         <is>
@@ -24960,7 +24960,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C214" t="n">
@@ -24973,7 +24973,7 @@
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F214" t="n">
@@ -24981,17 +24981,17 @@
       </c>
       <c r="G214" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H214" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I214" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J214" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K214" t="inlineStr">
         <is>
@@ -25083,7 +25083,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -25197,7 +25197,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:30 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C216" t="n">
@@ -25311,7 +25311,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C217" t="n">
@@ -25425,7 +25425,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -25539,7 +25539,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C219" t="n">
@@ -25653,7 +25653,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C220" t="n">
@@ -25767,7 +25767,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -25881,7 +25881,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C222" t="n">
@@ -25995,7 +25995,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C223" t="n">
@@ -26109,7 +26109,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C224" t="n">
@@ -26223,7 +26223,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C225" t="n">
@@ -26337,7 +26337,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C226" t="n">
@@ -26451,7 +26451,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -26565,7 +26565,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -26679,7 +26679,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -26793,7 +26793,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -26806,7 +26806,7 @@
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F230" t="n">
@@ -26814,17 +26814,17 @@
       </c>
       <c r="G230" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H230" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I230" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J230" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K230" t="inlineStr">
         <is>
@@ -26916,7 +26916,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -26929,7 +26929,7 @@
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F231" t="n">
@@ -26937,17 +26937,17 @@
       </c>
       <c r="G231" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H231" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I231" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J231" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K231" t="inlineStr">
         <is>
@@ -27039,7 +27039,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -27052,7 +27052,7 @@
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F232" t="n">
@@ -27060,17 +27060,17 @@
       </c>
       <c r="G232" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H232" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I232" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J232" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K232" t="inlineStr">
         <is>
@@ -27162,7 +27162,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -27175,7 +27175,7 @@
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F233" t="n">
@@ -27183,17 +27183,17 @@
       </c>
       <c r="G233" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H233" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I233" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J233" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K233" t="inlineStr">
         <is>
@@ -27285,7 +27285,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -27399,7 +27399,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -27513,7 +27513,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C236" t="n">
@@ -27627,7 +27627,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C237" t="n">
@@ -27741,7 +27741,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C238" t="n">
@@ -27855,7 +27855,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C239" t="n">
@@ -27969,7 +27969,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C240" t="n">
@@ -28083,7 +28083,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C241" t="n">
@@ -28197,7 +28197,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C242" t="n">
@@ -28311,7 +28311,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C243" t="n">
@@ -28425,7 +28425,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C244" t="n">
@@ -28539,7 +28539,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C245" t="n">
@@ -28653,7 +28653,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C246" t="n">
@@ -28767,7 +28767,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C247" t="n">
@@ -28881,7 +28881,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C248" t="n">
@@ -28995,7 +28995,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C249" t="n">
@@ -29109,7 +29109,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C250" t="n">
@@ -29223,7 +29223,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C251" t="n">
@@ -29337,7 +29337,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C252" t="n">
@@ -29451,7 +29451,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -29565,7 +29565,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -29679,7 +29679,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -29793,7 +29793,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -29907,7 +29907,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -30021,7 +30021,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -30135,7 +30135,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -30249,7 +30249,7 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -30363,7 +30363,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -30477,7 +30477,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -30591,7 +30591,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -30705,7 +30705,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -30819,7 +30819,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -30933,7 +30933,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -30946,7 +30946,7 @@
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F266" t="n">
@@ -30954,17 +30954,17 @@
       </c>
       <c r="G266" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H266" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I266" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J266" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K266" t="inlineStr">
         <is>
@@ -31056,7 +31056,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -31069,7 +31069,7 @@
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F267" t="n">
@@ -31077,17 +31077,17 @@
       </c>
       <c r="G267" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H267" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I267" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J267" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K267" t="inlineStr">
         <is>
@@ -31179,7 +31179,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -31192,7 +31192,7 @@
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F268" t="n">
@@ -31200,17 +31200,17 @@
       </c>
       <c r="G268" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H268" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I268" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J268" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K268" t="inlineStr">
         <is>
@@ -31302,7 +31302,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -31315,7 +31315,7 @@
       </c>
       <c r="E269" t="inlineStr">
         <is>
-          <t>Top 9 | 2 out</t>
+          <t>Bottom 9 | 0 out</t>
         </is>
       </c>
       <c r="F269" t="n">
@@ -31323,17 +31323,17 @@
       </c>
       <c r="G269" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="H269" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I269" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J269" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K269" t="inlineStr">
         <is>
@@ -31425,7 +31425,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -31539,7 +31539,7 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -31653,7 +31653,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -31767,7 +31767,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -31881,7 +31881,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -31995,7 +31995,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -32109,7 +32109,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:30 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -32223,7 +32223,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:30 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C277" t="n">
@@ -32337,7 +32337,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:30 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -32451,7 +32451,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C279" t="n">
@@ -32565,7 +32565,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -32679,7 +32679,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C281" t="n">
@@ -32793,7 +32793,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C282" t="n">
@@ -32907,7 +32907,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -33021,7 +33021,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C284" t="n">
@@ -33135,7 +33135,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -33249,7 +33249,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -33363,7 +33363,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C287" t="n">
@@ -33477,7 +33477,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -33591,7 +33591,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C289" t="n">
@@ -33705,7 +33705,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -33819,7 +33819,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C291" t="n">
@@ -33933,7 +33933,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C292" t="n">
@@ -34047,7 +34047,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C293" t="n">
@@ -34161,7 +34161,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C294" t="n">
@@ -34275,7 +34275,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:30 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C295" t="n">
@@ -34389,7 +34389,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:30 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C296" t="n">
@@ -34503,7 +34503,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:30 PM PT</t>
+          <t>2026-07-12 03:59:30 PM PT</t>
         </is>
       </c>
       <c r="C297" t="n">
@@ -34617,7 +34617,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C298" t="n">
@@ -34731,7 +34731,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C299" t="n">
@@ -34845,7 +34845,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C300" t="n">
@@ -34959,7 +34959,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C301" t="n">
@@ -35073,7 +35073,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C302" t="n">
@@ -35187,7 +35187,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C303" t="n">
@@ -35301,7 +35301,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C304" t="n">
@@ -35415,7 +35415,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C305" t="n">
@@ -35529,7 +35529,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C306" t="n">
@@ -35643,7 +35643,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C307" t="n">
@@ -35757,7 +35757,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C308" t="n">
@@ -35871,7 +35871,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C309" t="n">
@@ -35985,7 +35985,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C310" t="n">
@@ -36099,7 +36099,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C311" t="n">
@@ -36213,7 +36213,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -36327,7 +36327,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C313" t="n">
@@ -36441,7 +36441,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C314" t="n">
@@ -36555,7 +36555,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:32 PM PT</t>
+          <t>2026-07-12 03:59:32 PM PT</t>
         </is>
       </c>
       <c r="C315" t="n">
@@ -36669,7 +36669,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C316" t="n">
@@ -36783,7 +36783,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C317" t="n">
@@ -36897,7 +36897,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C318" t="n">
@@ -37011,7 +37011,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C319" t="n">
@@ -37125,7 +37125,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>2026-07-12 03:57:31 PM PT</t>
+          <t>2026-07-12 03:59:31 PM PT</t>
         </is>
       </c>
       <c r="C320" t="n">

</xml_diff>

<commit_message>
Update live MLB hitter fantasy scores 2026-07-12 04:01:33 PM PT
</commit_message>
<xml_diff>
--- a/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
+++ b/live_mlb_hitter_fantasy_scores_2026_07_12.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -807,7 +807,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:30 PM PT</t>
+          <t>2026-07-12 04:01:30 PM PT</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -921,7 +921,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:30 PM PT</t>
+          <t>2026-07-12 04:01:30 PM PT</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:32 PM PT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:32 PM PT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Bottom 9 | 0 out</t>
+          <t>Bottom 9 | 1 out</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -1516,7 +1516,7 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
@@ -1614,7 +1614,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1728,7 +1728,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1842,7 +1842,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:30 PM PT</t>
+          <t>2026-07-12 04:01:30 PM PT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1956,7 +1956,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -2070,7 +2070,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:30 PM PT</t>
+          <t>2026-07-12 04:01:30 PM PT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -2184,7 +2184,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -2298,7 +2298,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:30 PM PT</t>
+          <t>2026-07-12 04:01:30 PM PT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2412,7 +2412,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2640,7 +2640,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -2754,7 +2754,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2868,7 +2868,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2982,7 +2982,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:30 PM PT</t>
+          <t>2026-07-12 04:01:30 PM PT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -3096,7 +3096,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -3324,7 +3324,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -3438,7 +3438,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:32 PM PT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -3552,7 +3552,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:32 PM PT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -3565,7 +3565,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Bottom 9 | 0 out</t>
+          <t>Bottom 9 | 1 out</t>
         </is>
       </c>
       <c r="F27" t="n">
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I27" t="n">
         <v>0</v>
@@ -3675,7 +3675,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -3789,7 +3789,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:30 PM PT</t>
+          <t>2026-07-12 04:01:30 PM PT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -3903,7 +3903,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:30 PM PT</t>
+          <t>2026-07-12 04:01:30 PM PT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -4017,7 +4017,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -4131,7 +4131,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -4245,7 +4245,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -4359,7 +4359,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -4473,7 +4473,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -4587,7 +4587,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -4701,7 +4701,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -4815,7 +4815,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:30 PM PT</t>
+          <t>2026-07-12 04:01:30 PM PT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -4929,7 +4929,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -5043,7 +5043,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:30 PM PT</t>
+          <t>2026-07-12 04:01:30 PM PT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -5157,7 +5157,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:30 PM PT</t>
+          <t>2026-07-12 04:01:30 PM PT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -5271,7 +5271,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -5385,7 +5385,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -5499,7 +5499,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -5613,7 +5613,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:32 PM PT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -5727,7 +5727,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -5841,7 +5841,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:30 PM PT</t>
+          <t>2026-07-12 04:01:30 PM PT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -5955,7 +5955,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6069,7 +6069,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6183,7 +6183,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:30 PM PT</t>
+          <t>2026-07-12 04:01:30 PM PT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6297,7 +6297,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:30 PM PT</t>
+          <t>2026-07-12 04:01:30 PM PT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6411,7 +6411,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:32 PM PT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6525,7 +6525,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:32 PM PT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6538,7 +6538,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Bottom 9 | 0 out</t>
+          <t>Bottom 9 | 1 out</t>
         </is>
       </c>
       <c r="F53" t="n">
@@ -6550,7 +6550,7 @@
         </is>
       </c>
       <c r="H53" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I53" t="n">
         <v>0</v>
@@ -6648,7 +6648,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -6762,7 +6762,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -6876,7 +6876,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -6990,7 +6990,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -7104,7 +7104,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:30 PM PT</t>
+          <t>2026-07-12 04:01:30 PM PT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -7218,7 +7218,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -7332,7 +7332,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:32 PM PT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -7446,7 +7446,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -7560,7 +7560,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -7674,7 +7674,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -7788,7 +7788,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -7902,7 +7902,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:30 PM PT</t>
+          <t>2026-07-12 04:01:30 PM PT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -8016,7 +8016,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:30 PM PT</t>
+          <t>2026-07-12 04:01:30 PM PT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -8130,7 +8130,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -8244,7 +8244,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:32 PM PT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -8358,7 +8358,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -8472,7 +8472,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:32 PM PT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -8586,7 +8586,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:32 PM PT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -8700,7 +8700,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:32 PM PT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -8827,7 +8827,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Bottom 9 | 0 out</t>
+          <t>Bottom 9 | 1 out</t>
         </is>
       </c>
       <c r="F73" t="n">
@@ -8839,7 +8839,7 @@
         </is>
       </c>
       <c r="H73" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I73" t="n">
         <v>0</v>
@@ -8937,7 +8937,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:32 PM PT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -8950,7 +8950,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Bottom 9 | 0 out</t>
+          <t>Bottom 9 | 1 out</t>
         </is>
       </c>
       <c r="F74" t="n">
@@ -8962,7 +8962,7 @@
         </is>
       </c>
       <c r="H74" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I74" t="n">
         <v>0</v>
@@ -9060,7 +9060,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -9174,7 +9174,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -9288,7 +9288,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:30 PM PT</t>
+          <t>2026-07-12 04:01:30 PM PT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -9402,7 +9402,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -9516,7 +9516,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -9630,7 +9630,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -9744,7 +9744,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -9858,7 +9858,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:32 PM PT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -9972,7 +9972,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -10086,7 +10086,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -10200,7 +10200,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -10428,7 +10428,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -10542,7 +10542,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -10656,7 +10656,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -10770,7 +10770,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -10884,7 +10884,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:32 PM PT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -10998,7 +10998,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -11112,7 +11112,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:32 PM PT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -11226,7 +11226,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:32 PM PT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -11239,7 +11239,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Bottom 9 | 0 out</t>
+          <t>Bottom 9 | 1 out</t>
         </is>
       </c>
       <c r="F94" t="n">
@@ -11251,7 +11251,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I94" t="n">
         <v>0</v>
@@ -11349,7 +11349,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -11463,7 +11463,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -11577,7 +11577,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -11691,7 +11691,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -11805,7 +11805,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -11919,7 +11919,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:32 PM PT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -11932,7 +11932,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Bottom 9 | 0 out</t>
+          <t>Bottom 9 | 1 out</t>
         </is>
       </c>
       <c r="F100" t="n">
@@ -11944,7 +11944,7 @@
         </is>
       </c>
       <c r="H100" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I100" t="n">
         <v>0</v>
@@ -11986,10 +11986,10 @@
         </is>
       </c>
       <c r="R100" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S100" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T100" t="n">
         <v>1</v>
@@ -12042,7 +12042,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -12156,7 +12156,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:30 PM PT</t>
+          <t>2026-07-12 04:01:30 PM PT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -12270,7 +12270,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:30 PM PT</t>
+          <t>2026-07-12 04:01:30 PM PT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -12384,7 +12384,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:30 PM PT</t>
+          <t>2026-07-12 04:01:30 PM PT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -12498,7 +12498,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:30 PM PT</t>
+          <t>2026-07-12 04:01:30 PM PT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -12612,7 +12612,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -12726,7 +12726,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -12840,7 +12840,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -12954,7 +12954,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:32 PM PT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -13068,7 +13068,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:32 PM PT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -13182,7 +13182,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:32 PM PT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -13296,7 +13296,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -13410,7 +13410,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -13524,7 +13524,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -13638,7 +13638,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:32 PM PT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -13752,7 +13752,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -13866,7 +13866,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -13980,7 +13980,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:30 PM PT</t>
+          <t>2026-07-12 04:01:30 PM PT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -14094,7 +14094,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:32 PM PT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -14208,7 +14208,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -14322,7 +14322,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -14436,7 +14436,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:32 PM PT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -14449,7 +14449,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Bottom 9 | 0 out</t>
+          <t>Bottom 9 | 1 out</t>
         </is>
       </c>
       <c r="F122" t="n">
@@ -14461,7 +14461,7 @@
         </is>
       </c>
       <c r="H122" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I122" t="n">
         <v>0</v>
@@ -14559,7 +14559,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -14673,7 +14673,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:32 PM PT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -14787,7 +14787,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -14901,7 +14901,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:32 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -15015,7 +15015,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -15129,7 +15129,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>2026-07-12 03:59:31 PM PT</t>
+          <t>2026-07-12 04:01:31 PM PT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -15243,7 +15243,7 @@
       </